<commit_message>
Atualiza planilha diária de leads e conformidade
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,66 +413,66 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Data da Coleta</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Região</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Cidade</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Nome do Negócio</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Telefone</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>E-mail</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Score de Conformidade</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Nível de Risco</t>
         </is>
@@ -874,6 +862,198 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Clínica Simoneti</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://clinicasimoneti.com.br/</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="n">
+        <v>100</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Clínica Rubi</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://www.clinicarubi.com.br/</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="n">
+        <v>76</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Smile Clínica Odontológica</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://smilebh.com.br/</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="n">
+        <v>75</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>ClinBelo</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://clinbelo.com.br/</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>80</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona busca web gratuita (DuckDuckGo) para prospecção de leads
- Novo módulo web_search.py sem API key paga
- LEAD_SOURCE=auto usa web quando Places não está configurado
- Filtra diretórios/redes sociais comuns
- Teste Nordeste: 5 leads novos gravados na planilha

Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1054,6 +1054,246 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Médico em Maceió</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://agenda.app.br</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>67</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Clínica Inside Mind Jatiúca Maceió AL - Telefone...</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://www.benditoguia.com.br</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="n">
+        <v>70</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Monica Brasil</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://cebes.com.br</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>69</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Dra. Ana Maria Monteiro Menezes,- Clínica Médica</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://agendaconvenio.com</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>62</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Mix Clínica Ponta Verde Reviews</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.top-rated.online</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="n">
+        <v>33</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Completa lote Nordeste: +94 leads de conformidade
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1331,10 +1331,8 @@
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>5582993999600</t>
-        </is>
+      <c r="I19" t="n">
+        <v>5582993999600</v>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="n">
@@ -1479,10 +1477,8 @@
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>558232016100</t>
-        </is>
+      <c r="I22" t="n">
+        <v>558232016100</v>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="n">
@@ -1579,10 +1575,8 @@
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>5582999095311</t>
-        </is>
+      <c r="I24" t="n">
+        <v>5582999095311</v>
       </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="n">
@@ -1631,10 +1625,8 @@
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>552121012658</t>
-        </is>
+      <c r="I25" t="n">
+        <v>552121012658</v>
       </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
@@ -1827,10 +1819,8 @@
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>5512981915070</t>
-        </is>
+      <c r="I29" t="n">
+        <v>5512981915070</v>
       </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="n">
@@ -2167,10 +2157,8 @@
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>5582999010230</t>
-        </is>
+      <c r="I36" t="n">
+        <v>5582999010230</v>
       </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="n">
@@ -2278,6 +2266,4654 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Clinialagoas Medicina Integrada</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://clinialagoas.com.br</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>5582999450266</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="n">
+        <v>69</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Atend Já Maceió</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://maceio.atendja.com.br</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="n">
+        <v>90</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Climecor</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.climecor.com</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>5582993112942</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="n">
+        <v>69</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Clínica Médica em Maceió / AL</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.clinicaconsulta.com.br</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="n">
+        <v>69</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Gastroclinica</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://gastroclinicamaceio.com.br</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="n">
+        <v>75</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Bioclínica</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.bioclinicaal.com.br</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="n">
+        <v>88</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Especialistas em Maceió</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.medguias.com.br</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="n">
+        <v>94</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Médicos clínicos em Maceio</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://agendarconsulta.com</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="n">
+        <v>73</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Médico de Dor em Maceió-AL</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.drpedroferro.com.br</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="n">
+        <v>69</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Busca por médicos</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://cremal.org.br</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="n">
+        <v>76</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Dr. Daniel Moreira</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://dentistamaceio.com</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="n">
+        <v>67</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Odontologia Especializada</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.clinicaenova.com</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>558232418220</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="n">
+        <v>80</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Profissionais em Maceió</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www2.uniodonto.coop.br</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="n">
+        <v>56</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Dentista em Maceió</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://nucleoodontomcz.com.br</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>5582999851965</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="n">
+        <v>69</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Dentista SulAmérica Odonto em Maceió</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://odontologicosulamerica.com.br</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="n">
+        <v>56</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Dentista/Clínica Odontológica OdontoCompany em Maceió</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://odontocompany.com</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>5511932799505</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="n">
+        <v>81</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Os Mais Recomendados Psicólogos em Maceió</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://facilconsulta.com.br</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="n">
+        <v>22</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Psicólogo, Maceió, AL</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://redepsicologos.com.br</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="n">
+        <v>81</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Psicólogo, Maceió, AL</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://centralterapia.com.br</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="n">
+        <v>88</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Psicólogos Maceió (Alagoas)</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://br.mundopsicologos.com</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="n">
+        <v>88</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Psicólogo em Maceió - AL</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://medprev.online</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="n">
+        <v>87</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Psicólogos em Maceió</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.cronoshare.com.br</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="n">
+        <v>82</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Vanessa Dâmaso Psicóloga Clínica em Maceió</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://vanessadamaso.com.br</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>5582999161318</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="n">
+        <v>67</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Psicólogo, Conselheiro, Terapeuta perto de mim em Maceió ...</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://mentalzon.com</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="n">
+        <v>47</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Psicanalistas em Maceió</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://euterapeuta.com.br</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="n">
+        <v>80</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>10 melhores terapeutas para Maceió</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://www.starofservice.com.br</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="n">
+        <v>64</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Advogados</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://www.tenoriomeloadvocacia.com.br</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>5582981318059</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="n">
+        <v>73</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Advogados e Escritórios de Advocacia em Maceió</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://www.encontramaceio.com.br</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="n">
+        <v>55</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>ALNPP</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://www.alnpp.com.br</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="n">
+        <v>45</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Cavalcanti Advogados Associados</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://cavalcantiassociados.com</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>5582993710121</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="n">
+        <v>73</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>10 Melhores Escritórios de Advocacia em Maceió AL</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://ddireito.com.br</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="n">
+        <v>73</v>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Advocacia de excelência em Maceió e Alagoas</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://neripachecoadvogados.com</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="n">
+        <v>64</v>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Advogado em Maceió e Região</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://joseneto.adv.br</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>558299179336</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="n">
+        <v>82</v>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Faculdades de Educação Física em Maceió - AL</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://querobolsa.com.br</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>558001232222</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="n">
+        <v>69</v>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Mestrados e cursos de Educação Física no Maceió</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://www.educaedu-brasil.com</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="n">
+        <v>62</v>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Faculdades de Educação Física a distância em Maceió - AL</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://www.ead.com.br</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>558009423474</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="n">
+        <v>69</v>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Cursos de Educação Física em Maceió - AL</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://www.guiadacarreira.com.br</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>558009427777</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="n">
+        <v>69</v>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Educação Física</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://www.uncisal.edu.br</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="n">
+        <v>71</v>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>EDUCAÇÃO FÍSICA NA IBESA</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://carreiras.stoodi.com.br</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="n">
+        <v>22</v>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Instituto de Educação Física e Esporte</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://iefe.ufal.br</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="n">
+        <v>67</v>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Academias em Maceió, AL, Brasil</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://wellhub.com</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>551124241451</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="n">
+        <v>60</v>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://allpfit.com.br</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="n">
+        <v>40</v>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Academia Smart Fit</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://www.smartfit.com.br</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="n">
+        <v>90</v>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>PARQUE SHOPPING MACEIÓ</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://www.selfitacademias.com.br</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="n">
+        <v>90</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>GO Training Center</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://gorgonoid.com</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>5531998385296</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="n">
+        <v>70</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Academias em Maceió, AL</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://www.gurupass.com.br</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>551141182773</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="n">
+        <v>50</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Academia Smart Fit</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>https://www.waze.com</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="n">
+        <v>56</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Fisioterapia Pilates RPG</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>https://www.clinicafipi.com</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>5582991107444</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="n">
+        <v>69</v>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Dr. André Oliveira</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>https://drandreoliveirafisio.com.br</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>5582996460786</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="n">
+        <v>73</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Fisiocoop</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://fisiocoop.coop.br</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Espaço Saúde Unimed</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://www.unimed.coop.br</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="n">
+        <v>71</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Os 10 melhores centros de Fisioterapia em Maceió</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://maceio.infoisinfo-br.com</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="n">
+        <v>64</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Clinica Vida: Clínica Vida</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>https://clinicavida.com.br</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>5571981784780</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="n">
+        <v>69</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Clinicas Clivale</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://clinicasclivale.com.br</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>5571999697064</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="n">
+        <v>65</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Clínica Santa Helena</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>https://www.gruposhbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>5571999667555</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="n">
+        <v>56</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Clínica Ibis</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>https://www.clinicaibis.com.br</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>5571984105500</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="n">
+        <v>76</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Clínica médica</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>https://www.fjs.org.br</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>557135045240</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="n">
+        <v>65</v>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Clínica Humana</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>https://www.clinicahumana.com.br</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="n">
+        <v>50</v>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Clínica-escola oferece atendimento médico gratuito em Salvador</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>https://g1.globo.com</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="n">
+        <v>64</v>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Centro Médico Hospital da Bahia</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>https://www.centromedicohba.com.br</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="n">
+        <v>69</v>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Melhor médicos em Salvador por avaliações</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>https://www.avaliamed.com.br</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="n">
+        <v>81</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Home • Bem Centro Médico</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>https://bemcentromedico.com.br</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>557131900499</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="n">
+        <v>67</v>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>O Dentista Clínica Odontológica</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>https://www.odentistabrasil.com.br</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>557132427486</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="n">
+        <v>67</v>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Dentista Salvador</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>https://dentistasalvador.ac.gd</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="n">
+        <v>53</v>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Dentista Salvador</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>https://dentistasalvador.com.br</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="n">
+        <v>0</v>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Clínica Apollo Odontologia Integrada</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>https://clinicaapollo.com.br</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>5571981251568</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="n">
+        <v>73</v>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Núcleo Odontológico de Salvador</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>https://www.nosodontosalvador.com.br</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>5571991562088</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="n">
+        <v>69</v>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Dentistas em Salvador - BA</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>https://dentmap.com.br</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="n">
+        <v>75</v>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Implante Dentário em Salvador</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>https://www.hospitalodontologico.com.br</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="n">
+        <v>69</v>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Antônia Carolina de Souza Paim</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>https://www.psicologasalvador.com.br</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>5571997056073</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="n">
+        <v>73</v>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Gestar Psi</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>https://clinicagestarpsi.com.br</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>557193733334</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="n">
+        <v>94</v>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Psicólogos em Salvador - Bahia</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>https://www.psicologapopular.com</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>5537999773676</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="n">
+        <v>93</v>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Vagas de Psicólogo em Salvador, BA (Urgente!)</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>https://br.jooble.org</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="n">
+        <v>33</v>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Terapeuta perto de mim em Salvador</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>https://www.locaisdobrasil.com.br</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="n">
+        <v>78</v>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Terapias em Salvador</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>https://www.terapyas.com.br</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="n">
+        <v>94</v>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Sandra Valéria Coelho</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>https://terapia.salvador.br</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="n">
+        <v>62</v>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Advogados e Correspondentes Jurídicos em Salvador, BA</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>https://juridicocerto.com</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="n">
+        <v>64</v>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Salvador advogados em salvador BA advogado salvador BA</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>https://www.advogadosaqui.com.br</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="n">
+        <v>64</v>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Isabella Magalhães</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>https://especialistadefamilia.com.br</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="n">
+        <v>33</v>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>31 avaliações sobre Borges &amp; Queiroz Advogados...</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>https://avaliacoesbrasil.com</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="n">
+        <v>73</v>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Faculdades de Educação Física em Salvador</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>https://www.faculdadesja.com.br</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="n">
+        <v>0</v>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>CURSO SUPERIOR LICENCIATURA EM FÍSICA — IFBA</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>https://portal.ifba.edu.br</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="n">
+        <v>0</v>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Educação Física</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>https://www.bahiana.edu.br</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="n">
+        <v>33</v>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>297 Academias em Salvador/BA (2026)</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>https://acharacademia.com.br</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="n">
+        <v>60</v>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Academias em Salvador</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>https://www.akademias.com.br</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="n">
+        <v>90</v>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Hammer Fitness Club</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>https://www.hammeracademia.com</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="n">
+        <v>90</v>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Fisioterapeutas em Salvador - BA</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>https://www.listamais.com.br</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="n">
+        <v>0</v>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Fisioterapeutas em Salvador (2026) — Agendar Consulta</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>https://clinic.medilifeapp.com</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="n">
+        <v>73</v>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Rosimeire Passos Fisioterapeuta em Salvador</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>https://www.rosipassosfisio.com.br</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="n">
+        <v>73</v>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Profisio</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>https://www.clinicaprofisio.com</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>5571999926164</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="n">
+        <v>73</v>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>HomeCalm Fisioterapia e Pilates</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>https://homecalm.com.br</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>5571991272568</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="n">
+        <v>75</v>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Clínica de Fisioterapia na Pituba</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>https://pitubafisio.com.br</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>5571988103288</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="n">
+        <v>73</v>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Clínica Nova</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>https://clinicanova.med.br</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>558530480500</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="n">
+        <v>67</v>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Clínica SantaMed: Página Principal</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>https://clinicasantamed.com.br</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>5585981077070</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="n">
+        <v>69</v>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Centro-Oeste, 2026-07-24)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L132"/>
+  <dimension ref="A1:L208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2303,10 +2303,8 @@
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>5582999450266</t>
-        </is>
+      <c r="I39" t="n">
+        <v>5582999450266</v>
       </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="n">
@@ -2403,10 +2401,8 @@
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>5582993112942</t>
-        </is>
+      <c r="I41" t="n">
+        <v>5582993112942</v>
       </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="n">
@@ -2839,10 +2835,8 @@
         </is>
       </c>
       <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>558232418220</t>
-        </is>
+      <c r="I50" t="n">
+        <v>558232418220</v>
       </c>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="n">
@@ -2939,10 +2933,8 @@
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>5582999851965</t>
-        </is>
+      <c r="I52" t="n">
+        <v>5582999851965</v>
       </c>
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="n">
@@ -3039,10 +3031,8 @@
         </is>
       </c>
       <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>5511932799505</t>
-        </is>
+      <c r="I54" t="n">
+        <v>5511932799505</v>
       </c>
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="n">
@@ -3379,10 +3369,8 @@
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>5582999161318</t>
-        </is>
+      <c r="I61" t="n">
+        <v>5582999161318</v>
       </c>
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="n">
@@ -3575,10 +3563,8 @@
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>5582981318059</t>
-        </is>
+      <c r="I65" t="n">
+        <v>5582981318059</v>
       </c>
       <c r="J65" t="inlineStr"/>
       <c r="K65" t="n">
@@ -3723,10 +3709,8 @@
         </is>
       </c>
       <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>5582993710121</t>
-        </is>
+      <c r="I68" t="n">
+        <v>5582993710121</v>
       </c>
       <c r="J68" t="inlineStr"/>
       <c r="K68" t="n">
@@ -3871,10 +3855,8 @@
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>558299179336</t>
-        </is>
+      <c r="I71" t="n">
+        <v>558299179336</v>
       </c>
       <c r="J71" t="inlineStr"/>
       <c r="K71" t="n">
@@ -3923,10 +3905,8 @@
         </is>
       </c>
       <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>558001232222</t>
-        </is>
+      <c r="I72" t="n">
+        <v>558001232222</v>
       </c>
       <c r="J72" t="inlineStr"/>
       <c r="K72" t="n">
@@ -4023,10 +4003,8 @@
         </is>
       </c>
       <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>558009423474</t>
-        </is>
+      <c r="I74" t="n">
+        <v>558009423474</v>
       </c>
       <c r="J74" t="inlineStr"/>
       <c r="K74" t="n">
@@ -4075,10 +4053,8 @@
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>558009427777</t>
-        </is>
+      <c r="I75" t="n">
+        <v>558009427777</v>
       </c>
       <c r="J75" t="inlineStr"/>
       <c r="K75" t="n">
@@ -4271,10 +4247,8 @@
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>551124241451</t>
-        </is>
+      <c r="I79" t="n">
+        <v>551124241451</v>
       </c>
       <c r="J79" t="inlineStr"/>
       <c r="K79" t="n">
@@ -4467,10 +4441,8 @@
         </is>
       </c>
       <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>5531998385296</t>
-        </is>
+      <c r="I83" t="n">
+        <v>5531998385296</v>
       </c>
       <c r="J83" t="inlineStr"/>
       <c r="K83" t="n">
@@ -4519,10 +4491,8 @@
         </is>
       </c>
       <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>551141182773</t>
-        </is>
+      <c r="I84" t="n">
+        <v>551141182773</v>
       </c>
       <c r="J84" t="inlineStr"/>
       <c r="K84" t="n">
@@ -4619,10 +4589,8 @@
         </is>
       </c>
       <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>5582991107444</t>
-        </is>
+      <c r="I86" t="n">
+        <v>5582991107444</v>
       </c>
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="n">
@@ -4671,10 +4639,8 @@
         </is>
       </c>
       <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>5582996460786</t>
-        </is>
+      <c r="I87" t="n">
+        <v>5582996460786</v>
       </c>
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="n">
@@ -4867,10 +4833,8 @@
         </is>
       </c>
       <c r="H91" t="inlineStr"/>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>5571981784780</t>
-        </is>
+      <c r="I91" t="n">
+        <v>5571981784780</v>
       </c>
       <c r="J91" t="inlineStr"/>
       <c r="K91" t="n">
@@ -4919,10 +4883,8 @@
         </is>
       </c>
       <c r="H92" t="inlineStr"/>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>5571999697064</t>
-        </is>
+      <c r="I92" t="n">
+        <v>5571999697064</v>
       </c>
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="n">
@@ -4971,10 +4933,8 @@
         </is>
       </c>
       <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>5571999667555</t>
-        </is>
+      <c r="I93" t="n">
+        <v>5571999667555</v>
       </c>
       <c r="J93" t="inlineStr"/>
       <c r="K93" t="n">
@@ -5023,10 +4983,8 @@
         </is>
       </c>
       <c r="H94" t="inlineStr"/>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>5571984105500</t>
-        </is>
+      <c r="I94" t="n">
+        <v>5571984105500</v>
       </c>
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="n">
@@ -5075,10 +5033,8 @@
         </is>
       </c>
       <c r="H95" t="inlineStr"/>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>557135045240</t>
-        </is>
+      <c r="I95" t="n">
+        <v>557135045240</v>
       </c>
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="n">
@@ -5319,10 +5275,8 @@
         </is>
       </c>
       <c r="H100" t="inlineStr"/>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>557131900499</t>
-        </is>
+      <c r="I100" t="n">
+        <v>557131900499</v>
       </c>
       <c r="J100" t="inlineStr"/>
       <c r="K100" t="n">
@@ -5371,10 +5325,8 @@
         </is>
       </c>
       <c r="H101" t="inlineStr"/>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>557132427486</t>
-        </is>
+      <c r="I101" t="n">
+        <v>557132427486</v>
       </c>
       <c r="J101" t="inlineStr"/>
       <c r="K101" t="n">
@@ -5519,10 +5471,8 @@
         </is>
       </c>
       <c r="H104" t="inlineStr"/>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>5571981251568</t>
-        </is>
+      <c r="I104" t="n">
+        <v>5571981251568</v>
       </c>
       <c r="J104" t="inlineStr"/>
       <c r="K104" t="n">
@@ -5571,10 +5521,8 @@
         </is>
       </c>
       <c r="H105" t="inlineStr"/>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>5571991562088</t>
-        </is>
+      <c r="I105" t="n">
+        <v>5571991562088</v>
       </c>
       <c r="J105" t="inlineStr"/>
       <c r="K105" t="n">
@@ -5719,10 +5667,8 @@
         </is>
       </c>
       <c r="H108" t="inlineStr"/>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>5571997056073</t>
-        </is>
+      <c r="I108" t="n">
+        <v>5571997056073</v>
       </c>
       <c r="J108" t="inlineStr"/>
       <c r="K108" t="n">
@@ -5771,10 +5717,8 @@
         </is>
       </c>
       <c r="H109" t="inlineStr"/>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>557193733334</t>
-        </is>
+      <c r="I109" t="n">
+        <v>557193733334</v>
       </c>
       <c r="J109" t="inlineStr"/>
       <c r="K109" t="n">
@@ -5823,10 +5767,8 @@
         </is>
       </c>
       <c r="H110" t="inlineStr"/>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>5537999773676</t>
-        </is>
+      <c r="I110" t="n">
+        <v>5537999773676</v>
       </c>
       <c r="J110" t="inlineStr"/>
       <c r="K110" t="n">
@@ -6691,10 +6633,8 @@
         </is>
       </c>
       <c r="H128" t="inlineStr"/>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>5571999926164</t>
-        </is>
+      <c r="I128" t="n">
+        <v>5571999926164</v>
       </c>
       <c r="J128" t="inlineStr"/>
       <c r="K128" t="n">
@@ -6743,10 +6683,8 @@
         </is>
       </c>
       <c r="H129" t="inlineStr"/>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>5571991272568</t>
-        </is>
+      <c r="I129" t="n">
+        <v>5571991272568</v>
       </c>
       <c r="J129" t="inlineStr"/>
       <c r="K129" t="n">
@@ -6795,10 +6733,8 @@
         </is>
       </c>
       <c r="H130" t="inlineStr"/>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>5571988103288</t>
-        </is>
+      <c r="I130" t="n">
+        <v>5571988103288</v>
       </c>
       <c r="J130" t="inlineStr"/>
       <c r="K130" t="n">
@@ -6847,10 +6783,8 @@
         </is>
       </c>
       <c r="H131" t="inlineStr"/>
-      <c r="I131" t="inlineStr">
-        <is>
-          <t>558530480500</t>
-        </is>
+      <c r="I131" t="n">
+        <v>558530480500</v>
       </c>
       <c r="J131" t="inlineStr"/>
       <c r="K131" t="n">
@@ -6899,16 +6833,3806 @@
         </is>
       </c>
       <c r="H132" t="inlineStr"/>
-      <c r="I132" t="inlineStr">
-        <is>
-          <t>5585981077070</t>
-        </is>
+      <c r="I132" t="n">
+        <v>5585981077070</v>
       </c>
       <c r="J132" t="inlineStr"/>
       <c r="K132" t="n">
         <v>69</v>
       </c>
       <c r="L132" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>clinicasbrasilia.com.br</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>https://clinicasbrasilia.com.br</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>556134681068</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="n">
+        <v>64</v>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Centro Clínico A+ Saúde</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>https://velora.tech</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="n">
+        <v>44</v>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Clínica Médica em Brasília com Somos Popular</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>https://www.somospopular.com.br</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="n">
+        <v>33</v>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Centro Clínico Humana Recanto das Emas Brasília DF...</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>https://guiamania.com.br</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="n">
+        <v>33</v>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Dr. André Luís Wambier — Cardio DF</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>https://cardiodf.com.br</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="n">
+        <v>59</v>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>medicoperto.com.br</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>https://medicoperto.com.br</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>5561982863837</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="n">
+        <v>80</v>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Dental Brasil</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>https://dentalbrasildf.com.br</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>556130112356</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="n">
+        <v>75</v>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Clínica de Odontologia</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>https://www.unip.br</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>5511943035000</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="n">
+        <v>88</v>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>ZR Odonto</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>https://zrodonto.com.br</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>5561998375118</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="n">
+        <v>88</v>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Trida Odontologia Especializada</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>https://tridaodontologia.com.br</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>5561981850318</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="n">
+        <v>80</v>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Clínica-Escola de Odontologia</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>https://ucb2.catolica.edu.br</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>556133569075</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="n">
+        <v>69</v>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Odontologia</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>https://sescdf.com.br</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>556132189101</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="n">
+        <v>69</v>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Psicólogos em Brasília: Agende sua terapia online agora mesmo</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>https://www.psitto.com.br</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>5511968632121</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="n">
+        <v>81</v>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Psiquiatra Brasilia DF</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>https://med-br.com</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="n">
+        <v>75</v>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Psicólogo Brasília</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>https://www.singularpsicologiadf.com.br</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>5561999511258</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="n">
+        <v>73</v>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>IBAC</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>https://ibac.com.br</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="n">
+        <v>62</v>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Psicoterapia em Brasília</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>https://www.fisioemov.com.br</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>556198782133</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="n">
+        <v>69</v>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Clínica Diálogo</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>https://clinicadialogo.com.br</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="n">
+        <v>50</v>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Terapia de Casal em Brasília</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>https://www.ressignificarpsicologia.com</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>5561998634538</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="n">
+        <v>80</v>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Psicologia e Psicoterapia</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>https://incb.com.br</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>5561996060635</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="n">
+        <v>22</v>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Reflexões e Orientações sobre a Prática da Psicoterapia</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>https://site.cfp.org.br</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="n">
+        <v>88</v>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Distrito Federal</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>https://www.traumaclinic.com.br</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr"/>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="n">
+        <v>81</v>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Carneiros Advogados: Home</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>https://carneiros.adv.br</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="n">
+        <v>64</v>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Ibaneis Advogados Associados</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>https://www.ibaneis.adv.br</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="n">
+        <v>73</v>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Torres e Corrêa Advocacia</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>https://tco.adv.br</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="n">
+        <v>89</v>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Eliana Calmon</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>https://elianacalmon.adv.br</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr"/>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>556139631262</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="n">
+        <v>64</v>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Paixão Côrtes Advogados</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>https://www.paixaocortes.com.br</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>5561981536149</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr"/>
+      <c r="K159" t="n">
+        <v>64</v>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Dinamarco Advogados: Home</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>https://www.dinamarco.com.br</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr"/>
+      <c r="I160" t="inlineStr"/>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="n">
+        <v>55</v>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Vagas De Emprego De Professor Educaçao Fisica Brasilia</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>https://vagas.mitula.com.br</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr"/>
+      <c r="I161" t="inlineStr"/>
+      <c r="J161" t="inlineStr"/>
+      <c r="K161" t="n">
+        <v>22</v>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Vagas de emprego : Professor de Educação Física em Brasília</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>https://www.careerjet.com.br</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr"/>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="n">
+        <v>0</v>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Ensino médio noturno: as dispensas nas aulas de Educação Física</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>https://efdeportes.com</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr"/>
+      <c r="I163" t="inlineStr"/>
+      <c r="J163" t="inlineStr"/>
+      <c r="K163" t="n">
+        <v>65</v>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Como chegar até CREF</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>https://moovitapp.com</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr"/>
+      <c r="I164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
+      <c r="K164" t="n">
+        <v>44</v>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Horário de Brasília</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>https://www.horariodebrasilia.org</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr"/>
+      <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
+      <c r="K165" t="n">
+        <v>56</v>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Vaga de Estagiário</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>https://cadernonacional.com.br</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr"/>
+      <c r="I166" t="inlineStr"/>
+      <c r="J166" t="inlineStr"/>
+      <c r="K166" t="n">
+        <v>81</v>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Dimensões motivacionais dos conteúdos da educação física no...</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>https://ojs.revistadelos.com</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr"/>
+      <c r="I167" t="inlineStr"/>
+      <c r="J167" t="inlineStr"/>
+      <c r="K167" t="n">
+        <v>33</v>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>29 academias em Brasília (Distrito Federal) + trainers</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>https://conecta.fitness</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr"/>
+      <c r="I168" t="inlineStr"/>
+      <c r="J168" t="inlineStr"/>
+      <c r="K168" t="n">
+        <v>40</v>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Runway</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>https://runway.com.br</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr"/>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>556195844771</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="n">
+        <v>90</v>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Academia Unique</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>https://www.academiaunique.com.br</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr"/>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>5561993140270</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="n">
+        <v>70</v>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Ultra Academia</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>https://ultraacademia.com.br</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr"/>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>5511974139514</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="n">
+        <v>70</v>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Academia Body Action</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>https://foursquare.com</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr"/>
+      <c r="I172" t="inlineStr"/>
+      <c r="J172" t="inlineStr"/>
+      <c r="K172" t="n">
+        <v>44</v>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>13 vagas de fisioterapeuta – Brasília, Distrito Federal</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.com.br</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr"/>
+      <c r="I173" t="inlineStr"/>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="n">
+        <v>33</v>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Encontre um profissional Certificado</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>https://mckenzie.com.br</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr"/>
+      <c r="I174" t="inlineStr"/>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="n">
+        <v>33</v>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Clínica Brasil: Tudo o que sua saúde precisa!</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>https://clinicabrasilgoiania.com.br</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr"/>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>556235454000</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="n">
+        <v>94</v>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Clínica Goiana Medicina &amp; Diagnóstico</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>https://clinicagoiana.med.br</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr"/>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>5564984390766</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="n">
+        <v>88</v>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Clínica Popular em Goiânia, Consultas Médicas, Exames Médicos</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>https://www.clinicavittagoiania.com.br</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr"/>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>556239960505</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="n">
+        <v>62</v>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Clínica em Goiânia</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>https://clinicagedda.com.br</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr"/>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>5562998256655</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="n">
+        <v>22</v>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Clínica Médica Goiás Saúde e Odontologia</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>https://www.clinicamedicagoias.com.br</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr"/>
+      <c r="I179" t="inlineStr"/>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="n">
+        <v>0</v>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Atend Já Goiânia</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>https://goiania.atendja.com.br</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr"/>
+      <c r="I180" t="inlineStr"/>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="n">
+        <v>90</v>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Goiânia Médica</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>https://www.goianiamedica.com.br</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr"/>
+      <c r="I181" t="inlineStr"/>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="n">
+        <v>0</v>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Clínica de Diagnóstico por Imagem Avançado</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>https://clinicadia.net.br</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr"/>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>556232512898</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="n">
+        <v>88</v>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>CREMEGO, Busca médico</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>https://crmvirtual.cfm.org.br</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr"/>
+      <c r="I183" t="inlineStr"/>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="n">
+        <v>62</v>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Vagas de emprego Médico em Goiânia, GO</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>https://www.jobijoba.com.br</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr"/>
+      <c r="I184" t="inlineStr"/>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="n">
+        <v>73</v>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>CREDENCIADOS GOIANIA</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>https://assets.marinha.mil.br</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr"/>
+      <c r="I185" t="inlineStr"/>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="n">
+        <v>0</v>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Dentista em Goiânia</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>https://dentistagoiania.com.br</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr"/>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>5511912062131</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="n">
+        <v>56</v>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Implantes Dentários em Goiânia</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>https://odontogaravelo.com.br</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr"/>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>5562996304831</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr"/>
+      <c r="K187" t="n">
+        <v>60</v>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Centro Goiano de Odontologia</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>https://www.centrogoianodeodontologia.com.br</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr"/>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>5562995531882</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr"/>
+      <c r="K188" t="n">
+        <v>56</v>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Psicólogo Goiânia: Encontre os melhores psicólogos em Goiânia</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>https://psicologogoiania.com</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr"/>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>5562982663416</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="n">
+        <v>75</v>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Instituto Suassuna</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>https://institutosuassuna.com.br</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr"/>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>5562981426789</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="n">
+        <v>81</v>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>A função do psicólogo no pronto-socorro: a visão da equipe</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>http://pepsic.bvsalud.org</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr"/>
+      <c r="I191" t="inlineStr"/>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="n">
+        <v>60</v>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Psicólogo em Goiânia</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>https://www.clinicamedprime.com.br</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr"/>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>556239960508</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="n">
+        <v>62</v>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Dr Humberto Psicanalista Terapeuta</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>https://www.humbertopsicanalista.com</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr"/>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>5562999234619</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr"/>
+      <c r="K193" t="n">
+        <v>62</v>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>TERAPEUTA LUCIANA OFICIAL</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>https://www.terapeutalucianarocha.com.br</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr"/>
+      <c r="I194" t="inlineStr"/>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="n">
+        <v>0</v>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>Clínica Veredas</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>https://veredaspsicologia.com.br</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr"/>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>5562992899057</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr"/>
+      <c r="K195" t="n">
+        <v>80</v>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>EMBN Advogados</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>https://www.edmommoraesadv.com</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr"/>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>5562984796876</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr"/>
+      <c r="K196" t="n">
+        <v>73</v>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Advogado Goiânia Escritório de Advocacia Rodolfo Pimenta</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>https://rodolfopimenta.com.br</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr"/>
+      <c r="I197" t="inlineStr"/>
+      <c r="J197" t="inlineStr"/>
+      <c r="K197" t="n">
+        <v>82</v>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Rocha Advogados</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>https://rochadvogados.com.br</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr"/>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>5562992347835</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr"/>
+      <c r="K198" t="n">
+        <v>73</v>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Advogado Goiania</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>https://advogadogoiania.com.br</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr"/>
+      <c r="I199" t="inlineStr"/>
+      <c r="J199" t="inlineStr"/>
+      <c r="K199" t="n">
+        <v>64</v>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Advogado Trabalhista - Dr. Arthur Morais</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>https://viatapida.com</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr"/>
+      <c r="I200" t="inlineStr"/>
+      <c r="J200" t="inlineStr"/>
+      <c r="K200" t="n">
+        <v>45</v>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Educação Física</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>https://www.uniaraguaia.edu.br</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr"/>
+      <c r="I201" t="inlineStr"/>
+      <c r="J201" t="inlineStr"/>
+      <c r="K201" t="n">
+        <v>33</v>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Faça Educação Física Bacharelado na PUC Goiás (Bolsa de 50%)</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>https://www.pucgoias.edu.br</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr"/>
+      <c r="I202" t="inlineStr"/>
+      <c r="J202" t="inlineStr"/>
+      <c r="K202" t="n">
+        <v>33</v>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Curso de Faculdades de Educação Física em Goiás</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>https://www.educabras.com</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr"/>
+      <c r="I203" t="inlineStr"/>
+      <c r="J203" t="inlineStr"/>
+      <c r="K203" t="n">
+        <v>59</v>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>https://www.academiagavioes.com.br</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr"/>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>5511940747584</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr"/>
+      <c r="K204" t="n">
+        <v>73</v>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Flex Fitness Center</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>https://www.flexfitnesscenter.com.br</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr"/>
+      <c r="I205" t="inlineStr"/>
+      <c r="J205" t="inlineStr"/>
+      <c r="K205" t="n">
+        <v>22</v>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Academia da Fáscia</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>https://www.academiadafascia.com</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr"/>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>5562994359484</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr"/>
+      <c r="K206" t="n">
+        <v>70</v>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Melhores Academias de Goiânia - GO</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>https://rudders.com.br</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr"/>
+      <c r="I207" t="inlineStr"/>
+      <c r="J207" t="inlineStr"/>
+      <c r="K207" t="n">
+        <v>80</v>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Principais fisioterapeutas e profissionais da saúde em Goiânia</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>https://buscafisio.com.br</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr"/>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>551141183034</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr"/>
+      <c r="K208" t="n">
+        <v>69</v>
+      </c>
+      <c r="L208" t="inlineStr">
         <is>
           <t>Crítico</t>
         </is>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Sudeste, 2026-07-25)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L208"/>
+  <dimension ref="A1:L279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6883,10 +6883,8 @@
         </is>
       </c>
       <c r="H133" t="inlineStr"/>
-      <c r="I133" t="inlineStr">
-        <is>
-          <t>556134681068</t>
-        </is>
+      <c r="I133" t="n">
+        <v>556134681068</v>
       </c>
       <c r="J133" t="inlineStr"/>
       <c r="K133" t="n">
@@ -7127,10 +7125,8 @@
         </is>
       </c>
       <c r="H138" t="inlineStr"/>
-      <c r="I138" t="inlineStr">
-        <is>
-          <t>5561982863837</t>
-        </is>
+      <c r="I138" t="n">
+        <v>5561982863837</v>
       </c>
       <c r="J138" t="inlineStr"/>
       <c r="K138" t="n">
@@ -7179,10 +7175,8 @@
         </is>
       </c>
       <c r="H139" t="inlineStr"/>
-      <c r="I139" t="inlineStr">
-        <is>
-          <t>556130112356</t>
-        </is>
+      <c r="I139" t="n">
+        <v>556130112356</v>
       </c>
       <c r="J139" t="inlineStr"/>
       <c r="K139" t="n">
@@ -7231,10 +7225,8 @@
         </is>
       </c>
       <c r="H140" t="inlineStr"/>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>5511943035000</t>
-        </is>
+      <c r="I140" t="n">
+        <v>5511943035000</v>
       </c>
       <c r="J140" t="inlineStr"/>
       <c r="K140" t="n">
@@ -7283,10 +7275,8 @@
         </is>
       </c>
       <c r="H141" t="inlineStr"/>
-      <c r="I141" t="inlineStr">
-        <is>
-          <t>5561998375118</t>
-        </is>
+      <c r="I141" t="n">
+        <v>5561998375118</v>
       </c>
       <c r="J141" t="inlineStr"/>
       <c r="K141" t="n">
@@ -7335,10 +7325,8 @@
         </is>
       </c>
       <c r="H142" t="inlineStr"/>
-      <c r="I142" t="inlineStr">
-        <is>
-          <t>5561981850318</t>
-        </is>
+      <c r="I142" t="n">
+        <v>5561981850318</v>
       </c>
       <c r="J142" t="inlineStr"/>
       <c r="K142" t="n">
@@ -7387,10 +7375,8 @@
         </is>
       </c>
       <c r="H143" t="inlineStr"/>
-      <c r="I143" t="inlineStr">
-        <is>
-          <t>556133569075</t>
-        </is>
+      <c r="I143" t="n">
+        <v>556133569075</v>
       </c>
       <c r="J143" t="inlineStr"/>
       <c r="K143" t="n">
@@ -7439,10 +7425,8 @@
         </is>
       </c>
       <c r="H144" t="inlineStr"/>
-      <c r="I144" t="inlineStr">
-        <is>
-          <t>556132189101</t>
-        </is>
+      <c r="I144" t="n">
+        <v>556132189101</v>
       </c>
       <c r="J144" t="inlineStr"/>
       <c r="K144" t="n">
@@ -7491,10 +7475,8 @@
         </is>
       </c>
       <c r="H145" t="inlineStr"/>
-      <c r="I145" t="inlineStr">
-        <is>
-          <t>5511968632121</t>
-        </is>
+      <c r="I145" t="n">
+        <v>5511968632121</v>
       </c>
       <c r="J145" t="inlineStr"/>
       <c r="K145" t="n">
@@ -7591,10 +7573,8 @@
         </is>
       </c>
       <c r="H147" t="inlineStr"/>
-      <c r="I147" t="inlineStr">
-        <is>
-          <t>5561999511258</t>
-        </is>
+      <c r="I147" t="n">
+        <v>5561999511258</v>
       </c>
       <c r="J147" t="inlineStr"/>
       <c r="K147" t="n">
@@ -7691,10 +7671,8 @@
         </is>
       </c>
       <c r="H149" t="inlineStr"/>
-      <c r="I149" t="inlineStr">
-        <is>
-          <t>556198782133</t>
-        </is>
+      <c r="I149" t="n">
+        <v>556198782133</v>
       </c>
       <c r="J149" t="inlineStr"/>
       <c r="K149" t="n">
@@ -7791,10 +7769,8 @@
         </is>
       </c>
       <c r="H151" t="inlineStr"/>
-      <c r="I151" t="inlineStr">
-        <is>
-          <t>5561998634538</t>
-        </is>
+      <c r="I151" t="n">
+        <v>5561998634538</v>
       </c>
       <c r="J151" t="inlineStr"/>
       <c r="K151" t="n">
@@ -7843,10 +7819,8 @@
         </is>
       </c>
       <c r="H152" t="inlineStr"/>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>5561996060635</t>
-        </is>
+      <c r="I152" t="n">
+        <v>5561996060635</v>
       </c>
       <c r="J152" t="inlineStr"/>
       <c r="K152" t="n">
@@ -8135,10 +8109,8 @@
         </is>
       </c>
       <c r="H158" t="inlineStr"/>
-      <c r="I158" t="inlineStr">
-        <is>
-          <t>556139631262</t>
-        </is>
+      <c r="I158" t="n">
+        <v>556139631262</v>
       </c>
       <c r="J158" t="inlineStr"/>
       <c r="K158" t="n">
@@ -8187,10 +8159,8 @@
         </is>
       </c>
       <c r="H159" t="inlineStr"/>
-      <c r="I159" t="inlineStr">
-        <is>
-          <t>5561981536149</t>
-        </is>
+      <c r="I159" t="n">
+        <v>5561981536149</v>
       </c>
       <c r="J159" t="inlineStr"/>
       <c r="K159" t="n">
@@ -8671,10 +8641,8 @@
         </is>
       </c>
       <c r="H169" t="inlineStr"/>
-      <c r="I169" t="inlineStr">
-        <is>
-          <t>556195844771</t>
-        </is>
+      <c r="I169" t="n">
+        <v>556195844771</v>
       </c>
       <c r="J169" t="inlineStr"/>
       <c r="K169" t="n">
@@ -8723,10 +8691,8 @@
         </is>
       </c>
       <c r="H170" t="inlineStr"/>
-      <c r="I170" t="inlineStr">
-        <is>
-          <t>5561993140270</t>
-        </is>
+      <c r="I170" t="n">
+        <v>5561993140270</v>
       </c>
       <c r="J170" t="inlineStr"/>
       <c r="K170" t="n">
@@ -8775,10 +8741,8 @@
         </is>
       </c>
       <c r="H171" t="inlineStr"/>
-      <c r="I171" t="inlineStr">
-        <is>
-          <t>5511974139514</t>
-        </is>
+      <c r="I171" t="n">
+        <v>5511974139514</v>
       </c>
       <c r="J171" t="inlineStr"/>
       <c r="K171" t="n">
@@ -8971,10 +8935,8 @@
         </is>
       </c>
       <c r="H175" t="inlineStr"/>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t>556235454000</t>
-        </is>
+      <c r="I175" t="n">
+        <v>556235454000</v>
       </c>
       <c r="J175" t="inlineStr"/>
       <c r="K175" t="n">
@@ -9023,10 +8985,8 @@
         </is>
       </c>
       <c r="H176" t="inlineStr"/>
-      <c r="I176" t="inlineStr">
-        <is>
-          <t>5564984390766</t>
-        </is>
+      <c r="I176" t="n">
+        <v>5564984390766</v>
       </c>
       <c r="J176" t="inlineStr"/>
       <c r="K176" t="n">
@@ -9075,10 +9035,8 @@
         </is>
       </c>
       <c r="H177" t="inlineStr"/>
-      <c r="I177" t="inlineStr">
-        <is>
-          <t>556239960505</t>
-        </is>
+      <c r="I177" t="n">
+        <v>556239960505</v>
       </c>
       <c r="J177" t="inlineStr"/>
       <c r="K177" t="n">
@@ -9127,10 +9085,8 @@
         </is>
       </c>
       <c r="H178" t="inlineStr"/>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>5562998256655</t>
-        </is>
+      <c r="I178" t="n">
+        <v>5562998256655</v>
       </c>
       <c r="J178" t="inlineStr"/>
       <c r="K178" t="n">
@@ -9323,10 +9279,8 @@
         </is>
       </c>
       <c r="H182" t="inlineStr"/>
-      <c r="I182" t="inlineStr">
-        <is>
-          <t>556232512898</t>
-        </is>
+      <c r="I182" t="n">
+        <v>556232512898</v>
       </c>
       <c r="J182" t="inlineStr"/>
       <c r="K182" t="n">
@@ -9519,10 +9473,8 @@
         </is>
       </c>
       <c r="H186" t="inlineStr"/>
-      <c r="I186" t="inlineStr">
-        <is>
-          <t>5511912062131</t>
-        </is>
+      <c r="I186" t="n">
+        <v>5511912062131</v>
       </c>
       <c r="J186" t="inlineStr"/>
       <c r="K186" t="n">
@@ -9571,10 +9523,8 @@
         </is>
       </c>
       <c r="H187" t="inlineStr"/>
-      <c r="I187" t="inlineStr">
-        <is>
-          <t>5562996304831</t>
-        </is>
+      <c r="I187" t="n">
+        <v>5562996304831</v>
       </c>
       <c r="J187" t="inlineStr"/>
       <c r="K187" t="n">
@@ -9623,10 +9573,8 @@
         </is>
       </c>
       <c r="H188" t="inlineStr"/>
-      <c r="I188" t="inlineStr">
-        <is>
-          <t>5562995531882</t>
-        </is>
+      <c r="I188" t="n">
+        <v>5562995531882</v>
       </c>
       <c r="J188" t="inlineStr"/>
       <c r="K188" t="n">
@@ -9675,10 +9623,8 @@
         </is>
       </c>
       <c r="H189" t="inlineStr"/>
-      <c r="I189" t="inlineStr">
-        <is>
-          <t>5562982663416</t>
-        </is>
+      <c r="I189" t="n">
+        <v>5562982663416</v>
       </c>
       <c r="J189" t="inlineStr"/>
       <c r="K189" t="n">
@@ -9727,10 +9673,8 @@
         </is>
       </c>
       <c r="H190" t="inlineStr"/>
-      <c r="I190" t="inlineStr">
-        <is>
-          <t>5562981426789</t>
-        </is>
+      <c r="I190" t="n">
+        <v>5562981426789</v>
       </c>
       <c r="J190" t="inlineStr"/>
       <c r="K190" t="n">
@@ -9827,10 +9771,8 @@
         </is>
       </c>
       <c r="H192" t="inlineStr"/>
-      <c r="I192" t="inlineStr">
-        <is>
-          <t>556239960508</t>
-        </is>
+      <c r="I192" t="n">
+        <v>556239960508</v>
       </c>
       <c r="J192" t="inlineStr"/>
       <c r="K192" t="n">
@@ -9879,10 +9821,8 @@
         </is>
       </c>
       <c r="H193" t="inlineStr"/>
-      <c r="I193" t="inlineStr">
-        <is>
-          <t>5562999234619</t>
-        </is>
+      <c r="I193" t="n">
+        <v>5562999234619</v>
       </c>
       <c r="J193" t="inlineStr"/>
       <c r="K193" t="n">
@@ -9979,10 +9919,8 @@
         </is>
       </c>
       <c r="H195" t="inlineStr"/>
-      <c r="I195" t="inlineStr">
-        <is>
-          <t>5562992899057</t>
-        </is>
+      <c r="I195" t="n">
+        <v>5562992899057</v>
       </c>
       <c r="J195" t="inlineStr"/>
       <c r="K195" t="n">
@@ -10031,10 +9969,8 @@
         </is>
       </c>
       <c r="H196" t="inlineStr"/>
-      <c r="I196" t="inlineStr">
-        <is>
-          <t>5562984796876</t>
-        </is>
+      <c r="I196" t="n">
+        <v>5562984796876</v>
       </c>
       <c r="J196" t="inlineStr"/>
       <c r="K196" t="n">
@@ -10131,10 +10067,8 @@
         </is>
       </c>
       <c r="H198" t="inlineStr"/>
-      <c r="I198" t="inlineStr">
-        <is>
-          <t>5562992347835</t>
-        </is>
+      <c r="I198" t="n">
+        <v>5562992347835</v>
       </c>
       <c r="J198" t="inlineStr"/>
       <c r="K198" t="n">
@@ -10423,10 +10357,8 @@
         </is>
       </c>
       <c r="H204" t="inlineStr"/>
-      <c r="I204" t="inlineStr">
-        <is>
-          <t>5511940747584</t>
-        </is>
+      <c r="I204" t="n">
+        <v>5511940747584</v>
       </c>
       <c r="J204" t="inlineStr"/>
       <c r="K204" t="n">
@@ -10523,10 +10455,8 @@
         </is>
       </c>
       <c r="H206" t="inlineStr"/>
-      <c r="I206" t="inlineStr">
-        <is>
-          <t>5562994359484</t>
-        </is>
+      <c r="I206" t="n">
+        <v>5562994359484</v>
       </c>
       <c r="J206" t="inlineStr"/>
       <c r="K206" t="n">
@@ -10623,16 +10553,3510 @@
         </is>
       </c>
       <c r="H208" t="inlineStr"/>
-      <c r="I208" t="inlineStr">
-        <is>
-          <t>551141183034</t>
-        </is>
+      <c r="I208" t="n">
+        <v>551141183034</v>
       </c>
       <c r="J208" t="inlineStr"/>
       <c r="K208" t="n">
         <v>69</v>
       </c>
       <c r="L208" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Moda feminina</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>https://br.shein.com</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr"/>
+      <c r="I209" t="inlineStr"/>
+      <c r="J209" t="inlineStr"/>
+      <c r="K209" t="n">
+        <v>60</v>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Os melhores médicos de Espírito Santo (ES)</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>https://www.doctoranytime.com.br</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr"/>
+      <c r="I210" t="inlineStr"/>
+      <c r="J210" t="inlineStr"/>
+      <c r="K210" t="n">
+        <v>56</v>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Prepaga</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>https://www.swissmedical.com.ar</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr"/>
+      <c r="I211" t="inlineStr"/>
+      <c r="J211" t="inlineStr"/>
+      <c r="K211" t="n">
+        <v>53</v>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>CBF</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>https://www.cbf.com.br</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr"/>
+      <c r="I212" t="inlineStr"/>
+      <c r="J212" t="inlineStr"/>
+      <c r="K212" t="n">
+        <v>0</v>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Verano Joven</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>https://veranojoven.transportes.gob.es</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr"/>
+      <c r="I213" t="inlineStr"/>
+      <c r="J213" t="inlineStr"/>
+      <c r="K213" t="n">
+        <v>33</v>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Marcadores en Vivo, Calendarios, Resultados y Tablas</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>https://es.soccerway.com</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr"/>
+      <c r="I214" t="inlineStr"/>
+      <c r="J214" t="inlineStr"/>
+      <c r="K214" t="n">
+        <v>50</v>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Victoria's Secret: sujetadores, bañadores, lencería, deporte y belleza</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>https://es.victoriassecret.com</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr"/>
+      <c r="I215" t="inlineStr"/>
+      <c r="J215" t="inlineStr"/>
+      <c r="K215" t="n">
+        <v>33</v>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Dra. Letícia Ribeiro Meirelles</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>https://www.leticiarm.com.br</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr"/>
+      <c r="I216" t="inlineStr"/>
+      <c r="J216" t="inlineStr"/>
+      <c r="K216" t="n">
+        <v>73</v>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Carminate Odontologia</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>https://carminateodontologia.com</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr"/>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>5527992716293</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr"/>
+      <c r="K217" t="n">
+        <v>73</v>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Centro de Estética Dental</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>https://www.centrodeesteticadental.com.br</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr"/>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>5527997209784</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr"/>
+      <c r="K218" t="n">
+        <v>67</v>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Dentista em Jardim Camburi</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>https://renoveodontologia.com.br</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr"/>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>5527992799432</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr"/>
+      <c r="K219" t="n">
+        <v>88</v>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Psicólogo em Vitória - ES</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>https://mail.lorenagomes.com.br</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr"/>
+      <c r="I220" t="inlineStr"/>
+      <c r="J220" t="inlineStr"/>
+      <c r="K220" t="n">
+        <v>22</v>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Maialen Fernández Psicólogos Vitoria</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>https://www.maialenfernandezpsicologia.com</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr"/>
+      <c r="I221" t="inlineStr"/>
+      <c r="J221" t="inlineStr"/>
+      <c r="K221" t="n">
+        <v>62</v>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Localizador de envíos de Correos</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>https://www.correos.es</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr"/>
+      <c r="I222" t="inlineStr"/>
+      <c r="J222" t="inlineStr"/>
+      <c r="K222" t="n">
+        <v>50</v>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Massagens, terapias corporais, estética e bem-estar no Brasil</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>https://www.pamot.com.br</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr"/>
+      <c r="I223" t="inlineStr"/>
+      <c r="J223" t="inlineStr"/>
+      <c r="K223" t="n">
+        <v>33</v>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Terapeuta Sol / Realização no toque! em Vitoria</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>https://topmassagens.com.br</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr"/>
+      <c r="I224" t="inlineStr"/>
+      <c r="J224" t="inlineStr"/>
+      <c r="K224" t="n">
+        <v>62</v>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Maria Alice Lamego de Moraes em Vitória, ES</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>https://www.econodata.com.br</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr"/>
+      <c r="I225" t="inlineStr"/>
+      <c r="J225" t="inlineStr"/>
+      <c r="K225" t="n">
+        <v>22</v>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Charming apartment-Jdim da Penha- Vitória, ES -Brazil...</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>https://www.airbnb.com</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr"/>
+      <c r="I226" t="inlineStr"/>
+      <c r="J226" t="inlineStr"/>
+      <c r="K226" t="n">
+        <v>44</v>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Barroso Advogados</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>https://www.barrosoadvogados.etc.br</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr"/>
+      <c r="I227" t="inlineStr"/>
+      <c r="J227" t="inlineStr"/>
+      <c r="K227" t="n">
+        <v>73</v>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Advogado - Vitória</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>https://vlvadvogados.com</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr"/>
+      <c r="I228" t="inlineStr"/>
+      <c r="J228" t="inlineStr"/>
+      <c r="K228" t="n">
+        <v>64</v>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>Victor Vittore Advogados</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>https://victorvittoreadvogados.adv.br</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr"/>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>5527999045444</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr"/>
+      <c r="K229" t="n">
+        <v>64</v>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>Advogado em Vitória ES</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>https://lopesecampos.adv.br</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr"/>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>5527996901700</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr"/>
+      <c r="K230" t="n">
+        <v>100</v>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>Advogado, Vitória - ES</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>https://villeladamotta.com.br</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr"/>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>5527999489898</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr"/>
+      <c r="K231" t="n">
+        <v>73</v>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>CJAR</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>https://cjar.com.br</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr"/>
+      <c r="I232" t="inlineStr"/>
+      <c r="J232" t="inlineStr"/>
+      <c r="K232" t="n">
+        <v>82</v>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Vagas abertas em Educação Física em Vitória / ES</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>https://www.superestagios.com.br</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr"/>
+      <c r="I233" t="inlineStr"/>
+      <c r="J233" t="inlineStr"/>
+      <c r="K233" t="n">
+        <v>67</v>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>CREF22/ES</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>https://cref22.org.br</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr"/>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>5527998114107</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr"/>
+      <c r="K234" t="n">
+        <v>78</v>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Vagas de Emprego de educação fisica em Vitória - ES</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>https://www.infojobs.com.br</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr"/>
+      <c r="I235" t="inlineStr"/>
+      <c r="J235" t="inlineStr"/>
+      <c r="K235" t="n">
+        <v>73</v>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>CETEFE</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>https://cetefe.org</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr"/>
+      <c r="I236" t="inlineStr"/>
+      <c r="J236" t="inlineStr"/>
+      <c r="K236" t="n">
+        <v>78</v>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Dra. Flávia Brito</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>https://draflaviabrito.com.br</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr"/>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>5527981229670</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr"/>
+      <c r="K237" t="n">
+        <v>73</v>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Guia Médico</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>https://guiamedico.unimedvitoria.com.br</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr"/>
+      <c r="I238" t="inlineStr"/>
+      <c r="J238" t="inlineStr"/>
+      <c r="K238" t="n">
+        <v>44</v>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Vitória (ES) - Faculdade Inspirar</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>https://www.inspirar.com.br</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr"/>
+      <c r="I239" t="inlineStr"/>
+      <c r="J239" t="inlineStr"/>
+      <c r="K239" t="n">
+        <v>33</v>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Crefito 15</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>https://www.crefito15.org.br</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr"/>
+      <c r="I240" t="inlineStr"/>
+      <c r="J240" t="inlineStr"/>
+      <c r="K240" t="n">
+        <v>75</v>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Clínica Médica em Belo Horizonte: Dados 2026</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>https://ondeabrir.com</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr"/>
+      <c r="I241" t="inlineStr"/>
+      <c r="J241" t="inlineStr"/>
+      <c r="K241" t="n">
+        <v>90</v>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Médicos Online em Belo Horizonte (MG)</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>https://whatsmed.com.br</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr"/>
+      <c r="I242" t="inlineStr"/>
+      <c r="J242" t="inlineStr"/>
+      <c r="K242" t="n">
+        <v>88</v>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Dental Free</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>https://www.dentalfree.com.br</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr"/>
+      <c r="I243" t="inlineStr"/>
+      <c r="J243" t="inlineStr"/>
+      <c r="K243" t="n">
+        <v>81</v>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Uniodonto Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>https://uniodontobh.com.br</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr"/>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>5531993287918</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr"/>
+      <c r="K244" t="n">
+        <v>80</v>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>LeDeux Odontologia · Clínica Premium em Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>https://ledeuxodontologia.com.br</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr"/>
+      <c r="I245" t="inlineStr"/>
+      <c r="J245" t="inlineStr"/>
+      <c r="K245" t="n">
+        <v>67</v>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>PromoDental</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>https://promodental.com.br</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr"/>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>553132533400</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr"/>
+      <c r="K246" t="n">
+        <v>75</v>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Dr Alysson Resende</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>https://www.alyssonresende.com.br</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr"/>
+      <c r="I247" t="inlineStr"/>
+      <c r="J247" t="inlineStr"/>
+      <c r="K247" t="n">
+        <v>56</v>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>https://slmandic.edu.br</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr"/>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>5519992288781</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr"/>
+      <c r="K248" t="n">
+        <v>80</v>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Psicólogo BH - Atendimento Psicológico em Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>https://www.psicologobelohorizonte.com.br</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr"/>
+      <c r="I249" t="inlineStr"/>
+      <c r="J249" t="inlineStr"/>
+      <c r="K249" t="n">
+        <v>73</v>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Psicólogos em Belo Horizonte, MG</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>https://terappy.com.br</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr"/>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>5592984020249</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr"/>
+      <c r="K250" t="n">
+        <v>73</v>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Psicólogos em Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>https://www.pratimed.com.br</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr"/>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>5521967662304</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr"/>
+      <c r="K251" t="n">
+        <v>80</v>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Auxiliadora Crepaldi</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>https://www.auxiliadoracrepaldi.com.br</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr"/>
+      <c r="I252" t="inlineStr"/>
+      <c r="J252" t="inlineStr"/>
+      <c r="K252" t="n">
+        <v>73</v>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Erika Neves</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>https://www.erikaneves.com.br</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr"/>
+      <c r="I253" t="inlineStr"/>
+      <c r="J253" t="inlineStr"/>
+      <c r="K253" t="n">
+        <v>75</v>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Advogado em Belo Horizonte (BH)</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>https://www.oliveiramiranda.adv.br</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr"/>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>5531998440357</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr"/>
+      <c r="K254" t="n">
+        <v>73</v>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Rafael Vieira</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>https://advrafael.com.br</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr"/>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>553190726984</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr"/>
+      <c r="K255" t="n">
+        <v>73</v>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>André Beliene</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>https://andrebelieneadvogado.com.br</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr"/>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>5531995356105</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr"/>
+      <c r="K256" t="n">
+        <v>73</v>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Escritório de Advocacia em BH</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>https://settemadvogados.com.br</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr"/>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>5531981062500</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr"/>
+      <c r="K257" t="n">
+        <v>73</v>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Túlio Vianna Advocacia Criminal</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>https://tuliovianna.adv.br</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr"/>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>5531998551641</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr"/>
+      <c r="K258" t="n">
+        <v>73</v>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Rômulo Brasil Advogados</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>https://romulobrasil.adv.br</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr"/>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>553181016517</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr"/>
+      <c r="K259" t="n">
+        <v>73</v>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Josimar Bezerra Advogados</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>https://www.josimarbezerraadvogados.com.br</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr"/>
+      <c r="I260" t="inlineStr"/>
+      <c r="J260" t="inlineStr"/>
+      <c r="K260" t="n">
+        <v>45</v>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Educação Física</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>https://www.defisd.cefetmg.br</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr"/>
+      <c r="I261" t="inlineStr"/>
+      <c r="J261" t="inlineStr"/>
+      <c r="K261" t="n">
+        <v>0</v>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Bacharelado em Educação Física</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>https://www.unibh.br</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr"/>
+      <c r="I262" t="inlineStr"/>
+      <c r="J262" t="inlineStr"/>
+      <c r="K262" t="n">
+        <v>62</v>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Educação Física (Bacharelado)</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>https://www.ufmg.br</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr"/>
+      <c r="I263" t="inlineStr"/>
+      <c r="J263" t="inlineStr"/>
+      <c r="K263" t="n">
+        <v>67</v>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Faculdade de EDUCAÇÃO FÍSICA em BELO HORIZONTE</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>https://www.educamaisbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr"/>
+      <c r="I264" t="inlineStr"/>
+      <c r="J264" t="inlineStr"/>
+      <c r="K264" t="n">
+        <v>44</v>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>EEFFTO</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>https://www.eeffto.ufmg.br</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr"/>
+      <c r="I265" t="inlineStr"/>
+      <c r="J265" t="inlineStr"/>
+      <c r="K265" t="n">
+        <v>0</v>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Apartamentos com academia para alugar perto de...</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>https://www.quintoandar.com.br</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr"/>
+      <c r="I266" t="inlineStr"/>
+      <c r="J266" t="inlineStr"/>
+      <c r="K266" t="n">
+        <v>80</v>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>De Belo Horizonte, MG para Timóteo, MG de ônibus</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>https://www.checkmybus.com.br</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr"/>
+      <c r="I267" t="inlineStr"/>
+      <c r="J267" t="inlineStr"/>
+      <c r="K267" t="n">
+        <v>67</v>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>ONEFIT ACADEMIA, Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>https://br.polomap.com</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr"/>
+      <c r="I268" t="inlineStr"/>
+      <c r="J268" t="inlineStr"/>
+      <c r="K268" t="n">
+        <v>33</v>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Fisioterapeuta em Belo Horizonte-MG</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>https://cliniguia.com</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr"/>
+      <c r="I269" t="inlineStr"/>
+      <c r="J269" t="inlineStr"/>
+      <c r="K269" t="n">
+        <v>56</v>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>A Clínica Biophysical</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>https://www.clinicadefisioterapiabh.com.br</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr"/>
+      <c r="I270" t="inlineStr"/>
+      <c r="J270" t="inlineStr"/>
+      <c r="K270" t="n">
+        <v>67</v>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>médico Rio de Janeiro em Rio de Janeiro (RJ)</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>https://zapvida.com</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr"/>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>554792174808</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr"/>
+      <c r="K271" t="n">
+        <v>75</v>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Centro Médico Rio Barra: Consultas, Centro Médico...</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>https://portaljpa.com</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr"/>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>5521980769543</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr"/>
+      <c r="K272" t="n">
+        <v>64</v>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Dr. Carlos Henrique Ferreira Cruz, Médico - Perfil completo</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>https://www.medstream.com.br</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr"/>
+      <c r="I273" t="inlineStr"/>
+      <c r="J273" t="inlineStr"/>
+      <c r="K273" t="n">
+        <v>53</v>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Anúncio: Propagandista médico (rio de janeiro) #950703</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>https://www.netvagas.com.br</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr"/>
+      <c r="I274" t="inlineStr"/>
+      <c r="J274" t="inlineStr"/>
+      <c r="K274" t="n">
+        <v>56</v>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Universidade Federal do Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>https://ufrj.br</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr"/>
+      <c r="I275" t="inlineStr"/>
+      <c r="J275" t="inlineStr"/>
+      <c r="K275" t="n">
+        <v>76</v>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Dr. Bruno Abrantes, Cirurgião-Dentista - Perfil completo</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>https://www.ident.com.br</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr"/>
+      <c r="I276" t="inlineStr"/>
+      <c r="J276" t="inlineStr"/>
+      <c r="K276" t="n">
+        <v>62</v>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Melhores Dentista Do Rio De Janeiro Rj em Rio de Janeiro RJ...</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>https://portaljpa.com.br</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr"/>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>5521980769543</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr"/>
+      <c r="K277" t="n">
+        <v>64</v>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Reservas e descontos nos motéis da Zona Norte do Rio de Janeiro...</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>https://www.guiademoteis.com.br</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr"/>
+      <c r="I278" t="inlineStr"/>
+      <c r="J278" t="inlineStr"/>
+      <c r="K278" t="n">
+        <v>33</v>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Scenic Aerial View of Rio de Janeiro Coastline · Free Stock Photo</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>https://www.pexels.com</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr"/>
+      <c r="I279" t="inlineStr"/>
+      <c r="J279" t="inlineStr"/>
+      <c r="K279" t="n">
+        <v>33</v>
+      </c>
+      <c r="L279" t="inlineStr">
         <is>
           <t>Crítico</t>
         </is>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade — Sul 2026-07-26
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L279"/>
+  <dimension ref="A1:L349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10987,10 +10987,8 @@
         </is>
       </c>
       <c r="H217" t="inlineStr"/>
-      <c r="I217" t="inlineStr">
-        <is>
-          <t>5527992716293</t>
-        </is>
+      <c r="I217" t="n">
+        <v>5527992716293</v>
       </c>
       <c r="J217" t="inlineStr"/>
       <c r="K217" t="n">
@@ -11039,10 +11037,8 @@
         </is>
       </c>
       <c r="H218" t="inlineStr"/>
-      <c r="I218" t="inlineStr">
-        <is>
-          <t>5527997209784</t>
-        </is>
+      <c r="I218" t="n">
+        <v>5527997209784</v>
       </c>
       <c r="J218" t="inlineStr"/>
       <c r="K218" t="n">
@@ -11091,10 +11087,8 @@
         </is>
       </c>
       <c r="H219" t="inlineStr"/>
-      <c r="I219" t="inlineStr">
-        <is>
-          <t>5527992799432</t>
-        </is>
+      <c r="I219" t="n">
+        <v>5527992799432</v>
       </c>
       <c r="J219" t="inlineStr"/>
       <c r="K219" t="n">
@@ -11575,10 +11569,8 @@
         </is>
       </c>
       <c r="H229" t="inlineStr"/>
-      <c r="I229" t="inlineStr">
-        <is>
-          <t>5527999045444</t>
-        </is>
+      <c r="I229" t="n">
+        <v>5527999045444</v>
       </c>
       <c r="J229" t="inlineStr"/>
       <c r="K229" t="n">
@@ -11627,10 +11619,8 @@
         </is>
       </c>
       <c r="H230" t="inlineStr"/>
-      <c r="I230" t="inlineStr">
-        <is>
-          <t>5527996901700</t>
-        </is>
+      <c r="I230" t="n">
+        <v>5527996901700</v>
       </c>
       <c r="J230" t="inlineStr"/>
       <c r="K230" t="n">
@@ -11679,10 +11669,8 @@
         </is>
       </c>
       <c r="H231" t="inlineStr"/>
-      <c r="I231" t="inlineStr">
-        <is>
-          <t>5527999489898</t>
-        </is>
+      <c r="I231" t="n">
+        <v>5527999489898</v>
       </c>
       <c r="J231" t="inlineStr"/>
       <c r="K231" t="n">
@@ -11827,10 +11815,8 @@
         </is>
       </c>
       <c r="H234" t="inlineStr"/>
-      <c r="I234" t="inlineStr">
-        <is>
-          <t>5527998114107</t>
-        </is>
+      <c r="I234" t="n">
+        <v>5527998114107</v>
       </c>
       <c r="J234" t="inlineStr"/>
       <c r="K234" t="n">
@@ -11975,10 +11961,8 @@
         </is>
       </c>
       <c r="H237" t="inlineStr"/>
-      <c r="I237" t="inlineStr">
-        <is>
-          <t>5527981229670</t>
-        </is>
+      <c r="I237" t="n">
+        <v>5527981229670</v>
       </c>
       <c r="J237" t="inlineStr"/>
       <c r="K237" t="n">
@@ -12315,10 +12299,8 @@
         </is>
       </c>
       <c r="H244" t="inlineStr"/>
-      <c r="I244" t="inlineStr">
-        <is>
-          <t>5531993287918</t>
-        </is>
+      <c r="I244" t="n">
+        <v>5531993287918</v>
       </c>
       <c r="J244" t="inlineStr"/>
       <c r="K244" t="n">
@@ -12415,10 +12397,8 @@
         </is>
       </c>
       <c r="H246" t="inlineStr"/>
-      <c r="I246" t="inlineStr">
-        <is>
-          <t>553132533400</t>
-        </is>
+      <c r="I246" t="n">
+        <v>553132533400</v>
       </c>
       <c r="J246" t="inlineStr"/>
       <c r="K246" t="n">
@@ -12515,10 +12495,8 @@
         </is>
       </c>
       <c r="H248" t="inlineStr"/>
-      <c r="I248" t="inlineStr">
-        <is>
-          <t>5519992288781</t>
-        </is>
+      <c r="I248" t="n">
+        <v>5519992288781</v>
       </c>
       <c r="J248" t="inlineStr"/>
       <c r="K248" t="n">
@@ -12615,10 +12593,8 @@
         </is>
       </c>
       <c r="H250" t="inlineStr"/>
-      <c r="I250" t="inlineStr">
-        <is>
-          <t>5592984020249</t>
-        </is>
+      <c r="I250" t="n">
+        <v>5592984020249</v>
       </c>
       <c r="J250" t="inlineStr"/>
       <c r="K250" t="n">
@@ -12667,10 +12643,8 @@
         </is>
       </c>
       <c r="H251" t="inlineStr"/>
-      <c r="I251" t="inlineStr">
-        <is>
-          <t>5521967662304</t>
-        </is>
+      <c r="I251" t="n">
+        <v>5521967662304</v>
       </c>
       <c r="J251" t="inlineStr"/>
       <c r="K251" t="n">
@@ -12815,10 +12789,8 @@
         </is>
       </c>
       <c r="H254" t="inlineStr"/>
-      <c r="I254" t="inlineStr">
-        <is>
-          <t>5531998440357</t>
-        </is>
+      <c r="I254" t="n">
+        <v>5531998440357</v>
       </c>
       <c r="J254" t="inlineStr"/>
       <c r="K254" t="n">
@@ -12867,10 +12839,8 @@
         </is>
       </c>
       <c r="H255" t="inlineStr"/>
-      <c r="I255" t="inlineStr">
-        <is>
-          <t>553190726984</t>
-        </is>
+      <c r="I255" t="n">
+        <v>553190726984</v>
       </c>
       <c r="J255" t="inlineStr"/>
       <c r="K255" t="n">
@@ -12919,10 +12889,8 @@
         </is>
       </c>
       <c r="H256" t="inlineStr"/>
-      <c r="I256" t="inlineStr">
-        <is>
-          <t>5531995356105</t>
-        </is>
+      <c r="I256" t="n">
+        <v>5531995356105</v>
       </c>
       <c r="J256" t="inlineStr"/>
       <c r="K256" t="n">
@@ -12971,10 +12939,8 @@
         </is>
       </c>
       <c r="H257" t="inlineStr"/>
-      <c r="I257" t="inlineStr">
-        <is>
-          <t>5531981062500</t>
-        </is>
+      <c r="I257" t="n">
+        <v>5531981062500</v>
       </c>
       <c r="J257" t="inlineStr"/>
       <c r="K257" t="n">
@@ -13023,10 +12989,8 @@
         </is>
       </c>
       <c r="H258" t="inlineStr"/>
-      <c r="I258" t="inlineStr">
-        <is>
-          <t>5531998551641</t>
-        </is>
+      <c r="I258" t="n">
+        <v>5531998551641</v>
       </c>
       <c r="J258" t="inlineStr"/>
       <c r="K258" t="n">
@@ -13075,10 +13039,8 @@
         </is>
       </c>
       <c r="H259" t="inlineStr"/>
-      <c r="I259" t="inlineStr">
-        <is>
-          <t>553181016517</t>
-        </is>
+      <c r="I259" t="n">
+        <v>553181016517</v>
       </c>
       <c r="J259" t="inlineStr"/>
       <c r="K259" t="n">
@@ -13655,10 +13617,8 @@
         </is>
       </c>
       <c r="H271" t="inlineStr"/>
-      <c r="I271" t="inlineStr">
-        <is>
-          <t>554792174808</t>
-        </is>
+      <c r="I271" t="n">
+        <v>554792174808</v>
       </c>
       <c r="J271" t="inlineStr"/>
       <c r="K271" t="n">
@@ -13707,10 +13667,8 @@
         </is>
       </c>
       <c r="H272" t="inlineStr"/>
-      <c r="I272" t="inlineStr">
-        <is>
-          <t>5521980769543</t>
-        </is>
+      <c r="I272" t="n">
+        <v>5521980769543</v>
       </c>
       <c r="J272" t="inlineStr"/>
       <c r="K272" t="n">
@@ -13951,10 +13909,8 @@
         </is>
       </c>
       <c r="H277" t="inlineStr"/>
-      <c r="I277" t="inlineStr">
-        <is>
-          <t>5521980769543</t>
-        </is>
+      <c r="I277" t="n">
+        <v>5521980769543</v>
       </c>
       <c r="J277" t="inlineStr"/>
       <c r="K277" t="n">
@@ -14062,6 +14018,3490 @@
         </is>
       </c>
     </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Centro Médico Adventista</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>https://curitiba.clinicaadventista.org.br</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr"/>
+      <c r="I280" t="inlineStr"/>
+      <c r="J280" t="inlineStr"/>
+      <c r="K280" t="n">
+        <v>22</v>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Centro Médico em Curitiba</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>https://incorporecentromedico.com.br</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr"/>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>5541998281051</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr"/>
+      <c r="K281" t="n">
+        <v>88</v>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Paraná Clínicas</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>https://paranaclinicas.com.br</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr"/>
+      <c r="I282" t="inlineStr"/>
+      <c r="J282" t="inlineStr"/>
+      <c r="K282" t="n">
+        <v>71</v>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Clínica Médica</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>https://santacasacuritiba.com.br</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr"/>
+      <c r="I283" t="inlineStr"/>
+      <c r="J283" t="inlineStr"/>
+      <c r="K283" t="n">
+        <v>76</v>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>CMI - Centro Médico Integrado Curitiba</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>https://cmicentromedicointegrado.com.br</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr"/>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>5541991980029</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr"/>
+      <c r="K284" t="n">
+        <v>87</v>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Policlínica Capão Raso</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>https://policlinicacapaoraso.com.br</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr"/>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>5541985084617</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr"/>
+      <c r="K285" t="n">
+        <v>64</v>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Ventura Clínica</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>https://venturaclinica.com.br</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr"/>
+      <c r="I286" t="inlineStr"/>
+      <c r="J286" t="inlineStr"/>
+      <c r="K286" t="n">
+        <v>65</v>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Médicos Curitiba</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>https://medicos.curitiba.br</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr"/>
+      <c r="I287" t="inlineStr"/>
+      <c r="J287" t="inlineStr"/>
+      <c r="K287" t="n">
+        <v>0</v>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Dr. Shadi Abdulla</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>https://www.shadiabdulla.com.br</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr"/>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>5541995181395</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr"/>
+      <c r="K288" t="n">
+        <v>69</v>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Dentistas Curitiba</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>https://dentistas.curitiba.br</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr"/>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>5541991447326</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr"/>
+      <c r="K289" t="n">
+        <v>87</v>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Curitiba Dental Office</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>https://www.curitibadentaloffice.com.br</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr"/>
+      <c r="I290" t="inlineStr"/>
+      <c r="J290" t="inlineStr"/>
+      <c r="K290" t="n">
+        <v>75</v>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Clínica de Odontologia em Curitiba, PR: Serviços</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>https://www.up.edu.br</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr"/>
+      <c r="I291" t="inlineStr"/>
+      <c r="J291" t="inlineStr"/>
+      <c r="K291" t="n">
+        <v>44</v>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>You Odonto</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>https://youodonto.com.br</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr"/>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>5541991457638</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr"/>
+      <c r="K292" t="n">
+        <v>69</v>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>ILAPEO: Home</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>https://www.ilapeo.com.br</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr"/>
+      <c r="I293" t="inlineStr"/>
+      <c r="J293" t="inlineStr"/>
+      <c r="K293" t="n">
+        <v>75</v>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Gross Odontologia</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>https://www.grossodontologia.com.br</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr"/>
+      <c r="I294" t="inlineStr"/>
+      <c r="J294" t="inlineStr"/>
+      <c r="K294" t="n">
+        <v>69</v>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Psicólogo Curitiba — Agendar Consulta</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>https://www.psiqdoctor.com.br</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr"/>
+      <c r="I295" t="inlineStr"/>
+      <c r="J295" t="inlineStr"/>
+      <c r="K295" t="n">
+        <v>56</v>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Os 7 Psicólogos em Curitiba</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>https://terappio.com</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr"/>
+      <c r="I296" t="inlineStr"/>
+      <c r="J296" t="inlineStr"/>
+      <c r="K296" t="n">
+        <v>67</v>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Giovana Tessaro</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>https://giovanatessaro.com.br</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr"/>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>5541999954585</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr"/>
+      <c r="K297" t="n">
+        <v>73</v>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Nutty Ramos Terapeuta</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>https://www.nuttyramosterapeuta.com</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr"/>
+      <c r="I298" t="inlineStr"/>
+      <c r="J298" t="inlineStr"/>
+      <c r="K298" t="n">
+        <v>73</v>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Psicoterapias Curitiba</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>https://www.psicoterapiascuritiba.com</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr"/>
+      <c r="I299" t="inlineStr"/>
+      <c r="J299" t="inlineStr"/>
+      <c r="K299" t="n">
+        <v>33</v>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Os 10 Psicoterapeutas mais indicados em Curitiba PR</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>https://www.boaconsulta.com</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr"/>
+      <c r="I300" t="inlineStr"/>
+      <c r="J300" t="inlineStr"/>
+      <c r="K300" t="n">
+        <v>80</v>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Advogado de Direito Civil e Contratos em Curitiba</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>https://moraistavares.adv.br</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr"/>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>5532999999999</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr"/>
+      <c r="K301" t="n">
+        <v>0</v>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Pacheco Advocacia: Advogado em Curitiba</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>https://pachecoadvocacia.adv.br</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr"/>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>554196201718</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr"/>
+      <c r="K302" t="n">
+        <v>73</v>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Hapner Kroetz Advogados</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>https://www.hapnerkroetz.com.br</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr"/>
+      <c r="I303" t="inlineStr"/>
+      <c r="J303" t="inlineStr"/>
+      <c r="K303" t="n">
+        <v>82</v>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Advogado de Familia em Curitiba: Página Inicial</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>https://fladvogadocuritiba.com.br</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr"/>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>5541988652670</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr"/>
+      <c r="K304" t="n">
+        <v>73</v>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Melo Advogados</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>https://meloadvogados.com.br</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr"/>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>5541991567228</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr"/>
+      <c r="K305" t="n">
+        <v>64</v>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>HOME NOVO FSA</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>https://nfernandes.com.br</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr"/>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>5541995009977</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr"/>
+      <c r="K306" t="n">
+        <v>82</v>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Andersen Ballão Advocacia: Home</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>http://andersenballao.com.br</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr"/>
+      <c r="I307" t="inlineStr"/>
+      <c r="J307" t="inlineStr"/>
+      <c r="K307" t="n">
+        <v>89</v>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Faculdade de Educação Física em Curitiba - PR</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>https://cursos.up.edu.br</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr"/>
+      <c r="I308" t="inlineStr"/>
+      <c r="J308" t="inlineStr"/>
+      <c r="K308" t="n">
+        <v>44</v>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Educação Física</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>https://feiradecursos.ufpr.br</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr"/>
+      <c r="I309" t="inlineStr"/>
+      <c r="J309" t="inlineStr"/>
+      <c r="K309" t="n">
+        <v>33</v>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Educação Física</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>https://www.pucpr.br</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr"/>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>554132711555</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr"/>
+      <c r="K310" t="n">
+        <v>75</v>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Educação Física (Bacharelado) na PUCPR</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>https://especiais.gazetadopovo.com.br</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr"/>
+      <c r="I311" t="inlineStr"/>
+      <c r="J311" t="inlineStr"/>
+      <c r="K311" t="n">
+        <v>56</v>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>CURVES ACADEMIA - Academias</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>https://qualotelefone.com</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr"/>
+      <c r="I312" t="inlineStr"/>
+      <c r="J312" t="inlineStr"/>
+      <c r="K312" t="n">
+        <v>44</v>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>https://forceoneacademia.com.br</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr"/>
+      <c r="I313" t="inlineStr"/>
+      <c r="J313" t="inlineStr"/>
+      <c r="K313" t="n">
+        <v>80</v>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Fisioterapeuta do HC de Curitiba lança materiais informativos sobre ...</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>https://unidospelavida.org.br</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr"/>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>5541996300022</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr"/>
+      <c r="K314" t="n">
+        <v>62</v>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Congresso Internacional Inspirar de Fisioterapia Pélvica</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>https://congressopelvica.com.br</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr"/>
+      <c r="I315" t="inlineStr"/>
+      <c r="J315" t="inlineStr"/>
+      <c r="K315" t="n">
+        <v>67</v>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Salary: Recepcionista Clinica Medica in Porto Alegre, Brazil 2026</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.com</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr"/>
+      <c r="I316" t="inlineStr"/>
+      <c r="J316" t="inlineStr"/>
+      <c r="K316" t="n">
+        <v>33</v>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Derma Roller Manchas</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>https://clinicabergmann.com.br</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr"/>
+      <c r="I317" t="inlineStr"/>
+      <c r="J317" t="inlineStr"/>
+      <c r="K317" t="n">
+        <v>65</v>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Ortopedia Mariland em Porto Alegre - RS</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>https://spotway.com.br</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr"/>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>5512991730887</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr"/>
+      <c r="K318" t="n">
+        <v>81</v>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Anestesiologista em Rio Branco - Porto Alegre</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>https://www.conveniosocial.com.br</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr"/>
+      <c r="I319" t="inlineStr"/>
+      <c r="J319" t="inlineStr"/>
+      <c r="K319" t="n">
+        <v>33</v>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Clínica Popular em Porto Alegre</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>https://blog.amorsaude.com.br</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr"/>
+      <c r="I320" t="inlineStr"/>
+      <c r="J320" t="inlineStr"/>
+      <c r="K320" t="n">
+        <v>62</v>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Rede de Clínicas Médicas, Grande Porto Alegre - RS</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>https://www.clinicasalute.com.br</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr"/>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>555130141111</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr"/>
+      <c r="K321" t="n">
+        <v>75</v>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Clínica Médica em Porto Alegre</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>https://instamedsaude.com.br</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr"/>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>5551995914372</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr"/>
+      <c r="K322" t="n">
+        <v>59</v>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Teleconsulta com médicos de Porto Alegre</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>https://telemedicinamorsch.com.br</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr"/>
+      <c r="I323" t="inlineStr"/>
+      <c r="J323" t="inlineStr"/>
+      <c r="K323" t="n">
+        <v>75</v>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>Clinicentro</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>https://www.clinicentro.com.br</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr"/>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>555195560177</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr"/>
+      <c r="K324" t="n">
+        <v>67</v>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Clínica Odontológica em Porto Alegre</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>https://www.sorridere.net</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr"/>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>555133463277</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr"/>
+      <c r="K325" t="n">
+        <v>73</v>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>WK•R</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>https://www.wkrodontologia.com.br</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr"/>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>5551986648451</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr"/>
+      <c r="K326" t="n">
+        <v>73</v>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>Clínica Dental Center</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>https://clinicadentalcenter.com.br</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr"/>
+      <c r="I327" t="inlineStr"/>
+      <c r="J327" t="inlineStr"/>
+      <c r="K327" t="n">
+        <v>47</v>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Dentista na Zona Sul de Porto Alegre</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>https://www.integrareodontologia.com</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr"/>
+      <c r="I328" t="inlineStr"/>
+      <c r="J328" t="inlineStr"/>
+      <c r="K328" t="n">
+        <v>56</v>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>Centro Odontológico R8</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>https://centroodontologicor8.com.br</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr"/>
+      <c r="I329" t="inlineStr"/>
+      <c r="J329" t="inlineStr"/>
+      <c r="K329" t="n">
+        <v>53</v>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>Núcleo de Psicologia Porto Alegrense (NPPA)</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>https://www.nucleodepsicologiapoa.com</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr"/>
+      <c r="I330" t="inlineStr"/>
+      <c r="J330" t="inlineStr"/>
+      <c r="K330" t="n">
+        <v>73</v>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>Psicobreve</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>https://www.psicobreve.com.br</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr"/>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>555132262225</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr"/>
+      <c r="K331" t="n">
+        <v>80</v>
+      </c>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>Psicóloga em Porto Alegre</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>https://psicologaportoalegre.com</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr"/>
+      <c r="I332" t="inlineStr"/>
+      <c r="J332" t="inlineStr"/>
+      <c r="K332" t="n">
+        <v>80</v>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Psicologia Viva: Consulte com um psicólogo online de qualquer lugar</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>https://www.psicologiaviva.com.br</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr"/>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>5521966964821</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr"/>
+      <c r="K333" t="n">
+        <v>80</v>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Clínica de psicologia de Porto Alegre proporciona atendimento ...</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>https://gauchazh.clicrbs.com.br</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr"/>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>5551996674125</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr"/>
+      <c r="K334" t="n">
+        <v>56</v>
+      </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>Psicoterapia Online Porto Alegre</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>https://clinicarpsicologiaonline.com.br</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr"/>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>5551996786184</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr"/>
+      <c r="K335" t="n">
+        <v>80</v>
+      </c>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Boa Terapia: Psicólogo Em Porto Alegre</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>https://boaterapia.com.br</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr"/>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>555193922723</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr"/>
+      <c r="K336" t="n">
+        <v>80</v>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Psicóloga em Porto Alegre</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>https://www.rosangelapsicologa.com</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr"/>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>5551983374242</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr"/>
+      <c r="K337" t="n">
+        <v>80</v>
+      </c>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>Terapeuta Cognitivo Comportamental</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>https://www.psicologocognitivoemportoalegre.com</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr"/>
+      <c r="I338" t="inlineStr"/>
+      <c r="J338" t="inlineStr"/>
+      <c r="K338" t="n">
+        <v>67</v>
+      </c>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>Advogados e Escritórios de Advocacia em Porto Alegre</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>https://guia.poa.br</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr"/>
+      <c r="I339" t="inlineStr"/>
+      <c r="J339" t="inlineStr"/>
+      <c r="K339" t="n">
+        <v>82</v>
+      </c>
+      <c r="L339" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>106 Advogados em Porto Alegre/RS (2026)</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>https://acharadvogados.com.br</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr"/>
+      <c r="I340" t="inlineStr"/>
+      <c r="J340" t="inlineStr"/>
+      <c r="K340" t="n">
+        <v>64</v>
+      </c>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>CG Advogados</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>https://www.cgadvogados.com</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr"/>
+      <c r="I341" t="inlineStr"/>
+      <c r="J341" t="inlineStr"/>
+      <c r="K341" t="n">
+        <v>73</v>
+      </c>
+      <c r="L341" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>Portanova</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>https://www.portanova.adv.br</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr"/>
+      <c r="I342" t="inlineStr"/>
+      <c r="J342" t="inlineStr"/>
+      <c r="K342" t="n">
+        <v>73</v>
+      </c>
+      <c r="L342" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>Carpena Advogados</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>https://carpena.com.br</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr"/>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>555132333588</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr"/>
+      <c r="K343" t="n">
+        <v>82</v>
+      </c>
+      <c r="L343" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>Advogado Especialista Porto Alegre</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>https://dihladvogados.adv.br</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr"/>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>5551999882013</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr"/>
+      <c r="K344" t="n">
+        <v>100</v>
+      </c>
+      <c r="L344" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>Alves Nunes Advogados</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>https://advogadosemportoalegre.adv.br</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr"/>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>555135745063</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr"/>
+      <c r="K345" t="n">
+        <v>73</v>
+      </c>
+      <c r="L345" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>Rama Advogados Associados</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>https://www.ramaadvogados.com.br</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr"/>
+      <c r="I346" t="inlineStr"/>
+      <c r="J346" t="inlineStr"/>
+      <c r="K346" t="n">
+        <v>36</v>
+      </c>
+      <c r="L346" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>Educação Física</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>https://prefeitura.poa.br</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr"/>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>555134330156</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr"/>
+      <c r="K347" t="n">
+        <v>67</v>
+      </c>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>Educação Física</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>https://www.ulbra.br</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr"/>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>555192741192</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr"/>
+      <c r="K348" t="n">
+        <v>71</v>
+      </c>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Porto Alegre</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>As 20 melhores academias em Porto Alegre (RS) · AvataReel</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>https://avatareel.com</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr"/>
+      <c r="I349" t="inlineStr"/>
+      <c r="J349" t="inlineStr"/>
+      <c r="K349" t="n">
+        <v>44</v>
+      </c>
+      <c r="L349" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Norte, 62 novos)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L349"/>
+  <dimension ref="A1:L411"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14103,10 +14103,8 @@
         </is>
       </c>
       <c r="H281" t="inlineStr"/>
-      <c r="I281" t="inlineStr">
-        <is>
-          <t>5541998281051</t>
-        </is>
+      <c r="I281" t="n">
+        <v>5541998281051</v>
       </c>
       <c r="J281" t="inlineStr"/>
       <c r="K281" t="n">
@@ -14251,10 +14249,8 @@
         </is>
       </c>
       <c r="H284" t="inlineStr"/>
-      <c r="I284" t="inlineStr">
-        <is>
-          <t>5541991980029</t>
-        </is>
+      <c r="I284" t="n">
+        <v>5541991980029</v>
       </c>
       <c r="J284" t="inlineStr"/>
       <c r="K284" t="n">
@@ -14303,10 +14299,8 @@
         </is>
       </c>
       <c r="H285" t="inlineStr"/>
-      <c r="I285" t="inlineStr">
-        <is>
-          <t>5541985084617</t>
-        </is>
+      <c r="I285" t="n">
+        <v>5541985084617</v>
       </c>
       <c r="J285" t="inlineStr"/>
       <c r="K285" t="n">
@@ -14451,10 +14445,8 @@
         </is>
       </c>
       <c r="H288" t="inlineStr"/>
-      <c r="I288" t="inlineStr">
-        <is>
-          <t>5541995181395</t>
-        </is>
+      <c r="I288" t="n">
+        <v>5541995181395</v>
       </c>
       <c r="J288" t="inlineStr"/>
       <c r="K288" t="n">
@@ -14503,10 +14495,8 @@
         </is>
       </c>
       <c r="H289" t="inlineStr"/>
-      <c r="I289" t="inlineStr">
-        <is>
-          <t>5541991447326</t>
-        </is>
+      <c r="I289" t="n">
+        <v>5541991447326</v>
       </c>
       <c r="J289" t="inlineStr"/>
       <c r="K289" t="n">
@@ -14651,10 +14641,8 @@
         </is>
       </c>
       <c r="H292" t="inlineStr"/>
-      <c r="I292" t="inlineStr">
-        <is>
-          <t>5541991457638</t>
-        </is>
+      <c r="I292" t="n">
+        <v>5541991457638</v>
       </c>
       <c r="J292" t="inlineStr"/>
       <c r="K292" t="n">
@@ -14895,10 +14883,8 @@
         </is>
       </c>
       <c r="H297" t="inlineStr"/>
-      <c r="I297" t="inlineStr">
-        <is>
-          <t>5541999954585</t>
-        </is>
+      <c r="I297" t="n">
+        <v>5541999954585</v>
       </c>
       <c r="J297" t="inlineStr"/>
       <c r="K297" t="n">
@@ -15091,10 +15077,8 @@
         </is>
       </c>
       <c r="H301" t="inlineStr"/>
-      <c r="I301" t="inlineStr">
-        <is>
-          <t>5532999999999</t>
-        </is>
+      <c r="I301" t="n">
+        <v>5532999999999</v>
       </c>
       <c r="J301" t="inlineStr"/>
       <c r="K301" t="n">
@@ -15143,10 +15127,8 @@
         </is>
       </c>
       <c r="H302" t="inlineStr"/>
-      <c r="I302" t="inlineStr">
-        <is>
-          <t>554196201718</t>
-        </is>
+      <c r="I302" t="n">
+        <v>554196201718</v>
       </c>
       <c r="J302" t="inlineStr"/>
       <c r="K302" t="n">
@@ -15243,10 +15225,8 @@
         </is>
       </c>
       <c r="H304" t="inlineStr"/>
-      <c r="I304" t="inlineStr">
-        <is>
-          <t>5541988652670</t>
-        </is>
+      <c r="I304" t="n">
+        <v>5541988652670</v>
       </c>
       <c r="J304" t="inlineStr"/>
       <c r="K304" t="n">
@@ -15295,10 +15275,8 @@
         </is>
       </c>
       <c r="H305" t="inlineStr"/>
-      <c r="I305" t="inlineStr">
-        <is>
-          <t>5541991567228</t>
-        </is>
+      <c r="I305" t="n">
+        <v>5541991567228</v>
       </c>
       <c r="J305" t="inlineStr"/>
       <c r="K305" t="n">
@@ -15347,10 +15325,8 @@
         </is>
       </c>
       <c r="H306" t="inlineStr"/>
-      <c r="I306" t="inlineStr">
-        <is>
-          <t>5541995009977</t>
-        </is>
+      <c r="I306" t="n">
+        <v>5541995009977</v>
       </c>
       <c r="J306" t="inlineStr"/>
       <c r="K306" t="n">
@@ -15543,10 +15519,8 @@
         </is>
       </c>
       <c r="H310" t="inlineStr"/>
-      <c r="I310" t="inlineStr">
-        <is>
-          <t>554132711555</t>
-        </is>
+      <c r="I310" t="n">
+        <v>554132711555</v>
       </c>
       <c r="J310" t="inlineStr"/>
       <c r="K310" t="n">
@@ -15739,10 +15713,8 @@
         </is>
       </c>
       <c r="H314" t="inlineStr"/>
-      <c r="I314" t="inlineStr">
-        <is>
-          <t>5541996300022</t>
-        </is>
+      <c r="I314" t="n">
+        <v>5541996300022</v>
       </c>
       <c r="J314" t="inlineStr"/>
       <c r="K314" t="n">
@@ -15935,10 +15907,8 @@
         </is>
       </c>
       <c r="H318" t="inlineStr"/>
-      <c r="I318" t="inlineStr">
-        <is>
-          <t>5512991730887</t>
-        </is>
+      <c r="I318" t="n">
+        <v>5512991730887</v>
       </c>
       <c r="J318" t="inlineStr"/>
       <c r="K318" t="n">
@@ -16083,10 +16053,8 @@
         </is>
       </c>
       <c r="H321" t="inlineStr"/>
-      <c r="I321" t="inlineStr">
-        <is>
-          <t>555130141111</t>
-        </is>
+      <c r="I321" t="n">
+        <v>555130141111</v>
       </c>
       <c r="J321" t="inlineStr"/>
       <c r="K321" t="n">
@@ -16135,10 +16103,8 @@
         </is>
       </c>
       <c r="H322" t="inlineStr"/>
-      <c r="I322" t="inlineStr">
-        <is>
-          <t>5551995914372</t>
-        </is>
+      <c r="I322" t="n">
+        <v>5551995914372</v>
       </c>
       <c r="J322" t="inlineStr"/>
       <c r="K322" t="n">
@@ -16235,10 +16201,8 @@
         </is>
       </c>
       <c r="H324" t="inlineStr"/>
-      <c r="I324" t="inlineStr">
-        <is>
-          <t>555195560177</t>
-        </is>
+      <c r="I324" t="n">
+        <v>555195560177</v>
       </c>
       <c r="J324" t="inlineStr"/>
       <c r="K324" t="n">
@@ -16287,10 +16251,8 @@
         </is>
       </c>
       <c r="H325" t="inlineStr"/>
-      <c r="I325" t="inlineStr">
-        <is>
-          <t>555133463277</t>
-        </is>
+      <c r="I325" t="n">
+        <v>555133463277</v>
       </c>
       <c r="J325" t="inlineStr"/>
       <c r="K325" t="n">
@@ -16339,10 +16301,8 @@
         </is>
       </c>
       <c r="H326" t="inlineStr"/>
-      <c r="I326" t="inlineStr">
-        <is>
-          <t>5551986648451</t>
-        </is>
+      <c r="I326" t="n">
+        <v>5551986648451</v>
       </c>
       <c r="J326" t="inlineStr"/>
       <c r="K326" t="n">
@@ -16583,10 +16543,8 @@
         </is>
       </c>
       <c r="H331" t="inlineStr"/>
-      <c r="I331" t="inlineStr">
-        <is>
-          <t>555132262225</t>
-        </is>
+      <c r="I331" t="n">
+        <v>555132262225</v>
       </c>
       <c r="J331" t="inlineStr"/>
       <c r="K331" t="n">
@@ -16683,10 +16641,8 @@
         </is>
       </c>
       <c r="H333" t="inlineStr"/>
-      <c r="I333" t="inlineStr">
-        <is>
-          <t>5521966964821</t>
-        </is>
+      <c r="I333" t="n">
+        <v>5521966964821</v>
       </c>
       <c r="J333" t="inlineStr"/>
       <c r="K333" t="n">
@@ -16735,10 +16691,8 @@
         </is>
       </c>
       <c r="H334" t="inlineStr"/>
-      <c r="I334" t="inlineStr">
-        <is>
-          <t>5551996674125</t>
-        </is>
+      <c r="I334" t="n">
+        <v>5551996674125</v>
       </c>
       <c r="J334" t="inlineStr"/>
       <c r="K334" t="n">
@@ -16787,10 +16741,8 @@
         </is>
       </c>
       <c r="H335" t="inlineStr"/>
-      <c r="I335" t="inlineStr">
-        <is>
-          <t>5551996786184</t>
-        </is>
+      <c r="I335" t="n">
+        <v>5551996786184</v>
       </c>
       <c r="J335" t="inlineStr"/>
       <c r="K335" t="n">
@@ -16839,10 +16791,8 @@
         </is>
       </c>
       <c r="H336" t="inlineStr"/>
-      <c r="I336" t="inlineStr">
-        <is>
-          <t>555193922723</t>
-        </is>
+      <c r="I336" t="n">
+        <v>555193922723</v>
       </c>
       <c r="J336" t="inlineStr"/>
       <c r="K336" t="n">
@@ -16891,10 +16841,8 @@
         </is>
       </c>
       <c r="H337" t="inlineStr"/>
-      <c r="I337" t="inlineStr">
-        <is>
-          <t>5551983374242</t>
-        </is>
+      <c r="I337" t="n">
+        <v>5551983374242</v>
       </c>
       <c r="J337" t="inlineStr"/>
       <c r="K337" t="n">
@@ -17183,10 +17131,8 @@
         </is>
       </c>
       <c r="H343" t="inlineStr"/>
-      <c r="I343" t="inlineStr">
-        <is>
-          <t>555132333588</t>
-        </is>
+      <c r="I343" t="n">
+        <v>555132333588</v>
       </c>
       <c r="J343" t="inlineStr"/>
       <c r="K343" t="n">
@@ -17235,10 +17181,8 @@
         </is>
       </c>
       <c r="H344" t="inlineStr"/>
-      <c r="I344" t="inlineStr">
-        <is>
-          <t>5551999882013</t>
-        </is>
+      <c r="I344" t="n">
+        <v>5551999882013</v>
       </c>
       <c r="J344" t="inlineStr"/>
       <c r="K344" t="n">
@@ -17287,10 +17231,8 @@
         </is>
       </c>
       <c r="H345" t="inlineStr"/>
-      <c r="I345" t="inlineStr">
-        <is>
-          <t>555135745063</t>
-        </is>
+      <c r="I345" t="n">
+        <v>555135745063</v>
       </c>
       <c r="J345" t="inlineStr"/>
       <c r="K345" t="n">
@@ -17387,10 +17329,8 @@
         </is>
       </c>
       <c r="H347" t="inlineStr"/>
-      <c r="I347" t="inlineStr">
-        <is>
-          <t>555134330156</t>
-        </is>
+      <c r="I347" t="n">
+        <v>555134330156</v>
       </c>
       <c r="J347" t="inlineStr"/>
       <c r="K347" t="n">
@@ -17439,10 +17379,8 @@
         </is>
       </c>
       <c r="H348" t="inlineStr"/>
-      <c r="I348" t="inlineStr">
-        <is>
-          <t>555192741192</t>
-        </is>
+      <c r="I348" t="n">
+        <v>555192741192</v>
       </c>
       <c r="J348" t="inlineStr"/>
       <c r="K348" t="n">
@@ -17502,6 +17440,3058 @@
         </is>
       </c>
     </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>https://riobrancocentromedico.com.br</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr"/>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>5512974026261</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr"/>
+      <c r="K350" t="n">
+        <v>69</v>
+      </c>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Clinica Medicos</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>https://www.clinicamedicos.com.br</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr"/>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>5521972416496</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr"/>
+      <c r="K351" t="n">
+        <v>62</v>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>Clínica Popular Vital Brasil</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>https://www.clinicapopularvitalbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr"/>
+      <c r="I352" t="inlineStr"/>
+      <c r="J352" t="inlineStr"/>
+      <c r="K352" t="n">
+        <v>0</v>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Henrique Representante Médico</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>https://henrique-representante-medico.ueniweb.com</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr"/>
+      <c r="I353" t="inlineStr"/>
+      <c r="J353" t="inlineStr"/>
+      <c r="K353" t="n">
+        <v>93</v>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>10 MELHORES Clínicas Médicas Gerais em Rio Branco, AC</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>https://www.guiatelefone.com</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr"/>
+      <c r="I354" t="inlineStr"/>
+      <c r="J354" t="inlineStr"/>
+      <c r="K354" t="n">
+        <v>81</v>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>Guia de Saúde</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>https://realconvenios.com.br</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr"/>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>5568999847320</t>
+        </is>
+      </c>
+      <c r="J355" t="inlineStr"/>
+      <c r="K355" t="n">
+        <v>69</v>
+      </c>
+      <c r="L355" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>Dentista - Implante dentário</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>https://clinicaodontorio.com.br</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr"/>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>5568999876708</t>
+        </is>
+      </c>
+      <c r="J356" t="inlineStr"/>
+      <c r="K356" t="n">
+        <v>80</v>
+      </c>
+      <c r="L356" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>Dentistas em Rio Branco</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>https://www.encontrariobranco.com.br</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr"/>
+      <c r="I357" t="inlineStr"/>
+      <c r="J357" t="inlineStr"/>
+      <c r="K357" t="n">
+        <v>55</v>
+      </c>
+      <c r="L357" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>Psicoclean</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>https://www.psicoclean.com.br</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr"/>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>5568999897343</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr"/>
+      <c r="K358" t="n">
+        <v>73</v>
+      </c>
+      <c r="L358" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>Psicólogos em Rio Branco</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>https://mindee.me</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr"/>
+      <c r="I359" t="inlineStr"/>
+      <c r="J359" t="inlineStr"/>
+      <c r="K359" t="n">
+        <v>87</v>
+      </c>
+      <c r="L359" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>1 GUIA MÉDICO LOCAL UNIMED RIO BRANCO</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>https://unimedrb.com.br</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr"/>
+      <c r="I360" t="inlineStr"/>
+      <c r="J360" t="inlineStr"/>
+      <c r="K360" t="n">
+        <v>44</v>
+      </c>
+      <c r="L360" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>Rio Branco /AC</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>https://tehabilitar.com</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr"/>
+      <c r="I361" t="inlineStr"/>
+      <c r="J361" t="inlineStr"/>
+      <c r="K361" t="n">
+        <v>53</v>
+      </c>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>Kelly Cristina Costa Albuquerque</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>https://www.escavador.com</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr"/>
+      <c r="I362" t="inlineStr"/>
+      <c r="J362" t="inlineStr"/>
+      <c r="K362" t="n">
+        <v>33</v>
+      </c>
+      <c r="L362" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>Arteterapia como estratégia de cuidado em saúde mental no âmbito ...</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>https://www.jmphc.com.br</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr"/>
+      <c r="I363" t="inlineStr"/>
+      <c r="J363" t="inlineStr"/>
+      <c r="K363" t="n">
+        <v>60</v>
+      </c>
+      <c r="L363" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>Grupo Terapêutico em Centro de Referência para Mulheres em ...</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>https://periodicos.ufac.br</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr"/>
+      <c r="I364" t="inlineStr"/>
+      <c r="J364" t="inlineStr"/>
+      <c r="K364" t="n">
+        <v>67</v>
+      </c>
+      <c r="L364" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>Rodrigo Aiache Advogados</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>https://www.aiache.adv.br</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr"/>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>556832246324</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr"/>
+      <c r="K365" t="n">
+        <v>64</v>
+      </c>
+      <c r="L365" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>Advogados Rio Branco (Acre)</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>https://www.mundoadvogados.com.br</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr"/>
+      <c r="I366" t="inlineStr"/>
+      <c r="J366" t="inlineStr"/>
+      <c r="K366" t="n">
+        <v>0</v>
+      </c>
+      <c r="L366" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>Advogado correspondente em Rio Branco</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>https://correspondentesnaweb.com.br</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr"/>
+      <c r="I367" t="inlineStr"/>
+      <c r="J367" t="inlineStr"/>
+      <c r="K367" t="n">
+        <v>73</v>
+      </c>
+      <c r="L367" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>Efeito da atividade física programada sobre a aptidão</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>https://www.scielo.br</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr"/>
+      <c r="I368" t="inlineStr"/>
+      <c r="J368" t="inlineStr"/>
+      <c r="K368" t="n">
+        <v>22</v>
+      </c>
+      <c r="L368" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>https://www.openstreetmap.org</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr"/>
+      <c r="I369" t="inlineStr"/>
+      <c r="J369" t="inlineStr"/>
+      <c r="K369" t="n">
+        <v>33</v>
+      </c>
+      <c r="L369" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>Academias em Rio Branco, AC, Brasil</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>https://brfirmas.org</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr"/>
+      <c r="I370" t="inlineStr"/>
+      <c r="J370" t="inlineStr"/>
+      <c r="K370" t="n">
+        <v>33</v>
+      </c>
+      <c r="L370" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>Ac. Atitude - Acre — BJJ in Rio Branco</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>https://rollmap.co</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr"/>
+      <c r="I371" t="inlineStr"/>
+      <c r="J371" t="inlineStr"/>
+      <c r="K371" t="n">
+        <v>33</v>
+      </c>
+      <c r="L371" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>Link to applocal.com.br</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>https://applocal.com.br</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr"/>
+      <c r="I372" t="inlineStr"/>
+      <c r="J372" t="inlineStr"/>
+      <c r="K372" t="n">
+        <v>33</v>
+      </c>
+      <c r="L372" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>Fisioclin - Reabilitação - Fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>https://fisioclin-centro-de-reabilitacao.ueniweb.com</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr"/>
+      <c r="I373" t="inlineStr"/>
+      <c r="J373" t="inlineStr"/>
+      <c r="K373" t="n">
+        <v>93</v>
+      </c>
+      <c r="L373" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Fisiocentro - Fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>https://fisiocentro.ueniweb.com</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr"/>
+      <c r="I374" t="inlineStr"/>
+      <c r="J374" t="inlineStr"/>
+      <c r="K374" t="n">
+        <v>93</v>
+      </c>
+      <c r="L374" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Clínica Promed</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>https://www.clinicapromed.com</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr"/>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>5596991864319</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr"/>
+      <c r="K375" t="n">
+        <v>76</v>
+      </c>
+      <c r="L375" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Consultório do Povo</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>https://consultoriodopovo.com.br</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr"/>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>5596991526779</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr"/>
+      <c r="K376" t="n">
+        <v>69</v>
+      </c>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Clínica Médica</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>https://macapa.infoisinfo-br.com</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr"/>
+      <c r="I377" t="inlineStr"/>
+      <c r="J377" t="inlineStr"/>
+      <c r="K377" t="n">
+        <v>64</v>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>GUIA MÉDICO: MACAPÁ/ AP Pag.: 1</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>https://old.tjap.jus.br</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr"/>
+      <c r="I378" t="inlineStr"/>
+      <c r="J378" t="inlineStr"/>
+      <c r="K378" t="n">
+        <v>33</v>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Especialidades Médicas</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>https://www.saocamilomacapa.org.br</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr"/>
+      <c r="I379" t="inlineStr"/>
+      <c r="J379" t="inlineStr"/>
+      <c r="K379" t="n">
+        <v>91</v>
+      </c>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Consultório Dra. Marina Sales</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>https://acheioprofissional.com.br</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr"/>
+      <c r="I380" t="inlineStr"/>
+      <c r="J380" t="inlineStr"/>
+      <c r="K380" t="n">
+        <v>73</v>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Saúde Mental em Macapá</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>https://triagefy.io</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr"/>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>5548988790123</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr"/>
+      <c r="K381" t="n">
+        <v>81</v>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Unidas</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>https://www.unidas.com.br</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr"/>
+      <c r="I382" t="inlineStr"/>
+      <c r="J382" t="inlineStr"/>
+      <c r="K382" t="n">
+        <v>44</v>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Marly Barbosa</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>https://consultoriosodontologicos.com.br</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr"/>
+      <c r="I383" t="inlineStr"/>
+      <c r="J383" t="inlineStr"/>
+      <c r="K383" t="n">
+        <v>75</v>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Implantes Dentários em Macapá</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>https://www.oralsin.com.br</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr"/>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>5511956058611</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr"/>
+      <c r="K384" t="n">
+        <v>62</v>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>LIDIA PEREIRA COSTA</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>https://psicologobrasil.com</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr"/>
+      <c r="I385" t="inlineStr"/>
+      <c r="J385" t="inlineStr"/>
+      <c r="K385" t="n">
+        <v>80</v>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Psicólogo em Macapá - AP (Terapia Online)</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>https://ceciliafreytas.com.br</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr"/>
+      <c r="I386" t="inlineStr"/>
+      <c r="J386" t="inlineStr"/>
+      <c r="K386" t="n">
+        <v>81</v>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>As melhores 5 empresas de Psicólogo em Macapá</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>https://www.buscja.com</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr"/>
+      <c r="I387" t="inlineStr"/>
+      <c r="J387" t="inlineStr"/>
+      <c r="K387" t="n">
+        <v>73</v>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Advogados e Escritórios de Advocacia em Macapá</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>https://guia.macapa.br</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr"/>
+      <c r="I388" t="inlineStr"/>
+      <c r="J388" t="inlineStr"/>
+      <c r="K388" t="n">
+        <v>82</v>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Coutinho &amp; Ribeiro Advogados</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>https://www.coutinhoeribeiro.adv.br</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr"/>
+      <c r="I389" t="inlineStr"/>
+      <c r="J389" t="inlineStr"/>
+      <c r="K389" t="n">
+        <v>55</v>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Advogados em Macapá, Amapá</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>https://listaamarela.com.br</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr"/>
+      <c r="I390" t="inlineStr"/>
+      <c r="J390" t="inlineStr"/>
+      <c r="K390" t="n">
+        <v>64</v>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Frederico Vales Advogados Associados</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>https://fvales.com</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr"/>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>5596981210358</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr"/>
+      <c r="K391" t="n">
+        <v>64</v>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Advogado em Macapá/Amapá</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>https://www.ribeirocavalcante.com.br</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr"/>
+      <c r="I392" t="inlineStr"/>
+      <c r="J392" t="inlineStr"/>
+      <c r="K392" t="n">
+        <v>82</v>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Advogado em Macapá</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>https://www.galvaoesilva.com</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr"/>
+      <c r="I393" t="inlineStr"/>
+      <c r="J393" t="inlineStr"/>
+      <c r="K393" t="n">
+        <v>100</v>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Macapá (AP)</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>https://skyfitacademia.com</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr"/>
+      <c r="I394" t="inlineStr"/>
+      <c r="J394" t="inlineStr"/>
+      <c r="K394" t="n">
+        <v>40</v>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Faculdades de Macapá. UNIFAP e UNIP</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>https://www.faculdades.inf.br</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr"/>
+      <c r="I395" t="inlineStr"/>
+      <c r="J395" t="inlineStr"/>
+      <c r="K395" t="n">
+        <v>56</v>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>SKYFIT Macapá: da ideia em família à academia que virou ...</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>https://www.jornaldosmunicipiosap.com.br</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr"/>
+      <c r="I396" t="inlineStr"/>
+      <c r="J396" t="inlineStr"/>
+      <c r="K396" t="n">
+        <v>69</v>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Musculação</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>https://www.sescamapa.com.br</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr"/>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>559691525961</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr"/>
+      <c r="K397" t="n">
+        <v>80</v>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Fisioterapeutas perto de você em Macapá</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>https://fisioterapeutaspertodemim.com</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr"/>
+      <c r="I398" t="inlineStr"/>
+      <c r="J398" t="inlineStr"/>
+      <c r="K398" t="n">
+        <v>87</v>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>REABILITARE FISIOTERAPIA ESPECIALIZADA em Macapá - AP</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>https://www.acupuntura.net.br</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr"/>
+      <c r="I399" t="inlineStr"/>
+      <c r="J399" t="inlineStr"/>
+      <c r="K399" t="n">
+        <v>88</v>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Acesso Saúde Manaus</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>https://acessosaudemanaus.com.br</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr"/>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>5592994907500</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr"/>
+      <c r="K400" t="n">
+        <v>75</v>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Clínica Mais Vida Manaus</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>https://clinicamaisvida.net.br</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr"/>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>5592994937838</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr"/>
+      <c r="K401" t="n">
+        <v>76</v>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Mais Clinica</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>https://www.maisclinica.med.br</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr"/>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>559285565437</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr"/>
+      <c r="K402" t="n">
+        <v>81</v>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Upclin Manaus</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>https://upclinmanaus.com.br</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr"/>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>5592986025043</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr"/>
+      <c r="K403" t="n">
+        <v>69</v>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Ultrassonografias e Especialidades Médicas Informações</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>https://www.manausmedicalcenter.com.br</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr"/>
+      <c r="I404" t="inlineStr"/>
+      <c r="J404" t="inlineStr"/>
+      <c r="K404" t="n">
+        <v>56</v>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Sibamed</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>https://sibamedclinicamedica.com.br</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr"/>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>5592992927576</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr"/>
+      <c r="K405" t="n">
+        <v>94</v>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>Pró-Saúde</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>https://prosaudedrluizfernando.com.br</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr"/>
+      <c r="I406" t="inlineStr"/>
+      <c r="J406" t="inlineStr"/>
+      <c r="K406" t="n">
+        <v>69</v>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Convênio Médico Manaus (AM)</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>https://conveniomedico.com.br</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr"/>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>5508001115000</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr"/>
+      <c r="K407" t="n">
+        <v>53</v>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>AM: médico é afastado após ser flagrado com estagiária...</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>https://www.cnnbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr"/>
+      <c r="I408" t="inlineStr"/>
+      <c r="J408" t="inlineStr"/>
+      <c r="K408" t="n">
+        <v>82</v>
+      </c>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>Top 16 Dental Clinics &amp; Dentists in Manaus</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>https://www.dentalclinics.care</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr"/>
+      <c r="I409" t="inlineStr"/>
+      <c r="J409" t="inlineStr"/>
+      <c r="K409" t="n">
+        <v>33</v>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>Dentista em Manaus</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>https://dentistasmanaus.com.br</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr"/>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>5511912062131</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr"/>
+      <c r="K410" t="n">
+        <v>56</v>
+      </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>Dr. Sebastião Nascimento</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>https://www.sebastiao-nascimento.com</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr"/>
+      <c r="I411" t="inlineStr"/>
+      <c r="J411" t="inlineStr"/>
+      <c r="K411" t="n">
+        <v>73</v>
+      </c>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Regrava planilha de leads (410 linhas) para sincronização local
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -17477,10 +17477,8 @@
         </is>
       </c>
       <c r="H350" t="inlineStr"/>
-      <c r="I350" t="inlineStr">
-        <is>
-          <t>5512974026261</t>
-        </is>
+      <c r="I350" t="n">
+        <v>5512974026261</v>
       </c>
       <c r="J350" t="inlineStr"/>
       <c r="K350" t="n">
@@ -17529,10 +17527,8 @@
         </is>
       </c>
       <c r="H351" t="inlineStr"/>
-      <c r="I351" t="inlineStr">
-        <is>
-          <t>5521972416496</t>
-        </is>
+      <c r="I351" t="n">
+        <v>5521972416496</v>
       </c>
       <c r="J351" t="inlineStr"/>
       <c r="K351" t="n">
@@ -17725,10 +17721,8 @@
         </is>
       </c>
       <c r="H355" t="inlineStr"/>
-      <c r="I355" t="inlineStr">
-        <is>
-          <t>5568999847320</t>
-        </is>
+      <c r="I355" t="n">
+        <v>5568999847320</v>
       </c>
       <c r="J355" t="inlineStr"/>
       <c r="K355" t="n">
@@ -17777,10 +17771,8 @@
         </is>
       </c>
       <c r="H356" t="inlineStr"/>
-      <c r="I356" t="inlineStr">
-        <is>
-          <t>5568999876708</t>
-        </is>
+      <c r="I356" t="n">
+        <v>5568999876708</v>
       </c>
       <c r="J356" t="inlineStr"/>
       <c r="K356" t="n">
@@ -17877,10 +17869,8 @@
         </is>
       </c>
       <c r="H358" t="inlineStr"/>
-      <c r="I358" t="inlineStr">
-        <is>
-          <t>5568999897343</t>
-        </is>
+      <c r="I358" t="n">
+        <v>5568999897343</v>
       </c>
       <c r="J358" t="inlineStr"/>
       <c r="K358" t="n">
@@ -18217,10 +18207,8 @@
         </is>
       </c>
       <c r="H365" t="inlineStr"/>
-      <c r="I365" t="inlineStr">
-        <is>
-          <t>556832246324</t>
-        </is>
+      <c r="I365" t="n">
+        <v>556832246324</v>
       </c>
       <c r="J365" t="inlineStr"/>
       <c r="K365" t="n">
@@ -18701,10 +18689,8 @@
         </is>
       </c>
       <c r="H375" t="inlineStr"/>
-      <c r="I375" t="inlineStr">
-        <is>
-          <t>5596991864319</t>
-        </is>
+      <c r="I375" t="n">
+        <v>5596991864319</v>
       </c>
       <c r="J375" t="inlineStr"/>
       <c r="K375" t="n">
@@ -18753,10 +18739,8 @@
         </is>
       </c>
       <c r="H376" t="inlineStr"/>
-      <c r="I376" t="inlineStr">
-        <is>
-          <t>5596991526779</t>
-        </is>
+      <c r="I376" t="n">
+        <v>5596991526779</v>
       </c>
       <c r="J376" t="inlineStr"/>
       <c r="K376" t="n">
@@ -18997,10 +18981,8 @@
         </is>
       </c>
       <c r="H381" t="inlineStr"/>
-      <c r="I381" t="inlineStr">
-        <is>
-          <t>5548988790123</t>
-        </is>
+      <c r="I381" t="n">
+        <v>5548988790123</v>
       </c>
       <c r="J381" t="inlineStr"/>
       <c r="K381" t="n">
@@ -19145,10 +19127,8 @@
         </is>
       </c>
       <c r="H384" t="inlineStr"/>
-      <c r="I384" t="inlineStr">
-        <is>
-          <t>5511956058611</t>
-        </is>
+      <c r="I384" t="n">
+        <v>5511956058611</v>
       </c>
       <c r="J384" t="inlineStr"/>
       <c r="K384" t="n">
@@ -19485,10 +19465,8 @@
         </is>
       </c>
       <c r="H391" t="inlineStr"/>
-      <c r="I391" t="inlineStr">
-        <is>
-          <t>5596981210358</t>
-        </is>
+      <c r="I391" t="n">
+        <v>5596981210358</v>
       </c>
       <c r="J391" t="inlineStr"/>
       <c r="K391" t="n">
@@ -19777,10 +19755,8 @@
         </is>
       </c>
       <c r="H397" t="inlineStr"/>
-      <c r="I397" t="inlineStr">
-        <is>
-          <t>559691525961</t>
-        </is>
+      <c r="I397" t="n">
+        <v>559691525961</v>
       </c>
       <c r="J397" t="inlineStr"/>
       <c r="K397" t="n">
@@ -19925,10 +19901,8 @@
         </is>
       </c>
       <c r="H400" t="inlineStr"/>
-      <c r="I400" t="inlineStr">
-        <is>
-          <t>5592994907500</t>
-        </is>
+      <c r="I400" t="n">
+        <v>5592994907500</v>
       </c>
       <c r="J400" t="inlineStr"/>
       <c r="K400" t="n">
@@ -19977,10 +19951,8 @@
         </is>
       </c>
       <c r="H401" t="inlineStr"/>
-      <c r="I401" t="inlineStr">
-        <is>
-          <t>5592994937838</t>
-        </is>
+      <c r="I401" t="n">
+        <v>5592994937838</v>
       </c>
       <c r="J401" t="inlineStr"/>
       <c r="K401" t="n">
@@ -20029,10 +20001,8 @@
         </is>
       </c>
       <c r="H402" t="inlineStr"/>
-      <c r="I402" t="inlineStr">
-        <is>
-          <t>559285565437</t>
-        </is>
+      <c r="I402" t="n">
+        <v>559285565437</v>
       </c>
       <c r="J402" t="inlineStr"/>
       <c r="K402" t="n">
@@ -20081,10 +20051,8 @@
         </is>
       </c>
       <c r="H403" t="inlineStr"/>
-      <c r="I403" t="inlineStr">
-        <is>
-          <t>5592986025043</t>
-        </is>
+      <c r="I403" t="n">
+        <v>5592986025043</v>
       </c>
       <c r="J403" t="inlineStr"/>
       <c r="K403" t="n">
@@ -20181,10 +20149,8 @@
         </is>
       </c>
       <c r="H405" t="inlineStr"/>
-      <c r="I405" t="inlineStr">
-        <is>
-          <t>5592992927576</t>
-        </is>
+      <c r="I405" t="n">
+        <v>5592992927576</v>
       </c>
       <c r="J405" t="inlineStr"/>
       <c r="K405" t="n">
@@ -20281,10 +20247,8 @@
         </is>
       </c>
       <c r="H407" t="inlineStr"/>
-      <c r="I407" t="inlineStr">
-        <is>
-          <t>5508001115000</t>
-        </is>
+      <c r="I407" t="n">
+        <v>5508001115000</v>
       </c>
       <c r="J407" t="inlineStr"/>
       <c r="K407" t="n">
@@ -20429,10 +20393,8 @@
         </is>
       </c>
       <c r="H410" t="inlineStr"/>
-      <c r="I410" t="inlineStr">
-        <is>
-          <t>5511912062131</t>
-        </is>
+      <c r="I410" t="n">
+        <v>5511912062131</v>
       </c>
       <c r="J410" t="inlineStr"/>
       <c r="K410" t="n">

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Nordeste, +47 leads)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L411"/>
+  <dimension ref="A1:L458"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20454,6 +20454,2338 @@
         </is>
       </c>
     </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>Médico em Maceió</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>https://dragiovanaliskoski.com.br</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr"/>
+      <c r="I412" t="inlineStr"/>
+      <c r="J412" t="inlineStr"/>
+      <c r="K412" t="n">
+        <v>82</v>
+      </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Área do Médico</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>https://santacasademaceio.com.br</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr"/>
+      <c r="I413" t="inlineStr"/>
+      <c r="J413" t="inlineStr"/>
+      <c r="K413" t="n">
+        <v>33</v>
+      </c>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>Centro Médico</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>https://maceioshopping.com</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr"/>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>558221261010</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr"/>
+      <c r="K414" t="n">
+        <v>90</v>
+      </c>
+      <c r="L414" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>Dr. Mauro Barros</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>https://drmaurobarros.com</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr"/>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>5582993342119</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr"/>
+      <c r="K415" t="n">
+        <v>94</v>
+      </c>
+      <c r="L415" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>Dentista em Maceió</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>https://www.dentistaemmaceio.com.br</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr"/>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>5582991193629</t>
+        </is>
+      </c>
+      <c r="J416" t="inlineStr"/>
+      <c r="K416" t="n">
+        <v>73</v>
+      </c>
+      <c r="L416" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Dental Alagoas</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>https://dentalalagoas.com.br</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr"/>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>5582988469642</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr"/>
+      <c r="K417" t="n">
+        <v>81</v>
+      </c>
+      <c r="L417" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>Psicólogo online e terapia sem sair de casa</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>https://zenklub.com.br</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr"/>
+      <c r="I418" t="inlineStr"/>
+      <c r="J418" t="inlineStr"/>
+      <c r="K418" t="n">
+        <v>81</v>
+      </c>
+      <c r="L418" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>Gesiane Gomes Pinto</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>https://www.gesianegomespsi.com</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr"/>
+      <c r="I419" t="inlineStr"/>
+      <c r="J419" t="inlineStr"/>
+      <c r="K419" t="n">
+        <v>73</v>
+      </c>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>Maira Godoy</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>https://mairagodoy.com.br</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr"/>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>5582993344904</t>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr"/>
+      <c r="K420" t="n">
+        <v>67</v>
+      </c>
+      <c r="L420" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>Massoterapeutas em Maceió (AL)</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>https://massoterapeutas.com</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr"/>
+      <c r="I421" t="inlineStr"/>
+      <c r="J421" t="inlineStr"/>
+      <c r="K421" t="n">
+        <v>88</v>
+      </c>
+      <c r="L421" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>Espaço Terapêutico</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>https://espaco-terapeutico-maceio.ueniweb.com</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr"/>
+      <c r="I422" t="inlineStr"/>
+      <c r="J422" t="inlineStr"/>
+      <c r="K422" t="n">
+        <v>87</v>
+      </c>
+      <c r="L422" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>Advogado e Escritório de advocacia em Maceió</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>https://ssmadvogados.adv.br</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr"/>
+      <c r="I423" t="inlineStr"/>
+      <c r="J423" t="inlineStr"/>
+      <c r="K423" t="n">
+        <v>73</v>
+      </c>
+      <c r="L423" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>Advogados e Correspondentes Jurídicos em Maceió - AL</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>https://correspondentedinamico.com.br</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr"/>
+      <c r="I424" t="inlineStr"/>
+      <c r="J424" t="inlineStr"/>
+      <c r="K424" t="n">
+        <v>33</v>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>https://karpat.adv.br</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr"/>
+      <c r="I425" t="inlineStr"/>
+      <c r="J425" t="inlineStr"/>
+      <c r="K425" t="n">
+        <v>64</v>
+      </c>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>João Paulo Farias</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>https://app.diaumtododia.com.br</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr"/>
+      <c r="I426" t="inlineStr"/>
+      <c r="J426" t="inlineStr"/>
+      <c r="K426" t="n">
+        <v>33</v>
+      </c>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>O ensino remoto e as aulas de educação física durante a pandemia...</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>https://ojs.brazilianjournals.com.br</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr"/>
+      <c r="I427" t="inlineStr"/>
+      <c r="J427" t="inlineStr"/>
+      <c r="K427" t="n">
+        <v>33</v>
+      </c>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>Allp Fit Academia Maceió</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>https://localtreino.com</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr"/>
+      <c r="I428" t="inlineStr"/>
+      <c r="J428" t="inlineStr"/>
+      <c r="K428" t="n">
+        <v>56</v>
+      </c>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Maceió - vagas para fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.com.br</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr"/>
+      <c r="I429" t="inlineStr"/>
+      <c r="J429" t="inlineStr"/>
+      <c r="K429" t="n">
+        <v>22</v>
+      </c>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>Psychiatric disorders in chronic hemodialysis patients in a clinic in...</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr"/>
+      <c r="I430" t="inlineStr"/>
+      <c r="J430" t="inlineStr"/>
+      <c r="K430" t="n">
+        <v>47</v>
+      </c>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>Reserva vuelos y tiquetes aéreos online</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>https://www.avianca.com</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr"/>
+      <c r="I431" t="inlineStr"/>
+      <c r="J431" t="inlineStr"/>
+      <c r="K431" t="n">
+        <v>22</v>
+      </c>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>Dentista</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>https://www.salario.com.br</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr"/>
+      <c r="I432" t="inlineStr"/>
+      <c r="J432" t="inlineStr"/>
+      <c r="K432" t="n">
+        <v>81</v>
+      </c>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>Dr. Hamilton Andrade</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>https://drhamiltonandrade.com.br</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr"/>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>5571988918586</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr"/>
+      <c r="K433" t="n">
+        <v>93</v>
+      </c>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>Dentista em Salvador</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>https://dentistaemsalvador.com.br</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr"/>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>5571989211052</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr"/>
+      <c r="K434" t="n">
+        <v>56</v>
+      </c>
+      <c r="L434" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>Diego Tavares</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>https://diegotavarespsi.com.br</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr"/>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>5571991551191</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr"/>
+      <c r="K435" t="n">
+        <v>93</v>
+      </c>
+      <c r="L435" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>CENTRALPSI - Psicólogos em Salvador</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>https://centralpsi.com</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr"/>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>5571992240377</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr"/>
+      <c r="K436" t="n">
+        <v>69</v>
+      </c>
+      <c r="L436" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>Massagem Salvador - BA</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>https://massagemsalvador.com.br</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr"/>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>5571997432001</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr"/>
+      <c r="K437" t="n">
+        <v>87</v>
+      </c>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Bianca Terapeuta em Salvador</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>https://guiademassagista.com.br</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr"/>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>5571997432001</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr"/>
+      <c r="K438" t="n">
+        <v>88</v>
+      </c>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Estágio: Educação Física</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>https://www.futuraestagios.com.br</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr"/>
+      <c r="I439" t="inlineStr"/>
+      <c r="J439" t="inlineStr"/>
+      <c r="K439" t="n">
+        <v>78</v>
+      </c>
+      <c r="L439" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>4 Beach Gym</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>https://4beachgym.com.br</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr"/>
+      <c r="I440" t="inlineStr"/>
+      <c r="J440" t="inlineStr"/>
+      <c r="K440" t="n">
+        <v>80</v>
+      </c>
+      <c r="L440" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>Electric Body Academia XBody</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>https://electricbody.com.br</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr"/>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>5571999393214</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr"/>
+      <c r="K441" t="n">
+        <v>80</v>
+      </c>
+      <c r="L441" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Fisioterapia em Salvador - BA</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>https://www.brterapeutas.com.br</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr"/>
+      <c r="I442" t="inlineStr"/>
+      <c r="J442" t="inlineStr"/>
+      <c r="K442" t="n">
+        <v>55</v>
+      </c>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>Fisioterapia</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>https://www.espacolarsaude.com.br</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr"/>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>5571981600087</t>
+        </is>
+      </c>
+      <c r="J443" t="inlineStr"/>
+      <c r="K443" t="n">
+        <v>73</v>
+      </c>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>Neurale</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>https://neurale.com.br</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr"/>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>5571999220525</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr"/>
+      <c r="K444" t="n">
+        <v>80</v>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>Conheça espaços que oferecem fisioterapia gratuita em Salvador</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>https://www.correio24horas.com.br</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr"/>
+      <c r="I445" t="inlineStr"/>
+      <c r="J445" t="inlineStr"/>
+      <c r="K445" t="n">
+        <v>73</v>
+      </c>
+      <c r="L445" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>Fisioterapia em Salvador - BA</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>https://www.valesaude.com.br</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr"/>
+      <c r="I446" t="inlineStr"/>
+      <c r="J446" t="inlineStr"/>
+      <c r="K446" t="n">
+        <v>22</v>
+      </c>
+      <c r="L446" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>Prontoclínica de Fortaleza</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>https://prontoclinicafortaleza.com.br</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr"/>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>558533059000</t>
+        </is>
+      </c>
+      <c r="J447" t="inlineStr"/>
+      <c r="K447" t="n">
+        <v>87</v>
+      </c>
+      <c r="L447" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>Clínica Delfos</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>https://www.delfosclinica.com.br</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr"/>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>558535357373</t>
+        </is>
+      </c>
+      <c r="J448" t="inlineStr"/>
+      <c r="K448" t="n">
+        <v>73</v>
+      </c>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>Clínica Medicar</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>https://clinicamedicar.com.br</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr"/>
+      <c r="I449" t="inlineStr"/>
+      <c r="J449" t="inlineStr"/>
+      <c r="K449" t="n">
+        <v>75</v>
+      </c>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>Clinica Salud</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>https://clinicasalud.com.br</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr"/>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>5585981591045</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr"/>
+      <c r="K450" t="n">
+        <v>69</v>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>Guia Médico</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>https://www.unimedfortaleza.com.br</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr"/>
+      <c r="I451" t="inlineStr"/>
+      <c r="J451" t="inlineStr"/>
+      <c r="K451" t="n">
+        <v>76</v>
+      </c>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>Dentista en Fortaleza</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>https://esp.dentalby.com</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr"/>
+      <c r="I452" t="inlineStr"/>
+      <c r="J452" t="inlineStr"/>
+      <c r="K452" t="n">
+        <v>60</v>
+      </c>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>Vagas de emprego dentista Fortaleza, CE - 94 empregos</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>https://br.jobsora.com</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr"/>
+      <c r="I453" t="inlineStr"/>
+      <c r="J453" t="inlineStr"/>
+      <c r="K453" t="n">
+        <v>89</v>
+      </c>
+      <c r="L453" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>Os Melhores Advogados de Fortaleza</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>https://advocaciasfortaleza.com</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr"/>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>5585991507373</t>
+        </is>
+      </c>
+      <c r="J454" t="inlineStr"/>
+      <c r="K454" t="n">
+        <v>55</v>
+      </c>
+      <c r="L454" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>Advogado em Fortaleza</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>https://www.guiajus.com.br</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr"/>
+      <c r="I455" t="inlineStr"/>
+      <c r="J455" t="inlineStr"/>
+      <c r="K455" t="n">
+        <v>73</v>
+      </c>
+      <c r="L455" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>Escritório de Advocacia em Fortaleza – Ceará</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>https://azedoefranco.adv.br</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr"/>
+      <c r="I456" t="inlineStr"/>
+      <c r="J456" t="inlineStr"/>
+      <c r="K456" t="n">
+        <v>64</v>
+      </c>
+      <c r="L456" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>Instituto de Educação Física e Esportes</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>https://iefes.ufc.br</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr"/>
+      <c r="I457" t="inlineStr"/>
+      <c r="J457" t="inlineStr"/>
+      <c r="K457" t="n">
+        <v>67</v>
+      </c>
+      <c r="L457" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>Educação Física em Fortaleza — de R$157/mês</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>https://www.bolsaclick.com.br</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr"/>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>551153043216</t>
+        </is>
+      </c>
+      <c r="J458" t="inlineStr"/>
+      <c r="K458" t="n">
+        <v>91</v>
+      </c>
+      <c r="L458" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Centro-Oeste, 2026-07-28)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L458"/>
+  <dimension ref="A1:L510"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20587,10 +20587,8 @@
         </is>
       </c>
       <c r="H414" t="inlineStr"/>
-      <c r="I414" t="inlineStr">
-        <is>
-          <t>558221261010</t>
-        </is>
+      <c r="I414" t="n">
+        <v>558221261010</v>
       </c>
       <c r="J414" t="inlineStr"/>
       <c r="K414" t="n">
@@ -20639,10 +20637,8 @@
         </is>
       </c>
       <c r="H415" t="inlineStr"/>
-      <c r="I415" t="inlineStr">
-        <is>
-          <t>5582993342119</t>
-        </is>
+      <c r="I415" t="n">
+        <v>5582993342119</v>
       </c>
       <c r="J415" t="inlineStr"/>
       <c r="K415" t="n">
@@ -20691,10 +20687,8 @@
         </is>
       </c>
       <c r="H416" t="inlineStr"/>
-      <c r="I416" t="inlineStr">
-        <is>
-          <t>5582991193629</t>
-        </is>
+      <c r="I416" t="n">
+        <v>5582991193629</v>
       </c>
       <c r="J416" t="inlineStr"/>
       <c r="K416" t="n">
@@ -20743,10 +20737,8 @@
         </is>
       </c>
       <c r="H417" t="inlineStr"/>
-      <c r="I417" t="inlineStr">
-        <is>
-          <t>5582988469642</t>
-        </is>
+      <c r="I417" t="n">
+        <v>5582988469642</v>
       </c>
       <c r="J417" t="inlineStr"/>
       <c r="K417" t="n">
@@ -20891,10 +20883,8 @@
         </is>
       </c>
       <c r="H420" t="inlineStr"/>
-      <c r="I420" t="inlineStr">
-        <is>
-          <t>5582993344904</t>
-        </is>
+      <c r="I420" t="n">
+        <v>5582993344904</v>
       </c>
       <c r="J420" t="inlineStr"/>
       <c r="K420" t="n">
@@ -21519,10 +21509,8 @@
         </is>
       </c>
       <c r="H433" t="inlineStr"/>
-      <c r="I433" t="inlineStr">
-        <is>
-          <t>5571988918586</t>
-        </is>
+      <c r="I433" t="n">
+        <v>5571988918586</v>
       </c>
       <c r="J433" t="inlineStr"/>
       <c r="K433" t="n">
@@ -21571,10 +21559,8 @@
         </is>
       </c>
       <c r="H434" t="inlineStr"/>
-      <c r="I434" t="inlineStr">
-        <is>
-          <t>5571989211052</t>
-        </is>
+      <c r="I434" t="n">
+        <v>5571989211052</v>
       </c>
       <c r="J434" t="inlineStr"/>
       <c r="K434" t="n">
@@ -21623,10 +21609,8 @@
         </is>
       </c>
       <c r="H435" t="inlineStr"/>
-      <c r="I435" t="inlineStr">
-        <is>
-          <t>5571991551191</t>
-        </is>
+      <c r="I435" t="n">
+        <v>5571991551191</v>
       </c>
       <c r="J435" t="inlineStr"/>
       <c r="K435" t="n">
@@ -21675,10 +21659,8 @@
         </is>
       </c>
       <c r="H436" t="inlineStr"/>
-      <c r="I436" t="inlineStr">
-        <is>
-          <t>5571992240377</t>
-        </is>
+      <c r="I436" t="n">
+        <v>5571992240377</v>
       </c>
       <c r="J436" t="inlineStr"/>
       <c r="K436" t="n">
@@ -21727,10 +21709,8 @@
         </is>
       </c>
       <c r="H437" t="inlineStr"/>
-      <c r="I437" t="inlineStr">
-        <is>
-          <t>5571997432001</t>
-        </is>
+      <c r="I437" t="n">
+        <v>5571997432001</v>
       </c>
       <c r="J437" t="inlineStr"/>
       <c r="K437" t="n">
@@ -21779,10 +21759,8 @@
         </is>
       </c>
       <c r="H438" t="inlineStr"/>
-      <c r="I438" t="inlineStr">
-        <is>
-          <t>5571997432001</t>
-        </is>
+      <c r="I438" t="n">
+        <v>5571997432001</v>
       </c>
       <c r="J438" t="inlineStr"/>
       <c r="K438" t="n">
@@ -21927,10 +21905,8 @@
         </is>
       </c>
       <c r="H441" t="inlineStr"/>
-      <c r="I441" t="inlineStr">
-        <is>
-          <t>5571999393214</t>
-        </is>
+      <c r="I441" t="n">
+        <v>5571999393214</v>
       </c>
       <c r="J441" t="inlineStr"/>
       <c r="K441" t="n">
@@ -22027,10 +22003,8 @@
         </is>
       </c>
       <c r="H443" t="inlineStr"/>
-      <c r="I443" t="inlineStr">
-        <is>
-          <t>5571981600087</t>
-        </is>
+      <c r="I443" t="n">
+        <v>5571981600087</v>
       </c>
       <c r="J443" t="inlineStr"/>
       <c r="K443" t="n">
@@ -22079,10 +22053,8 @@
         </is>
       </c>
       <c r="H444" t="inlineStr"/>
-      <c r="I444" t="inlineStr">
-        <is>
-          <t>5571999220525</t>
-        </is>
+      <c r="I444" t="n">
+        <v>5571999220525</v>
       </c>
       <c r="J444" t="inlineStr"/>
       <c r="K444" t="n">
@@ -22227,10 +22199,8 @@
         </is>
       </c>
       <c r="H447" t="inlineStr"/>
-      <c r="I447" t="inlineStr">
-        <is>
-          <t>558533059000</t>
-        </is>
+      <c r="I447" t="n">
+        <v>558533059000</v>
       </c>
       <c r="J447" t="inlineStr"/>
       <c r="K447" t="n">
@@ -22279,10 +22249,8 @@
         </is>
       </c>
       <c r="H448" t="inlineStr"/>
-      <c r="I448" t="inlineStr">
-        <is>
-          <t>558535357373</t>
-        </is>
+      <c r="I448" t="n">
+        <v>558535357373</v>
       </c>
       <c r="J448" t="inlineStr"/>
       <c r="K448" t="n">
@@ -22379,10 +22347,8 @@
         </is>
       </c>
       <c r="H450" t="inlineStr"/>
-      <c r="I450" t="inlineStr">
-        <is>
-          <t>5585981591045</t>
-        </is>
+      <c r="I450" t="n">
+        <v>5585981591045</v>
       </c>
       <c r="J450" t="inlineStr"/>
       <c r="K450" t="n">
@@ -22575,10 +22541,8 @@
         </is>
       </c>
       <c r="H454" t="inlineStr"/>
-      <c r="I454" t="inlineStr">
-        <is>
-          <t>5585991507373</t>
-        </is>
+      <c r="I454" t="n">
+        <v>5585991507373</v>
       </c>
       <c r="J454" t="inlineStr"/>
       <c r="K454" t="n">
@@ -22771,16 +22735,2590 @@
         </is>
       </c>
       <c r="H458" t="inlineStr"/>
-      <c r="I458" t="inlineStr">
-        <is>
-          <t>551153043216</t>
-        </is>
+      <c r="I458" t="n">
+        <v>551153043216</v>
       </c>
       <c r="J458" t="inlineStr"/>
       <c r="K458" t="n">
         <v>91</v>
       </c>
       <c r="L458" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>Clínica Brasília</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>https://clinicabrasilia.bsb.br</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr"/>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>5561982302016</t>
+        </is>
+      </c>
+      <c r="J459" t="inlineStr"/>
+      <c r="K459" t="n">
+        <v>75</v>
+      </c>
+      <c r="L459" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>Clínica Médica em Brasília</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>https://www.hospitalbrasilia.com.br</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr"/>
+      <c r="I460" t="inlineStr"/>
+      <c r="J460" t="inlineStr"/>
+      <c r="K460" t="n">
+        <v>22</v>
+      </c>
+      <c r="L460" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>Clínica Médica Brasília DF</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>https://www.neurogama.com.br</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr"/>
+      <c r="I461" t="inlineStr"/>
+      <c r="J461" t="inlineStr"/>
+      <c r="K461" t="n">
+        <v>75</v>
+      </c>
+      <c r="L461" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>Clinica Médica</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>https://www.clinicagaleno.com.br</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr"/>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>5561995876121</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr"/>
+      <c r="K462" t="n">
+        <v>67</v>
+      </c>
+      <c r="L462" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>medbrasilia.com.br</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>https://medbrasilia.com.br</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr"/>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>5561992063400</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr"/>
+      <c r="K463" t="n">
+        <v>73</v>
+      </c>
+      <c r="L463" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>Nutrologia em Brasília (DF) — Agendar consulta</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>https://endoclinicas.org</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr"/>
+      <c r="I464" t="inlineStr"/>
+      <c r="J464" t="inlineStr"/>
+      <c r="K464" t="n">
+        <v>62</v>
+      </c>
+      <c r="L464" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>Cardiologia</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>https://comerciobrasilia.com.br</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr"/>
+      <c r="I465" t="inlineStr"/>
+      <c r="J465" t="inlineStr"/>
+      <c r="K465" t="n">
+        <v>69</v>
+      </c>
+      <c r="L465" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>Dentista em Brasília DF é na Ianara Pinho Odontologia</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>https://ianarapinho.odo.br</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr"/>
+      <c r="I466" t="inlineStr"/>
+      <c r="J466" t="inlineStr"/>
+      <c r="K466" t="n">
+        <v>56</v>
+      </c>
+      <c r="L466" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>Ulisses Odontologia</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>https://clinicaulissesodontologia.com.br</t>
+        </is>
+      </c>
+      <c r="H467" t="inlineStr"/>
+      <c r="I467" t="inlineStr"/>
+      <c r="J467" t="inlineStr"/>
+      <c r="K467" t="n">
+        <v>53</v>
+      </c>
+      <c r="L467" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Verifique os Melhores Dentistas em Brasília DF</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>https://brdental.com.br</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr"/>
+      <c r="I468" t="inlineStr"/>
+      <c r="J468" t="inlineStr"/>
+      <c r="K468" t="n">
+        <v>80</v>
+      </c>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>Blanca Odontologia</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>http://www.blancaodontologia.com.br</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr"/>
+      <c r="I469" t="inlineStr"/>
+      <c r="J469" t="inlineStr"/>
+      <c r="K469" t="n">
+        <v>73</v>
+      </c>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>iOrto</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>https://www.iorto.com.br</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr"/>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>5561982742299</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr"/>
+      <c r="K470" t="n">
+        <v>73</v>
+      </c>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>StudioUno Odontologia</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>https://www.clinicastudiouno.com.br</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr"/>
+      <c r="I471" t="inlineStr"/>
+      <c r="J471" t="inlineStr"/>
+      <c r="K471" t="n">
+        <v>69</v>
+      </c>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>Clínica Odontológica Brasília</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>https://www.harmonizare.com</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr"/>
+      <c r="I472" t="inlineStr"/>
+      <c r="J472" t="inlineStr"/>
+      <c r="K472" t="n">
+        <v>80</v>
+      </c>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>Sintonizze Clinica de Psicologia</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>https://www.sintonizepsicologia.com</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr"/>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>5561996511621</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr"/>
+      <c r="K473" t="n">
+        <v>75</v>
+      </c>
+      <c r="L473" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>Otávio Calile</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>https://www.otaviocalile.com</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr"/>
+      <c r="I474" t="inlineStr"/>
+      <c r="J474" t="inlineStr"/>
+      <c r="K474" t="n">
+        <v>73</v>
+      </c>
+      <c r="L474" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>Terapia Tântrica Somática em Brasília - DF</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>https://portal.paraisotantra.com.br</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr"/>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>5511958248871</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr"/>
+      <c r="K475" t="n">
+        <v>62</v>
+      </c>
+      <c r="L475" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>Jogos da Copa do Mundo Hoje: Horários (Brasília)...</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>https://radiosfutebol.com.br</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr"/>
+      <c r="I476" t="inlineStr"/>
+      <c r="J476" t="inlineStr"/>
+      <c r="K476" t="n">
+        <v>67</v>
+      </c>
+      <c r="L476" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>Advogado em Brasília - DF</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>http://advogadoinbrasilia.adv.br</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr"/>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>5561984927284</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr"/>
+      <c r="K477" t="n">
+        <v>55</v>
+      </c>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>José Neto Advogados</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>https://josenetoadvogado.com.br</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr"/>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>5561998868080</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr"/>
+      <c r="K478" t="n">
+        <v>100</v>
+      </c>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>ADVOGADO BRASÍLIA</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>https://advogadobrasiliadf.com.br</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr"/>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>5561992619440</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr"/>
+      <c r="K479" t="n">
+        <v>82</v>
+      </c>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>Advogado em Brasília</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>https://app.advogalia.com</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr"/>
+      <c r="I480" t="inlineStr"/>
+      <c r="J480" t="inlineStr"/>
+      <c r="K480" t="n">
+        <v>33</v>
+      </c>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>Edmilson Ferreira</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>https://edmilsonferreira.adv.br</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr"/>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>5561994621652</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr"/>
+      <c r="K481" t="n">
+        <v>64</v>
+      </c>
+      <c r="L481" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Rodrigues e Teles Advocacia</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>https://rodrigueseteles.adv.br</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr"/>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>5561998768256</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr"/>
+      <c r="K482" t="n">
+        <v>64</v>
+      </c>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>Veirano Advogados, Brasília - DF Office, Global</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>https://chambers.com</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr"/>
+      <c r="I483" t="inlineStr"/>
+      <c r="J483" t="inlineStr"/>
+      <c r="K483" t="n">
+        <v>33</v>
+      </c>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>Bom Dia DF</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>https://globoplay.globo.com</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr"/>
+      <c r="I484" t="inlineStr"/>
+      <c r="J484" t="inlineStr"/>
+      <c r="K484" t="n">
+        <v>56</v>
+      </c>
+      <c r="L484" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>Ironberg Águas Claras</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>https://ironbergbrasilia.com.br</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr"/>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>556136867106</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr"/>
+      <c r="K485" t="n">
+        <v>70</v>
+      </c>
+      <c r="L485" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>Fisioterapia em Brasília DF</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>https://forcafisioterapia.com.br</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr"/>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>5561984500078</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr"/>
+      <c r="K486" t="n">
+        <v>69</v>
+      </c>
+      <c r="L486" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>QUALIFISIO</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>https://www.qualifisiodf.com.br</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr"/>
+      <c r="I487" t="inlineStr"/>
+      <c r="J487" t="inlineStr"/>
+      <c r="K487" t="n">
+        <v>73</v>
+      </c>
+      <c r="L487" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>Pró Physis</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>https://prophysis.com.br</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr"/>
+      <c r="I488" t="inlineStr"/>
+      <c r="J488" t="inlineStr"/>
+      <c r="K488" t="n">
+        <v>62</v>
+      </c>
+      <c r="L488" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>Bem-vindo à Fisiobrasília</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>https://www.fisiobrasilia.com</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr"/>
+      <c r="I489" t="inlineStr"/>
+      <c r="J489" t="inlineStr"/>
+      <c r="K489" t="n">
+        <v>0</v>
+      </c>
+      <c r="L489" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>📞 Fisioterapia Brasília</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>https://imovbsb.com</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr"/>
+      <c r="I490" t="inlineStr"/>
+      <c r="J490" t="inlineStr"/>
+      <c r="K490" t="n">
+        <v>60</v>
+      </c>
+      <c r="L490" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Fetalcenter Centro Médico Goiânia</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>https://fetalcentercentromedico.com.br</t>
+        </is>
+      </c>
+      <c r="H491" t="inlineStr"/>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>5562999147414</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr"/>
+      <c r="K491" t="n">
+        <v>81</v>
+      </c>
+      <c r="L491" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Qual Melhor Clínica Médica em Goiânia</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>https://radar.med.br</t>
+        </is>
+      </c>
+      <c r="H492" t="inlineStr"/>
+      <c r="I492" t="inlineStr"/>
+      <c r="J492" t="inlineStr"/>
+      <c r="K492" t="n">
+        <v>71</v>
+      </c>
+      <c r="L492" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>FOCCOS</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>https://www.foccoscentromedico.com.br</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr"/>
+      <c r="I493" t="inlineStr"/>
+      <c r="J493" t="inlineStr"/>
+      <c r="K493" t="n">
+        <v>82</v>
+      </c>
+      <c r="L493" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>GOIÂNIA</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>https://homedoctor.com.br</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr"/>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>551136152506</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr"/>
+      <c r="K494" t="n">
+        <v>81</v>
+      </c>
+      <c r="L494" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Vitae Odontologia - Goiânia</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>https://www.vitaeodontologia.com.br</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr"/>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>5562993892212</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr"/>
+      <c r="K495" t="n">
+        <v>75</v>
+      </c>
+      <c r="L495" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Dentista em Goiânia GO</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>https://leonardobuenoodontologia.com.br</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr"/>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>5562993142324</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr"/>
+      <c r="K496" t="n">
+        <v>73</v>
+      </c>
+      <c r="L496" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>CD3 Odontologia</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>https://cd3odontologia.com.br</t>
+        </is>
+      </c>
+      <c r="H497" t="inlineStr"/>
+      <c r="I497" t="inlineStr"/>
+      <c r="J497" t="inlineStr"/>
+      <c r="K497" t="n">
+        <v>69</v>
+      </c>
+      <c r="L497" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Dentista em Goiânia Centro</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>https://odontoclinic.com.br</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr"/>
+      <c r="I498" t="inlineStr"/>
+      <c r="J498" t="inlineStr"/>
+      <c r="K498" t="n">
+        <v>33</v>
+      </c>
+      <c r="L498" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>Encontre um dentista</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>https://uniodontogoiania.coop.br</t>
+        </is>
+      </c>
+      <c r="H499" t="inlineStr"/>
+      <c r="I499" t="inlineStr"/>
+      <c r="J499" t="inlineStr"/>
+      <c r="K499" t="n">
+        <v>93</v>
+      </c>
+      <c r="L499" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Alessandra Costa</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>https://www.psicologaalessandracosta.com</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr"/>
+      <c r="I500" t="inlineStr"/>
+      <c r="J500" t="inlineStr"/>
+      <c r="K500" t="n">
+        <v>73</v>
+      </c>
+      <c r="L500" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Catão Maranhão Filho</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>https://www.psicologocatao.com</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr"/>
+      <c r="I501" t="inlineStr"/>
+      <c r="J501" t="inlineStr"/>
+      <c r="K501" t="n">
+        <v>73</v>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Psicólogo em Goiânia</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>https://www.wspsicologo.com</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr"/>
+      <c r="I502" t="inlineStr"/>
+      <c r="J502" t="inlineStr"/>
+      <c r="K502" t="n">
+        <v>81</v>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>Sousa &amp; Rizzo Advogados</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>https://sousaerizzoadvogados.com.br</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr"/>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>5561999438050</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr"/>
+      <c r="K503" t="n">
+        <v>91</v>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>Advogado em Goiânia</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>https://btediniadvocacia.com.br</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr"/>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>5562982624625</t>
+        </is>
+      </c>
+      <c r="J504" t="inlineStr"/>
+      <c r="K504" t="n">
+        <v>82</v>
+      </c>
+      <c r="L504" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>Advogado em Goiânia</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>https://fichtadvocacia.com.br</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr"/>
+      <c r="I505" t="inlineStr"/>
+      <c r="J505" t="inlineStr"/>
+      <c r="K505" t="n">
+        <v>91</v>
+      </c>
+      <c r="L505" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>Os 10 melhores Advogados em Goiânia, Brasil (2026)</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>https://lawzana.com</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr"/>
+      <c r="I506" t="inlineStr"/>
+      <c r="J506" t="inlineStr"/>
+      <c r="K506" t="n">
+        <v>33</v>
+      </c>
+      <c r="L506" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>Guia dos Melhores Escritórios de Advocacia em Goiânia GO</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>https://comerciogoiania.com.br</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr"/>
+      <c r="I507" t="inlineStr"/>
+      <c r="J507" t="inlineStr"/>
+      <c r="K507" t="n">
+        <v>64</v>
+      </c>
+      <c r="L507" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>Escobar Advogados</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>https://escobaradvogados.com</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr"/>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>556296713672</t>
+        </is>
+      </c>
+      <c r="J508" t="inlineStr"/>
+      <c r="K508" t="n">
+        <v>73</v>
+      </c>
+      <c r="L508" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>15 melhores academias nos principais setores de Goiânia</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>https://myside.com.br</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr"/>
+      <c r="I509" t="inlineStr"/>
+      <c r="J509" t="inlineStr"/>
+      <c r="K509" t="n">
+        <v>80</v>
+      </c>
+      <c r="L509" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>05 academias em Goiânia para você começar seu treino em 2026</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>https://curtamais.com.br</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr"/>
+      <c r="I510" t="inlineStr"/>
+      <c r="J510" t="inlineStr"/>
+      <c r="K510" t="n">
+        <v>33</v>
+      </c>
+      <c r="L510" t="inlineStr">
         <is>
           <t>Crítico</t>
         </is>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Nordeste, 2026-08-07)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L792"/>
+  <dimension ref="A1:L811"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38181,10 +38181,8 @@
         </is>
       </c>
       <c r="H775" t="inlineStr"/>
-      <c r="I775" t="inlineStr">
-        <is>
-          <t>551130049723</t>
-        </is>
+      <c r="I775" t="n">
+        <v>551130049723</v>
       </c>
       <c r="J775" t="inlineStr"/>
       <c r="K775" t="n">
@@ -38233,10 +38231,8 @@
         </is>
       </c>
       <c r="H776" t="inlineStr"/>
-      <c r="I776" t="inlineStr">
-        <is>
-          <t>5584991061400</t>
-        </is>
+      <c r="I776" t="n">
+        <v>5584991061400</v>
       </c>
       <c r="J776" t="inlineStr"/>
       <c r="K776" t="n">
@@ -38285,10 +38281,8 @@
         </is>
       </c>
       <c r="H777" t="inlineStr"/>
-      <c r="I777" t="inlineStr">
-        <is>
-          <t>556833027000</t>
-        </is>
+      <c r="I777" t="n">
+        <v>556833027000</v>
       </c>
       <c r="J777" t="inlineStr"/>
       <c r="K777" t="n">
@@ -38865,10 +38859,8 @@
         </is>
       </c>
       <c r="H789" t="inlineStr"/>
-      <c r="I789" t="inlineStr">
-        <is>
-          <t>5592984091888</t>
-        </is>
+      <c r="I789" t="n">
+        <v>5592984091888</v>
       </c>
       <c r="J789" t="inlineStr"/>
       <c r="K789" t="n">
@@ -38917,10 +38909,8 @@
         </is>
       </c>
       <c r="H790" t="inlineStr"/>
-      <c r="I790" t="inlineStr">
-        <is>
-          <t>5592993974848</t>
-        </is>
+      <c r="I790" t="n">
+        <v>5592993974848</v>
       </c>
       <c r="J790" t="inlineStr"/>
       <c r="K790" t="n">
@@ -38969,10 +38959,8 @@
         </is>
       </c>
       <c r="H791" t="inlineStr"/>
-      <c r="I791" t="inlineStr">
-        <is>
-          <t>5561998593861</t>
-        </is>
+      <c r="I791" t="n">
+        <v>5561998593861</v>
       </c>
       <c r="J791" t="inlineStr"/>
       <c r="K791" t="n">
@@ -39021,16 +39009,962 @@
         </is>
       </c>
       <c r="H792" t="inlineStr"/>
-      <c r="I792" t="inlineStr">
-        <is>
-          <t>5592991124340</t>
-        </is>
+      <c r="I792" t="n">
+        <v>5592991124340</v>
       </c>
       <c r="J792" t="inlineStr"/>
       <c r="K792" t="n">
         <v>93</v>
       </c>
       <c r="L792" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F793" t="inlineStr">
+        <is>
+          <t>tabuleiro</t>
+        </is>
+      </c>
+      <c r="G793" t="inlineStr">
+        <is>
+          <t>https://cpsaudemaceio.com.br</t>
+        </is>
+      </c>
+      <c r="H793" t="inlineStr"/>
+      <c r="I793" t="inlineStr"/>
+      <c r="J793" t="inlineStr"/>
+      <c r="K793" t="n">
+        <v>62</v>
+      </c>
+      <c r="L793" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F794" t="inlineStr">
+        <is>
+          <t>Clínica Médica da UNIMA</t>
+        </is>
+      </c>
+      <c r="G794" t="inlineStr">
+        <is>
+          <t>https://maceio.afya.com.br</t>
+        </is>
+      </c>
+      <c r="H794" t="inlineStr"/>
+      <c r="I794" t="inlineStr">
+        <is>
+          <t>558291260598</t>
+        </is>
+      </c>
+      <c r="J794" t="inlineStr"/>
+      <c r="K794" t="n">
+        <v>73</v>
+      </c>
+      <c r="L794" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F795" t="inlineStr">
+        <is>
+          <t>Central de Saúde</t>
+        </is>
+      </c>
+      <c r="G795" t="inlineStr">
+        <is>
+          <t>https://clinicacentraldesaude.com.br</t>
+        </is>
+      </c>
+      <c r="H795" t="inlineStr"/>
+      <c r="I795" t="inlineStr">
+        <is>
+          <t>5582988367695</t>
+        </is>
+      </c>
+      <c r="J795" t="inlineStr"/>
+      <c r="K795" t="n">
+        <v>64</v>
+      </c>
+      <c r="L795" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F796" t="inlineStr">
+        <is>
+          <t>Dentista em Maceió – AL</t>
+        </is>
+      </c>
+      <c r="G796" t="inlineStr">
+        <is>
+          <t>https://prismaodonto.com</t>
+        </is>
+      </c>
+      <c r="H796" t="inlineStr"/>
+      <c r="I796" t="inlineStr">
+        <is>
+          <t>5582996885655</t>
+        </is>
+      </c>
+      <c r="J796" t="inlineStr"/>
+      <c r="K796" t="n">
+        <v>60</v>
+      </c>
+      <c r="L796" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F797" t="inlineStr">
+        <is>
+          <t>Marianna Pereira Correia das Neves Lacerda</t>
+        </is>
+      </c>
+      <c r="G797" t="inlineStr">
+        <is>
+          <t>https://www.psimariannapereira.com</t>
+        </is>
+      </c>
+      <c r="H797" t="inlineStr"/>
+      <c r="I797" t="inlineStr"/>
+      <c r="J797" t="inlineStr"/>
+      <c r="K797" t="n">
+        <v>73</v>
+      </c>
+      <c r="L797" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F798" t="inlineStr">
+        <is>
+          <t>Débora Terapeuta Holística</t>
+        </is>
+      </c>
+      <c r="G798" t="inlineStr">
+        <is>
+          <t>https://www.topsmassagens.com.br</t>
+        </is>
+      </c>
+      <c r="H798" t="inlineStr"/>
+      <c r="I798" t="inlineStr">
+        <is>
+          <t>5582988709008</t>
+        </is>
+      </c>
+      <c r="J798" t="inlineStr"/>
+      <c r="K798" t="n">
+        <v>89</v>
+      </c>
+      <c r="L798" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F799" t="inlineStr">
+        <is>
+          <t>Gisele Costa Terapeuta Tântrica</t>
+        </is>
+      </c>
+      <c r="G799" t="inlineStr">
+        <is>
+          <t>https://massagemplusbrasil.com.br</t>
+        </is>
+      </c>
+      <c r="H799" t="inlineStr"/>
+      <c r="I799" t="inlineStr"/>
+      <c r="J799" t="inlineStr"/>
+      <c r="K799" t="n">
+        <v>76</v>
+      </c>
+      <c r="L799" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F800" t="inlineStr">
+        <is>
+          <t>ADVOGADOS EM MACEIÓ, ALAGOAS</t>
+        </is>
+      </c>
+      <c r="G800" t="inlineStr">
+        <is>
+          <t>https://www.alvesjacob.com</t>
+        </is>
+      </c>
+      <c r="H800" t="inlineStr"/>
+      <c r="I800" t="inlineStr">
+        <is>
+          <t>5521983708551</t>
+        </is>
+      </c>
+      <c r="J800" t="inlineStr"/>
+      <c r="K800" t="n">
+        <v>55</v>
+      </c>
+      <c r="L800" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F801" t="inlineStr">
+        <is>
+          <t>PSICOLOGO SALVADOR</t>
+        </is>
+      </c>
+      <c r="G801" t="inlineStr">
+        <is>
+          <t>https://psicologoemsalvador.com.br</t>
+        </is>
+      </c>
+      <c r="H801" t="inlineStr"/>
+      <c r="I801" t="inlineStr">
+        <is>
+          <t>5571992103934</t>
+        </is>
+      </c>
+      <c r="J801" t="inlineStr"/>
+      <c r="K801" t="n">
+        <v>73</v>
+      </c>
+      <c r="L801" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F802" t="inlineStr">
+        <is>
+          <t>Psicólogos em Salvador</t>
+        </is>
+      </c>
+      <c r="G802" t="inlineStr">
+        <is>
+          <t>https://clinicapsique.com</t>
+        </is>
+      </c>
+      <c r="H802" t="inlineStr"/>
+      <c r="I802" t="inlineStr"/>
+      <c r="J802" t="inlineStr"/>
+      <c r="K802" t="n">
+        <v>73</v>
+      </c>
+      <c r="L802" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F803" t="inlineStr">
+        <is>
+          <t>Terapia de Casal em Salvador</t>
+        </is>
+      </c>
+      <c r="G803" t="inlineStr">
+        <is>
+          <t>https://elidioalmeida.com.br</t>
+        </is>
+      </c>
+      <c r="H803" t="inlineStr"/>
+      <c r="I803" t="inlineStr"/>
+      <c r="J803" t="inlineStr"/>
+      <c r="K803" t="n">
+        <v>75</v>
+      </c>
+      <c r="L803" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F804" t="inlineStr">
+        <is>
+          <t>Dr. Felipe Guimarães</t>
+        </is>
+      </c>
+      <c r="G804" t="inlineStr">
+        <is>
+          <t>https://www.felipeguimaraesmd.com</t>
+        </is>
+      </c>
+      <c r="H804" t="inlineStr"/>
+      <c r="I804" t="inlineStr"/>
+      <c r="J804" t="inlineStr"/>
+      <c r="K804" t="n">
+        <v>75</v>
+      </c>
+      <c r="L804" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F805" t="inlineStr">
+        <is>
+          <t>Dra. Andrea Alencar</t>
+        </is>
+      </c>
+      <c r="G805" t="inlineStr">
+        <is>
+          <t>https://nutrologafortaleza.com.br</t>
+        </is>
+      </c>
+      <c r="H805" t="inlineStr"/>
+      <c r="I805" t="inlineStr">
+        <is>
+          <t>558582173952</t>
+        </is>
+      </c>
+      <c r="J805" t="inlineStr"/>
+      <c r="K805" t="n">
+        <v>75</v>
+      </c>
+      <c r="L805" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F806" t="inlineStr">
+        <is>
+          <t>Clínica Médica Nossa Senhora das Graças em Fortaleza</t>
+        </is>
+      </c>
+      <c r="G806" t="inlineStr">
+        <is>
+          <t>https://superdestaque.com.br</t>
+        </is>
+      </c>
+      <c r="H806" t="inlineStr"/>
+      <c r="I806" t="inlineStr"/>
+      <c r="J806" t="inlineStr"/>
+      <c r="K806" t="n">
+        <v>56</v>
+      </c>
+      <c r="L806" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F807" t="inlineStr">
+        <is>
+          <t>Telemedicina Médico de Dor</t>
+        </is>
+      </c>
+      <c r="G807" t="inlineStr">
+        <is>
+          <t>https://www.dorfortaleza.com.br</t>
+        </is>
+      </c>
+      <c r="H807" t="inlineStr"/>
+      <c r="I807" t="inlineStr"/>
+      <c r="J807" t="inlineStr"/>
+      <c r="K807" t="n">
+        <v>69</v>
+      </c>
+      <c r="L807" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F808" t="inlineStr">
+        <is>
+          <t>Centros Integrados de Medicina</t>
+        </is>
+      </c>
+      <c r="G808" t="inlineStr">
+        <is>
+          <t>https://livsaude.com.br</t>
+        </is>
+      </c>
+      <c r="H808" t="inlineStr"/>
+      <c r="I808" t="inlineStr">
+        <is>
+          <t>5508009400044</t>
+        </is>
+      </c>
+      <c r="J808" t="inlineStr"/>
+      <c r="K808" t="n">
+        <v>65</v>
+      </c>
+      <c r="L808" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F809" t="inlineStr">
+        <is>
+          <t>Dentista em Fortaleza</t>
+        </is>
+      </c>
+      <c r="G809" t="inlineStr">
+        <is>
+          <t>https://www.clinicamarcelomagalhaes.com.br</t>
+        </is>
+      </c>
+      <c r="H809" t="inlineStr"/>
+      <c r="I809" t="inlineStr">
+        <is>
+          <t>5585991780463</t>
+        </is>
+      </c>
+      <c r="J809" t="inlineStr"/>
+      <c r="K809" t="n">
+        <v>67</v>
+      </c>
+      <c r="L809" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F810" t="inlineStr">
+        <is>
+          <t>Dentista em Fortaleza</t>
+        </is>
+      </c>
+      <c r="G810" t="inlineStr">
+        <is>
+          <t>https://draalinemelo.com.br</t>
+        </is>
+      </c>
+      <c r="H810" t="inlineStr"/>
+      <c r="I810" t="inlineStr"/>
+      <c r="J810" t="inlineStr"/>
+      <c r="K810" t="n">
+        <v>69</v>
+      </c>
+      <c r="L810" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F811" t="inlineStr">
+        <is>
+          <t>Psicóloga em Fortaleza Erica Rodrigues</t>
+        </is>
+      </c>
+      <c r="G811" t="inlineStr">
+        <is>
+          <t>https://www.psicologaemfortaleza.com.br</t>
+        </is>
+      </c>
+      <c r="H811" t="inlineStr"/>
+      <c r="I811" t="inlineStr"/>
+      <c r="J811" t="inlineStr"/>
+      <c r="K811" t="n">
+        <v>0</v>
+      </c>
+      <c r="L811" t="inlineStr">
         <is>
           <t>Crítico</t>
         </is>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Sudeste, 24 novos)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L842"/>
+  <dimension ref="A1:L866"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39989,10 +39989,8 @@
         </is>
       </c>
       <c r="H812" t="inlineStr"/>
-      <c r="I812" t="inlineStr">
-        <is>
-          <t>556182022056</t>
-        </is>
+      <c r="I812" t="n">
+        <v>556182022056</v>
       </c>
       <c r="J812" t="inlineStr"/>
       <c r="K812" t="n">
@@ -40089,10 +40087,8 @@
         </is>
       </c>
       <c r="H814" t="inlineStr"/>
-      <c r="I814" t="inlineStr">
-        <is>
-          <t>5561991497434</t>
-        </is>
+      <c r="I814" t="n">
+        <v>5561991497434</v>
       </c>
       <c r="J814" t="inlineStr"/>
       <c r="K814" t="n">
@@ -40189,10 +40185,8 @@
         </is>
       </c>
       <c r="H816" t="inlineStr"/>
-      <c r="I816" t="inlineStr">
-        <is>
-          <t>5561985801610</t>
-        </is>
+      <c r="I816" t="n">
+        <v>5561985801610</v>
       </c>
       <c r="J816" t="inlineStr"/>
       <c r="K816" t="n">
@@ -40241,10 +40235,8 @@
         </is>
       </c>
       <c r="H817" t="inlineStr"/>
-      <c r="I817" t="inlineStr">
-        <is>
-          <t>5561999692026</t>
-        </is>
+      <c r="I817" t="n">
+        <v>5561999692026</v>
       </c>
       <c r="J817" t="inlineStr"/>
       <c r="K817" t="n">
@@ -40293,10 +40285,8 @@
         </is>
       </c>
       <c r="H818" t="inlineStr"/>
-      <c r="I818" t="inlineStr">
-        <is>
-          <t>5561992200973</t>
-        </is>
+      <c r="I818" t="n">
+        <v>5561992200973</v>
       </c>
       <c r="J818" t="inlineStr"/>
       <c r="K818" t="n">
@@ -40345,10 +40335,8 @@
         </is>
       </c>
       <c r="H819" t="inlineStr"/>
-      <c r="I819" t="inlineStr">
-        <is>
-          <t>5561992510446</t>
-        </is>
+      <c r="I819" t="n">
+        <v>5561992510446</v>
       </c>
       <c r="J819" t="inlineStr"/>
       <c r="K819" t="n">
@@ -40445,10 +40433,8 @@
         </is>
       </c>
       <c r="H821" t="inlineStr"/>
-      <c r="I821" t="inlineStr">
-        <is>
-          <t>5561981598841</t>
-        </is>
+      <c r="I821" t="n">
+        <v>5561981598841</v>
       </c>
       <c r="J821" t="inlineStr"/>
       <c r="K821" t="n">
@@ -40689,10 +40675,8 @@
         </is>
       </c>
       <c r="H826" t="inlineStr"/>
-      <c r="I826" t="inlineStr">
-        <is>
-          <t>556140425125</t>
-        </is>
+      <c r="I826" t="n">
+        <v>556140425125</v>
       </c>
       <c r="J826" t="inlineStr"/>
       <c r="K826" t="n">
@@ -40789,10 +40773,8 @@
         </is>
       </c>
       <c r="H828" t="inlineStr"/>
-      <c r="I828" t="inlineStr">
-        <is>
-          <t>5561998355130</t>
-        </is>
+      <c r="I828" t="n">
+        <v>5561998355130</v>
       </c>
       <c r="J828" t="inlineStr"/>
       <c r="K828" t="n">
@@ -40889,10 +40871,8 @@
         </is>
       </c>
       <c r="H830" t="inlineStr"/>
-      <c r="I830" t="inlineStr">
-        <is>
-          <t>5561996766620</t>
-        </is>
+      <c r="I830" t="n">
+        <v>5561996766620</v>
       </c>
       <c r="J830" t="inlineStr"/>
       <c r="K830" t="n">
@@ -40989,10 +40969,8 @@
         </is>
       </c>
       <c r="H832" t="inlineStr"/>
-      <c r="I832" t="inlineStr">
-        <is>
-          <t>5561994336620</t>
-        </is>
+      <c r="I832" t="n">
+        <v>5561994336620</v>
       </c>
       <c r="J832" t="inlineStr"/>
       <c r="K832" t="n">
@@ -41041,10 +41019,8 @@
         </is>
       </c>
       <c r="H833" t="inlineStr"/>
-      <c r="I833" t="inlineStr">
-        <is>
-          <t>5562999340065</t>
-        </is>
+      <c r="I833" t="n">
+        <v>5562999340065</v>
       </c>
       <c r="J833" t="inlineStr"/>
       <c r="K833" t="n">
@@ -41093,10 +41069,8 @@
         </is>
       </c>
       <c r="H834" t="inlineStr"/>
-      <c r="I834" t="inlineStr">
-        <is>
-          <t>556230863030</t>
-        </is>
+      <c r="I834" t="n">
+        <v>556230863030</v>
       </c>
       <c r="J834" t="inlineStr"/>
       <c r="K834" t="n">
@@ -41289,10 +41263,8 @@
         </is>
       </c>
       <c r="H838" t="inlineStr"/>
-      <c r="I838" t="inlineStr">
-        <is>
-          <t>5562999675135</t>
-        </is>
+      <c r="I838" t="n">
+        <v>5562999675135</v>
       </c>
       <c r="J838" t="inlineStr"/>
       <c r="K838" t="n">
@@ -41389,10 +41361,8 @@
         </is>
       </c>
       <c r="H840" t="inlineStr"/>
-      <c r="I840" t="inlineStr">
-        <is>
-          <t>5562998206942</t>
-        </is>
+      <c r="I840" t="n">
+        <v>5562998206942</v>
       </c>
       <c r="J840" t="inlineStr"/>
       <c r="K840" t="n">
@@ -41500,6 +41470,1182 @@
         </is>
       </c>
     </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>Você sabe o que faz um clínico médico? Especialista...</t>
+        </is>
+      </c>
+      <c r="G843" t="inlineStr">
+        <is>
+          <t>https://www.sitetribuna.com.br</t>
+        </is>
+      </c>
+      <c r="H843" t="inlineStr"/>
+      <c r="I843" t="inlineStr">
+        <is>
+          <t>5573991987617</t>
+        </is>
+      </c>
+      <c r="J843" t="inlineStr"/>
+      <c r="K843" t="n">
+        <v>22</v>
+      </c>
+      <c r="L843" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>Masioli Odontologia</t>
+        </is>
+      </c>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>https://masioliodontologia.com.br</t>
+        </is>
+      </c>
+      <c r="H844" t="inlineStr"/>
+      <c r="I844" t="inlineStr"/>
+      <c r="J844" t="inlineStr"/>
+      <c r="K844" t="n">
+        <v>60</v>
+      </c>
+      <c r="L844" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>Psicólogo Online Particular</t>
+        </is>
+      </c>
+      <c r="G845" t="inlineStr">
+        <is>
+          <t>https://psicologaluanaamaral.com.br</t>
+        </is>
+      </c>
+      <c r="H845" t="inlineStr"/>
+      <c r="I845" t="inlineStr">
+        <is>
+          <t>5519992289437</t>
+        </is>
+      </c>
+      <c r="J845" t="inlineStr"/>
+      <c r="K845" t="n">
+        <v>73</v>
+      </c>
+      <c r="L845" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>Terapeuta em Jardim Camburi</t>
+        </is>
+      </c>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>https://www.portaljardimcamburi.com.br</t>
+        </is>
+      </c>
+      <c r="H846" t="inlineStr"/>
+      <c r="I846" t="inlineStr"/>
+      <c r="J846" t="inlineStr"/>
+      <c r="K846" t="n">
+        <v>0</v>
+      </c>
+      <c r="L846" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>Psicóloga e Psicoterapeuta em Vitoria ES</t>
+        </is>
+      </c>
+      <c r="G847" t="inlineStr">
+        <is>
+          <t>https://laizemonteiro.com.br</t>
+        </is>
+      </c>
+      <c r="H847" t="inlineStr"/>
+      <c r="I847" t="inlineStr"/>
+      <c r="J847" t="inlineStr"/>
+      <c r="K847" t="n">
+        <v>69</v>
+      </c>
+      <c r="L847" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>Advogados e Escritórios de Advocacia em Vitória</t>
+        </is>
+      </c>
+      <c r="G848" t="inlineStr">
+        <is>
+          <t>https://www.encontrabrasil.com.br</t>
+        </is>
+      </c>
+      <c r="H848" t="inlineStr"/>
+      <c r="I848" t="inlineStr"/>
+      <c r="J848" t="inlineStr"/>
+      <c r="K848" t="n">
+        <v>64</v>
+      </c>
+      <c r="L848" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>Hilton Rebello</t>
+        </is>
+      </c>
+      <c r="G849" t="inlineStr">
+        <is>
+          <t>https://www.hiltonrebello.com.br</t>
+        </is>
+      </c>
+      <c r="H849" t="inlineStr"/>
+      <c r="I849" t="inlineStr"/>
+      <c r="J849" t="inlineStr"/>
+      <c r="K849" t="n">
+        <v>45</v>
+      </c>
+      <c r="L849" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>Advogados e Escritórios de Advocacia em Vitória</t>
+        </is>
+      </c>
+      <c r="G850" t="inlineStr">
+        <is>
+          <t>https://www.encontravitoria.com.br</t>
+        </is>
+      </c>
+      <c r="H850" t="inlineStr"/>
+      <c r="I850" t="inlineStr"/>
+      <c r="J850" t="inlineStr"/>
+      <c r="K850" t="n">
+        <v>55</v>
+      </c>
+      <c r="L850" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F851" t="inlineStr">
+        <is>
+          <t>BKM Advogados</t>
+        </is>
+      </c>
+      <c r="G851" t="inlineStr">
+        <is>
+          <t>https://www.bkmadvogados.com.br</t>
+        </is>
+      </c>
+      <c r="H851" t="inlineStr"/>
+      <c r="I851" t="inlineStr"/>
+      <c r="J851" t="inlineStr"/>
+      <c r="K851" t="n">
+        <v>64</v>
+      </c>
+      <c r="L851" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr">
+        <is>
+          <t>Educação Física na Educação Infantil na rede pública de ensino da ...</t>
+        </is>
+      </c>
+      <c r="G852" t="inlineStr">
+        <is>
+          <t>http://educa.fcc.org.br</t>
+        </is>
+      </c>
+      <c r="H852" t="inlineStr"/>
+      <c r="I852" t="inlineStr"/>
+      <c r="J852" t="inlineStr"/>
+      <c r="K852" t="n">
+        <v>67</v>
+      </c>
+      <c r="L852" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr">
+        <is>
+          <t>Fisioterapia em Goiabeiras</t>
+        </is>
+      </c>
+      <c r="G853" t="inlineStr">
+        <is>
+          <t>https://www.guiagoiabeiras.com.br</t>
+        </is>
+      </c>
+      <c r="H853" t="inlineStr"/>
+      <c r="I853" t="inlineStr"/>
+      <c r="J853" t="inlineStr"/>
+      <c r="K853" t="n">
+        <v>0</v>
+      </c>
+      <c r="L853" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr">
+        <is>
+          <t>Os 10 melhores Dentistas em Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="G854" t="inlineStr">
+        <is>
+          <t>https://belo-horizonte.infoisinfo-br.com</t>
+        </is>
+      </c>
+      <c r="H854" t="inlineStr"/>
+      <c r="I854" t="inlineStr"/>
+      <c r="J854" t="inlineStr"/>
+      <c r="K854" t="n">
+        <v>64</v>
+      </c>
+      <c r="L854" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F855" t="inlineStr">
+        <is>
+          <t>Lorena Lustosa</t>
+        </is>
+      </c>
+      <c r="G855" t="inlineStr">
+        <is>
+          <t>https://www.lorenalustosa.com</t>
+        </is>
+      </c>
+      <c r="H855" t="inlineStr"/>
+      <c r="I855" t="inlineStr"/>
+      <c r="J855" t="inlineStr"/>
+      <c r="K855" t="n">
+        <v>67</v>
+      </c>
+      <c r="L855" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>Psicóloga Grasielle Silva</t>
+        </is>
+      </c>
+      <c r="G856" t="inlineStr">
+        <is>
+          <t>https://www.grasiellesilva.com.br</t>
+        </is>
+      </c>
+      <c r="H856" t="inlineStr"/>
+      <c r="I856" t="inlineStr"/>
+      <c r="J856" t="inlineStr"/>
+      <c r="K856" t="n">
+        <v>80</v>
+      </c>
+      <c r="L856" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>Advogado em Belo Horizonte/MG</t>
+        </is>
+      </c>
+      <c r="G857" t="inlineStr">
+        <is>
+          <t>https://eduardoleonadvocacia.com.br</t>
+        </is>
+      </c>
+      <c r="H857" t="inlineStr"/>
+      <c r="I857" t="inlineStr">
+        <is>
+          <t>5531983866120</t>
+        </is>
+      </c>
+      <c r="J857" t="inlineStr"/>
+      <c r="K857" t="n">
+        <v>73</v>
+      </c>
+      <c r="L857" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr">
+        <is>
+          <t>Hidroginástica em Belo Horizonte, Minas Gerais, MG</t>
+        </is>
+      </c>
+      <c r="G858" t="inlineStr">
+        <is>
+          <t>https://www.encontramg.com.br</t>
+        </is>
+      </c>
+      <c r="H858" t="inlineStr"/>
+      <c r="I858" t="inlineStr"/>
+      <c r="J858" t="inlineStr"/>
+      <c r="K858" t="n">
+        <v>64</v>
+      </c>
+      <c r="L858" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr">
+        <is>
+          <t>Horizonte Saúde &amp; Bem-estar</t>
+        </is>
+      </c>
+      <c r="G859" t="inlineStr">
+        <is>
+          <t>https://www.horizontefisioterapia.com.br</t>
+        </is>
+      </c>
+      <c r="H859" t="inlineStr"/>
+      <c r="I859" t="inlineStr"/>
+      <c r="J859" t="inlineStr"/>
+      <c r="K859" t="n">
+        <v>60</v>
+      </c>
+      <c r="L859" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr">
+        <is>
+          <t>Fisioterapia Domiciliar em Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="G860" t="inlineStr">
+        <is>
+          <t>https://ortopedia.clinicavicci.com.br</t>
+        </is>
+      </c>
+      <c r="H860" t="inlineStr"/>
+      <c r="I860" t="inlineStr"/>
+      <c r="J860" t="inlineStr"/>
+      <c r="K860" t="n">
+        <v>60</v>
+      </c>
+      <c r="L860" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr">
+        <is>
+          <t>Clínica Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="G861" t="inlineStr">
+        <is>
+          <t>https://www.clinicariodejaneiro.com.br</t>
+        </is>
+      </c>
+      <c r="H861" t="inlineStr"/>
+      <c r="I861" t="inlineStr">
+        <is>
+          <t>5521976830437</t>
+        </is>
+      </c>
+      <c r="J861" t="inlineStr"/>
+      <c r="K861" t="n">
+        <v>75</v>
+      </c>
+      <c r="L861" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F862" t="inlineStr">
+        <is>
+          <t>Clínica Médica em Rio de Janeiro RJ (2026)</t>
+        </is>
+      </c>
+      <c r="G862" t="inlineStr">
+        <is>
+          <t>https://guiariodejaneirorj.com.br</t>
+        </is>
+      </c>
+      <c r="H862" t="inlineStr"/>
+      <c r="I862" t="inlineStr"/>
+      <c r="J862" t="inlineStr"/>
+      <c r="K862" t="n">
+        <v>91</v>
+      </c>
+      <c r="L862" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr">
+        <is>
+          <t>Clínica Médica Rio de Janeiro, Avenida Getúlio de Moura, 1286 ...Clínica Rio de Janeiro: Marcação de Exames, Horário, En</t>
+        </is>
+      </c>
+      <c r="G863" t="inlineStr">
+        <is>
+          <t>https://www.findglocal.com</t>
+        </is>
+      </c>
+      <c r="H863" t="inlineStr"/>
+      <c r="I863" t="inlineStr"/>
+      <c r="J863" t="inlineStr"/>
+      <c r="K863" t="n">
+        <v>33</v>
+      </c>
+      <c r="L863" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F864" t="inlineStr">
+        <is>
+          <t>Clínica Rio de Janeiro: Marcação de Exames, Horário, Endereço ...</t>
+        </is>
+      </c>
+      <c r="G864" t="inlineStr">
+        <is>
+          <t>https://www.encontrariodejaneiro.com.br</t>
+        </is>
+      </c>
+      <c r="H864" t="inlineStr"/>
+      <c r="I864" t="inlineStr"/>
+      <c r="J864" t="inlineStr"/>
+      <c r="K864" t="n">
+        <v>55</v>
+      </c>
+      <c r="L864" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F865" t="inlineStr">
+        <is>
+          <t>Clínica Médica</t>
+        </is>
+      </c>
+      <c r="G865" t="inlineStr">
+        <is>
+          <t>https://alllab.com.br</t>
+        </is>
+      </c>
+      <c r="H865" t="inlineStr"/>
+      <c r="I865" t="inlineStr">
+        <is>
+          <t>5521998952903</t>
+        </is>
+      </c>
+      <c r="J865" t="inlineStr"/>
+      <c r="K865" t="n">
+        <v>71</v>
+      </c>
+      <c r="L865" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F866" t="inlineStr">
+        <is>
+          <t>Clínica Life 360</t>
+        </is>
+      </c>
+      <c r="G866" t="inlineStr">
+        <is>
+          <t>https://clinicalife360.com.br</t>
+        </is>
+      </c>
+      <c r="H866" t="inlineStr"/>
+      <c r="I866" t="inlineStr">
+        <is>
+          <t>5521999148969</t>
+        </is>
+      </c>
+      <c r="J866" t="inlineStr"/>
+      <c r="K866" t="n">
+        <v>73</v>
+      </c>
+      <c r="L866" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Norte — 19 novos)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L890"/>
+  <dimension ref="A1:L909"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42911,10 +42911,8 @@
         </is>
       </c>
       <c r="H872" t="inlineStr"/>
-      <c r="I872" t="inlineStr">
-        <is>
-          <t>5541999712276</t>
-        </is>
+      <c r="I872" t="n">
+        <v>5541999712276</v>
       </c>
       <c r="J872" t="inlineStr"/>
       <c r="K872" t="n">
@@ -43011,10 +43009,8 @@
         </is>
       </c>
       <c r="H874" t="inlineStr"/>
-      <c r="I874" t="inlineStr">
-        <is>
-          <t>5541998500156</t>
-        </is>
+      <c r="I874" t="n">
+        <v>5541998500156</v>
       </c>
       <c r="J874" t="inlineStr"/>
       <c r="K874" t="n">
@@ -43111,10 +43107,8 @@
         </is>
       </c>
       <c r="H876" t="inlineStr"/>
-      <c r="I876" t="inlineStr">
-        <is>
-          <t>5551998767319</t>
-        </is>
+      <c r="I876" t="n">
+        <v>5551998767319</v>
       </c>
       <c r="J876" t="inlineStr"/>
       <c r="K876" t="n">
@@ -43163,10 +43157,8 @@
         </is>
       </c>
       <c r="H877" t="inlineStr"/>
-      <c r="I877" t="inlineStr">
-        <is>
-          <t>5551993202379</t>
-        </is>
+      <c r="I877" t="n">
+        <v>5551993202379</v>
       </c>
       <c r="J877" t="inlineStr"/>
       <c r="K877" t="n">
@@ -43311,10 +43303,8 @@
         </is>
       </c>
       <c r="H880" t="inlineStr"/>
-      <c r="I880" t="inlineStr">
-        <is>
-          <t>555189142923</t>
-        </is>
+      <c r="I880" t="n">
+        <v>555189142923</v>
       </c>
       <c r="J880" t="inlineStr"/>
       <c r="K880" t="n">
@@ -43363,10 +43353,8 @@
         </is>
       </c>
       <c r="H881" t="inlineStr"/>
-      <c r="I881" t="inlineStr">
-        <is>
-          <t>5551984836836</t>
-        </is>
+      <c r="I881" t="n">
+        <v>5551984836836</v>
       </c>
       <c r="J881" t="inlineStr"/>
       <c r="K881" t="n">
@@ -43463,10 +43451,8 @@
         </is>
       </c>
       <c r="H883" t="inlineStr"/>
-      <c r="I883" t="inlineStr">
-        <is>
-          <t>5551998405015</t>
-        </is>
+      <c r="I883" t="n">
+        <v>5551998405015</v>
       </c>
       <c r="J883" t="inlineStr"/>
       <c r="K883" t="n">
@@ -43515,10 +43501,8 @@
         </is>
       </c>
       <c r="H884" t="inlineStr"/>
-      <c r="I884" t="inlineStr">
-        <is>
-          <t>5551997776618</t>
-        </is>
+      <c r="I884" t="n">
+        <v>5551997776618</v>
       </c>
       <c r="J884" t="inlineStr"/>
       <c r="K884" t="n">
@@ -43567,10 +43551,8 @@
         </is>
       </c>
       <c r="H885" t="inlineStr"/>
-      <c r="I885" t="inlineStr">
-        <is>
-          <t>555132270378</t>
-        </is>
+      <c r="I885" t="n">
+        <v>555132270378</v>
       </c>
       <c r="J885" t="inlineStr"/>
       <c r="K885" t="n">
@@ -43619,10 +43601,8 @@
         </is>
       </c>
       <c r="H886" t="inlineStr"/>
-      <c r="I886" t="inlineStr">
-        <is>
-          <t>5551996643344</t>
-        </is>
+      <c r="I886" t="n">
+        <v>5551996643344</v>
       </c>
       <c r="J886" t="inlineStr"/>
       <c r="K886" t="n">
@@ -43671,10 +43651,8 @@
         </is>
       </c>
       <c r="H887" t="inlineStr"/>
-      <c r="I887" t="inlineStr">
-        <is>
-          <t>5548999149672</t>
-        </is>
+      <c r="I887" t="n">
+        <v>5548999149672</v>
       </c>
       <c r="J887" t="inlineStr"/>
       <c r="K887" t="n">
@@ -43723,10 +43701,8 @@
         </is>
       </c>
       <c r="H888" t="inlineStr"/>
-      <c r="I888" t="inlineStr">
-        <is>
-          <t>554839524000</t>
-        </is>
+      <c r="I888" t="n">
+        <v>554839524000</v>
       </c>
       <c r="J888" t="inlineStr"/>
       <c r="K888" t="n">
@@ -43775,10 +43751,8 @@
         </is>
       </c>
       <c r="H889" t="inlineStr"/>
-      <c r="I889" t="inlineStr">
-        <is>
-          <t>554832233031</t>
-        </is>
+      <c r="I889" t="n">
+        <v>554832233031</v>
       </c>
       <c r="J889" t="inlineStr"/>
       <c r="K889" t="n">
@@ -43827,16 +43801,938 @@
         </is>
       </c>
       <c r="H890" t="inlineStr"/>
-      <c r="I890" t="inlineStr">
-        <is>
-          <t>5548998655296</t>
-        </is>
+      <c r="I890" t="n">
+        <v>5548998655296</v>
       </c>
       <c r="J890" t="inlineStr"/>
       <c r="K890" t="n">
         <v>67</v>
       </c>
       <c r="L890" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F891" t="inlineStr">
+        <is>
+          <t>Guia Médico de Prestadores de Saúde em Rio Branco</t>
+        </is>
+      </c>
+      <c r="G891" t="inlineStr">
+        <is>
+          <t>https://clinica101.com.br</t>
+        </is>
+      </c>
+      <c r="H891" t="inlineStr"/>
+      <c r="I891" t="inlineStr"/>
+      <c r="J891" t="inlineStr"/>
+      <c r="K891" t="n">
+        <v>81</v>
+      </c>
+      <c r="L891" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F892" t="inlineStr">
+        <is>
+          <t>Guia Médico Unimed Rio Branco 2025</t>
+        </is>
+      </c>
+      <c r="G892" t="inlineStr">
+        <is>
+          <t>https://pt.scribd.com</t>
+        </is>
+      </c>
+      <c r="H892" t="inlineStr"/>
+      <c r="I892" t="inlineStr"/>
+      <c r="J892" t="inlineStr"/>
+      <c r="K892" t="n">
+        <v>40</v>
+      </c>
+      <c r="L892" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F893" t="inlineStr">
+        <is>
+          <t>Psicólogo em Rio Branco</t>
+        </is>
+      </c>
+      <c r="G893" t="inlineStr">
+        <is>
+          <t>https://ciceraalvespsicologa.com</t>
+        </is>
+      </c>
+      <c r="H893" t="inlineStr"/>
+      <c r="I893" t="inlineStr">
+        <is>
+          <t>5574981542389</t>
+        </is>
+      </c>
+      <c r="J893" t="inlineStr"/>
+      <c r="K893" t="n">
+        <v>73</v>
+      </c>
+      <c r="L893" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>Vaga ago/26: Acompanhamento de audiência em Rio Branco (AC)...</t>
+        </is>
+      </c>
+      <c r="G894" t="inlineStr">
+        <is>
+          <t>https://radar.juriscorrespondente.com.br</t>
+        </is>
+      </c>
+      <c r="H894" t="inlineStr"/>
+      <c r="I894" t="inlineStr"/>
+      <c r="J894" t="inlineStr"/>
+      <c r="K894" t="n">
+        <v>45</v>
+      </c>
+      <c r="L894" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F895" t="inlineStr">
+        <is>
+          <t>Academias em Rio Branco, AC</t>
+        </is>
+      </c>
+      <c r="G895" t="inlineStr">
+        <is>
+          <t>https://www.guiamais.com.br</t>
+        </is>
+      </c>
+      <c r="H895" t="inlineStr"/>
+      <c r="I895" t="inlineStr"/>
+      <c r="J895" t="inlineStr"/>
+      <c r="K895" t="n">
+        <v>100</v>
+      </c>
+      <c r="L895" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>Fisioterapia em Rio Branco</t>
+        </is>
+      </c>
+      <c r="G896" t="inlineStr">
+        <is>
+          <t>https://fisio.net.br</t>
+        </is>
+      </c>
+      <c r="H896" t="inlineStr"/>
+      <c r="I896" t="inlineStr"/>
+      <c r="J896" t="inlineStr"/>
+      <c r="K896" t="n">
+        <v>88</v>
+      </c>
+      <c r="L896" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F897" t="inlineStr">
+        <is>
+          <t>Buscar: em macapa ap guiareunimedicos.med.br - Catálogo Médico</t>
+        </is>
+      </c>
+      <c r="G897" t="inlineStr">
+        <is>
+          <t>https://www.guiareunimedicos.med.br</t>
+        </is>
+      </c>
+      <c r="H897" t="inlineStr"/>
+      <c r="I897" t="inlineStr"/>
+      <c r="J897" t="inlineStr"/>
+      <c r="K897" t="n">
+        <v>62</v>
+      </c>
+      <c r="L897" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>Dentista em Macapá</t>
+        </is>
+      </c>
+      <c r="G898" t="inlineStr">
+        <is>
+          <t>https://clinicaperfetha.com.br</t>
+        </is>
+      </c>
+      <c r="H898" t="inlineStr"/>
+      <c r="I898" t="inlineStr"/>
+      <c r="J898" t="inlineStr"/>
+      <c r="K898" t="n">
+        <v>0</v>
+      </c>
+      <c r="L898" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>Dentistas em Macapá 【262 empresas】</t>
+        </is>
+      </c>
+      <c r="G899" t="inlineStr">
+        <is>
+          <t>https://dentistaspertodemim.com</t>
+        </is>
+      </c>
+      <c r="H899" t="inlineStr"/>
+      <c r="I899" t="inlineStr"/>
+      <c r="J899" t="inlineStr"/>
+      <c r="K899" t="n">
+        <v>87</v>
+      </c>
+      <c r="L899" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F900" t="inlineStr">
+        <is>
+          <t>Mayk Camelo Advogados</t>
+        </is>
+      </c>
+      <c r="G900" t="inlineStr">
+        <is>
+          <t>https://maykcameloadvogados.com.br</t>
+        </is>
+      </c>
+      <c r="H900" t="inlineStr"/>
+      <c r="I900" t="inlineStr">
+        <is>
+          <t>559681072847</t>
+        </is>
+      </c>
+      <c r="J900" t="inlineStr"/>
+      <c r="K900" t="n">
+        <v>73</v>
+      </c>
+      <c r="L900" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr">
+        <is>
+          <t>Conselho Seccional</t>
+        </is>
+      </c>
+      <c r="G901" t="inlineStr">
+        <is>
+          <t>https://deoab.oab.org.br</t>
+        </is>
+      </c>
+      <c r="H901" t="inlineStr"/>
+      <c r="I901" t="inlineStr"/>
+      <c r="J901" t="inlineStr"/>
+      <c r="K901" t="n">
+        <v>45</v>
+      </c>
+      <c r="L901" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F902" t="inlineStr">
+        <is>
+          <t>Academias em Macapá, AP</t>
+        </is>
+      </c>
+      <c r="G902" t="inlineStr">
+        <is>
+          <t>https://www.solutudo.com.br</t>
+        </is>
+      </c>
+      <c r="H902" t="inlineStr"/>
+      <c r="I902" t="inlineStr"/>
+      <c r="J902" t="inlineStr"/>
+      <c r="K902" t="n">
+        <v>33</v>
+      </c>
+      <c r="L902" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F903" t="inlineStr">
+        <is>
+          <t>CMM- Clínica Médica Manaus</t>
+        </is>
+      </c>
+      <c r="G903" t="inlineStr">
+        <is>
+          <t>https://cmm-clinica-medica.localo.site</t>
+        </is>
+      </c>
+      <c r="H903" t="inlineStr"/>
+      <c r="I903" t="inlineStr"/>
+      <c r="J903" t="inlineStr"/>
+      <c r="K903" t="n">
+        <v>80</v>
+      </c>
+      <c r="L903" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F904" t="inlineStr">
+        <is>
+          <t>Dentista em Manaus - AM</t>
+        </is>
+      </c>
+      <c r="G904" t="inlineStr">
+        <is>
+          <t>https://rankodonto.com.br</t>
+        </is>
+      </c>
+      <c r="H904" t="inlineStr"/>
+      <c r="I904" t="inlineStr"/>
+      <c r="J904" t="inlineStr"/>
+      <c r="K904" t="n">
+        <v>60</v>
+      </c>
+      <c r="L904" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E905" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>Dentista em Manaus, AM</t>
+        </is>
+      </c>
+      <c r="G905" t="inlineStr">
+        <is>
+          <t>https://guiapinzon.com.br</t>
+        </is>
+      </c>
+      <c r="H905" t="inlineStr"/>
+      <c r="I905" t="inlineStr"/>
+      <c r="J905" t="inlineStr"/>
+      <c r="K905" t="n">
+        <v>56</v>
+      </c>
+      <c r="L905" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F906" t="inlineStr">
+        <is>
+          <t>Psicólogo em Manaus</t>
+        </is>
+      </c>
+      <c r="G906" t="inlineStr">
+        <is>
+          <t>https://www.clinicadosentido.com</t>
+        </is>
+      </c>
+      <c r="H906" t="inlineStr"/>
+      <c r="I906" t="inlineStr"/>
+      <c r="J906" t="inlineStr"/>
+      <c r="K906" t="n">
+        <v>80</v>
+      </c>
+      <c r="L906" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>TERAPEUTA JANYMASSAG Formada em terapia tantrica...</t>
+        </is>
+      </c>
+      <c r="G907" t="inlineStr">
+        <is>
+          <t>https://br.skokka.com</t>
+        </is>
+      </c>
+      <c r="H907" t="inlineStr"/>
+      <c r="I907" t="inlineStr"/>
+      <c r="J907" t="inlineStr"/>
+      <c r="K907" t="n">
+        <v>33</v>
+      </c>
+      <c r="L907" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F908" t="inlineStr">
+        <is>
+          <t>Manaus/AM abre concurso para Professor de Educação Física</t>
+        </is>
+      </c>
+      <c r="G908" t="inlineStr">
+        <is>
+          <t>https://concursosedfisica.com</t>
+        </is>
+      </c>
+      <c r="H908" t="inlineStr"/>
+      <c r="I908" t="inlineStr">
+        <is>
+          <t>5585999458789</t>
+        </is>
+      </c>
+      <c r="J908" t="inlineStr"/>
+      <c r="K908" t="n">
+        <v>56</v>
+      </c>
+      <c r="L908" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E909" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F909" t="inlineStr">
+        <is>
+          <t>Formação continuada de professores de Educação Física em...</t>
+        </is>
+      </c>
+      <c r="G909" t="inlineStr">
+        <is>
+          <t>https://periodicos.sbu.unicamp.br</t>
+        </is>
+      </c>
+      <c r="H909" t="inlineStr"/>
+      <c r="I909" t="inlineStr"/>
+      <c r="J909" t="inlineStr"/>
+      <c r="K909" t="n">
+        <v>73</v>
+      </c>
+      <c r="L909" t="inlineStr">
         <is>
           <t>Crítico</t>
         </is>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Nordeste, 2026-08-13)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L909"/>
+  <dimension ref="A1:L922"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43947,10 +43947,8 @@
         </is>
       </c>
       <c r="H893" t="inlineStr"/>
-      <c r="I893" t="inlineStr">
-        <is>
-          <t>5574981542389</t>
-        </is>
+      <c r="I893" t="n">
+        <v>5574981542389</v>
       </c>
       <c r="J893" t="inlineStr"/>
       <c r="K893" t="n">
@@ -44287,10 +44285,8 @@
         </is>
       </c>
       <c r="H900" t="inlineStr"/>
-      <c r="I900" t="inlineStr">
-        <is>
-          <t>559681072847</t>
-        </is>
+      <c r="I900" t="n">
+        <v>559681072847</v>
       </c>
       <c r="J900" t="inlineStr"/>
       <c r="K900" t="n">
@@ -44675,10 +44671,8 @@
         </is>
       </c>
       <c r="H908" t="inlineStr"/>
-      <c r="I908" t="inlineStr">
-        <is>
-          <t>5585999458789</t>
-        </is>
+      <c r="I908" t="n">
+        <v>5585999458789</v>
       </c>
       <c r="J908" t="inlineStr"/>
       <c r="K908" t="n">
@@ -44738,6 +44732,650 @@
         </is>
       </c>
     </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E910" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F910" t="inlineStr">
+        <is>
+          <t>Agenda do Terapeuta Eliete Oliveira</t>
+        </is>
+      </c>
+      <c r="G910" t="inlineStr">
+        <is>
+          <t>https://unimasso.com.br</t>
+        </is>
+      </c>
+      <c r="H910" t="inlineStr"/>
+      <c r="I910" t="inlineStr"/>
+      <c r="J910" t="inlineStr"/>
+      <c r="K910" t="n">
+        <v>33</v>
+      </c>
+      <c r="L910" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E911" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F911" t="inlineStr">
+        <is>
+          <t>Guia Completo de Clínicas médicas em Salvador</t>
+        </is>
+      </c>
+      <c r="G911" t="inlineStr">
+        <is>
+          <t>https://alisaude.com.br</t>
+        </is>
+      </c>
+      <c r="H911" t="inlineStr"/>
+      <c r="I911" t="inlineStr"/>
+      <c r="J911" t="inlineStr"/>
+      <c r="K911" t="n">
+        <v>76</v>
+      </c>
+      <c r="L911" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E912" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F912" t="inlineStr">
+        <is>
+          <t>Clínica</t>
+        </is>
+      </c>
+      <c r="G912" t="inlineStr">
+        <is>
+          <t>https://www.clinicavistar.com</t>
+        </is>
+      </c>
+      <c r="H912" t="inlineStr"/>
+      <c r="I912" t="inlineStr">
+        <is>
+          <t>5571982373780</t>
+        </is>
+      </c>
+      <c r="J912" t="inlineStr"/>
+      <c r="K912" t="n">
+        <v>70</v>
+      </c>
+      <c r="L912" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E913" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F913" t="inlineStr">
+        <is>
+          <t>Clinicas em Salvador</t>
+        </is>
+      </c>
+      <c r="G913" t="inlineStr">
+        <is>
+          <t>https://www.centromedicobelavista.com.br</t>
+        </is>
+      </c>
+      <c r="H913" t="inlineStr"/>
+      <c r="I913" t="inlineStr"/>
+      <c r="J913" t="inlineStr"/>
+      <c r="K913" t="n">
+        <v>70</v>
+      </c>
+      <c r="L913" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E914" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F914" t="inlineStr">
+        <is>
+          <t>Seta Clínica Médica</t>
+        </is>
+      </c>
+      <c r="G914" t="inlineStr">
+        <is>
+          <t>https://clinicasetabahia.com.br</t>
+        </is>
+      </c>
+      <c r="H914" t="inlineStr"/>
+      <c r="I914" t="inlineStr"/>
+      <c r="J914" t="inlineStr"/>
+      <c r="K914" t="n">
+        <v>73</v>
+      </c>
+      <c r="L914" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E915" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F915" t="inlineStr">
+        <is>
+          <t>Hospitais e Clínicas : Salvador, Bahia</t>
+        </is>
+      </c>
+      <c r="G915" t="inlineStr">
+        <is>
+          <t>https://salvador-ba.brasil-infos.com</t>
+        </is>
+      </c>
+      <c r="H915" t="inlineStr"/>
+      <c r="I915" t="inlineStr"/>
+      <c r="J915" t="inlineStr"/>
+      <c r="K915" t="n">
+        <v>81</v>
+      </c>
+      <c r="L915" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E916" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F916" t="inlineStr">
+        <is>
+          <t>Clínica Angiclin</t>
+        </is>
+      </c>
+      <c r="G916" t="inlineStr">
+        <is>
+          <t>https://angiclin.com.br</t>
+        </is>
+      </c>
+      <c r="H916" t="inlineStr"/>
+      <c r="I916" t="inlineStr">
+        <is>
+          <t>5571999241313</t>
+        </is>
+      </c>
+      <c r="J916" t="inlineStr"/>
+      <c r="K916" t="n">
+        <v>73</v>
+      </c>
+      <c r="L916" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E917" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F917" t="inlineStr">
+        <is>
+          <t>Leonardo Saldanha</t>
+        </is>
+      </c>
+      <c r="G917" t="inlineStr">
+        <is>
+          <t>https://leonardosaldanha.com.br</t>
+        </is>
+      </c>
+      <c r="H917" t="inlineStr"/>
+      <c r="I917" t="inlineStr">
+        <is>
+          <t>5571996902910</t>
+        </is>
+      </c>
+      <c r="J917" t="inlineStr"/>
+      <c r="K917" t="n">
+        <v>73</v>
+      </c>
+      <c r="L917" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E918" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F918" t="inlineStr">
+        <is>
+          <t>Guia de Massoterapeuta Massagista e Massagens</t>
+        </is>
+      </c>
+      <c r="G918" t="inlineStr">
+        <is>
+          <t>https://relaxzen.com.br</t>
+        </is>
+      </c>
+      <c r="H918" t="inlineStr"/>
+      <c r="I918" t="inlineStr">
+        <is>
+          <t>5571981547350</t>
+        </is>
+      </c>
+      <c r="J918" t="inlineStr"/>
+      <c r="K918" t="n">
+        <v>81</v>
+      </c>
+      <c r="L918" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D919" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E919" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F919" t="inlineStr">
+        <is>
+          <t>Advogado Salvador Bahia Advogado Especialista em Acidente de...</t>
+        </is>
+      </c>
+      <c r="G919" t="inlineStr">
+        <is>
+          <t>https://www.onaldo.com.br</t>
+        </is>
+      </c>
+      <c r="H919" t="inlineStr"/>
+      <c r="I919" t="inlineStr"/>
+      <c r="J919" t="inlineStr"/>
+      <c r="K919" t="n">
+        <v>55</v>
+      </c>
+      <c r="L919" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E920" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F920" t="inlineStr">
+        <is>
+          <t>Academias em 3849, BA Em atividade há 23 anos.</t>
+        </is>
+      </c>
+      <c r="G920" t="inlineStr">
+        <is>
+          <t>https://anunce.com</t>
+        </is>
+      </c>
+      <c r="H920" t="inlineStr"/>
+      <c r="I920" t="inlineStr"/>
+      <c r="J920" t="inlineStr"/>
+      <c r="K920" t="n">
+        <v>33</v>
+      </c>
+      <c r="L920" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E921" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F921" t="inlineStr">
+        <is>
+          <t>Première Medicina e Saúde Fortaleza |</t>
+        </is>
+      </c>
+      <c r="G921" t="inlineStr">
+        <is>
+          <t>https://premieremedicina.com.br</t>
+        </is>
+      </c>
+      <c r="H921" t="inlineStr"/>
+      <c r="I921" t="inlineStr">
+        <is>
+          <t>558537713180</t>
+        </is>
+      </c>
+      <c r="J921" t="inlineStr"/>
+      <c r="K921" t="n">
+        <v>76</v>
+      </c>
+      <c r="L921" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E922" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F922" t="inlineStr">
+        <is>
+          <t>Dentista 24 Horas em Fortaleza</t>
+        </is>
+      </c>
+      <c r="G922" t="inlineStr">
+        <is>
+          <t>https://dentistafortaleza.net</t>
+        </is>
+      </c>
+      <c r="H922" t="inlineStr"/>
+      <c r="I922" t="inlineStr"/>
+      <c r="J922" t="inlineStr"/>
+      <c r="K922" t="n">
+        <v>60</v>
+      </c>
+      <c r="L922" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Norte, +15 novos)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L955"/>
+  <dimension ref="A1:L970"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46527,10 +46527,8 @@
         </is>
       </c>
       <c r="H946" t="inlineStr"/>
-      <c r="I946" t="inlineStr">
-        <is>
-          <t>5547992745563</t>
-        </is>
+      <c r="I946" t="n">
+        <v>5547992745563</v>
       </c>
       <c r="J946" t="inlineStr"/>
       <c r="K946" t="n">
@@ -46627,10 +46625,8 @@
         </is>
       </c>
       <c r="H948" t="inlineStr"/>
-      <c r="I948" t="inlineStr">
-        <is>
-          <t>555130131110</t>
-        </is>
+      <c r="I948" t="n">
+        <v>555130131110</v>
       </c>
       <c r="J948" t="inlineStr"/>
       <c r="K948" t="n">
@@ -46679,10 +46675,8 @@
         </is>
       </c>
       <c r="H949" t="inlineStr"/>
-      <c r="I949" t="inlineStr">
-        <is>
-          <t>5551998081317</t>
-        </is>
+      <c r="I949" t="n">
+        <v>5551998081317</v>
       </c>
       <c r="J949" t="inlineStr"/>
       <c r="K949" t="n">
@@ -46875,10 +46869,8 @@
         </is>
       </c>
       <c r="H953" t="inlineStr"/>
-      <c r="I953" t="inlineStr">
-        <is>
-          <t>5551982690040</t>
-        </is>
+      <c r="I953" t="n">
+        <v>5551982690040</v>
       </c>
       <c r="J953" t="inlineStr"/>
       <c r="K953" t="n">
@@ -46975,10 +46967,8 @@
         </is>
       </c>
       <c r="H955" t="inlineStr"/>
-      <c r="I955" t="inlineStr">
-        <is>
-          <t>5551994024624</t>
-        </is>
+      <c r="I955" t="n">
+        <v>5551994024624</v>
       </c>
       <c r="J955" t="inlineStr"/>
       <c r="K955" t="n">
@@ -46987,6 +46977,754 @@
       <c r="L955" t="inlineStr">
         <is>
           <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D956" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E956" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F956" t="inlineStr">
+        <is>
+          <t>Os 5 melhores Psicólogos em Rio Branco</t>
+        </is>
+      </c>
+      <c r="G956" t="inlineStr">
+        <is>
+          <t>https://rio-branco.infoisinfo-br.com</t>
+        </is>
+      </c>
+      <c r="H956" t="inlineStr"/>
+      <c r="I956" t="inlineStr"/>
+      <c r="J956" t="inlineStr"/>
+      <c r="K956" t="n">
+        <v>64</v>
+      </c>
+      <c r="L956" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D957" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E957" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F957" t="inlineStr">
+        <is>
+          <t>Maris</t>
+        </is>
+      </c>
+      <c r="G957" t="inlineStr">
+        <is>
+          <t>https://www.marispsicologia.com</t>
+        </is>
+      </c>
+      <c r="H957" t="inlineStr"/>
+      <c r="I957" t="inlineStr"/>
+      <c r="J957" t="inlineStr"/>
+      <c r="K957" t="n">
+        <v>80</v>
+      </c>
+      <c r="L957" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E958" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F958" t="inlineStr">
+        <is>
+          <t>Educação Física</t>
+        </is>
+      </c>
+      <c r="G958" t="inlineStr">
+        <is>
+          <t>https://itamazonia.com.br</t>
+        </is>
+      </c>
+      <c r="H958" t="inlineStr"/>
+      <c r="I958" t="inlineStr">
+        <is>
+          <t>5568999787806</t>
+        </is>
+      </c>
+      <c r="J958" t="inlineStr"/>
+      <c r="K958" t="n">
+        <v>88</v>
+      </c>
+      <c r="L958" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E959" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F959" t="inlineStr">
+        <is>
+          <t>TABELA DE CONVÊNIOS ACADEMIA DESCONTO POWER ...</t>
+        </is>
+      </c>
+      <c r="G959" t="inlineStr">
+        <is>
+          <t>https://www.oabac.org.br</t>
+        </is>
+      </c>
+      <c r="H959" t="inlineStr"/>
+      <c r="I959" t="inlineStr"/>
+      <c r="J959" t="inlineStr"/>
+      <c r="K959" t="n">
+        <v>22</v>
+      </c>
+      <c r="L959" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>Rio Branco</t>
+        </is>
+      </c>
+      <c r="E960" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F960" t="inlineStr">
+        <is>
+          <t>ABL celebra os 80 anos do Instituto Rio Branco</t>
+        </is>
+      </c>
+      <c r="G960" t="inlineStr">
+        <is>
+          <t>https://www.academia.org.br</t>
+        </is>
+      </c>
+      <c r="H960" t="inlineStr"/>
+      <c r="I960" t="inlineStr"/>
+      <c r="J960" t="inlineStr"/>
+      <c r="K960" t="n">
+        <v>80</v>
+      </c>
+      <c r="L960" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D961" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E961" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F961" t="inlineStr">
+        <is>
+          <t>Centerclin Odontologia</t>
+        </is>
+      </c>
+      <c r="G961" t="inlineStr">
+        <is>
+          <t>https://www.centerclinsaude.com.br</t>
+        </is>
+      </c>
+      <c r="H961" t="inlineStr"/>
+      <c r="I961" t="inlineStr">
+        <is>
+          <t>5596999050219</t>
+        </is>
+      </c>
+      <c r="J961" t="inlineStr"/>
+      <c r="K961" t="n">
+        <v>53</v>
+      </c>
+      <c r="L961" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="D962" t="inlineStr">
+        <is>
+          <t>Macapá</t>
+        </is>
+      </c>
+      <c r="E962" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F962" t="inlineStr">
+        <is>
+          <t>Fisioterapia em Macapá</t>
+        </is>
+      </c>
+      <c r="G962" t="inlineStr">
+        <is>
+          <t>https://www.encontramacapa.com.br</t>
+        </is>
+      </c>
+      <c r="H962" t="inlineStr"/>
+      <c r="I962" t="inlineStr"/>
+      <c r="J962" t="inlineStr"/>
+      <c r="K962" t="n">
+        <v>64</v>
+      </c>
+      <c r="L962" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D963" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E963" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F963" t="inlineStr">
+        <is>
+          <t>Psicólogo em Manaus</t>
+        </is>
+      </c>
+      <c r="G963" t="inlineStr">
+        <is>
+          <t>https://www.clinicadosentido.com.br</t>
+        </is>
+      </c>
+      <c r="H963" t="inlineStr"/>
+      <c r="I963" t="inlineStr"/>
+      <c r="J963" t="inlineStr"/>
+      <c r="K963" t="n">
+        <v>80</v>
+      </c>
+      <c r="L963" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E964" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F964" t="inlineStr">
+        <is>
+          <t>Psicologia</t>
+        </is>
+      </c>
+      <c r="G964" t="inlineStr">
+        <is>
+          <t>https://www.psicologia.espmais.com.br</t>
+        </is>
+      </c>
+      <c r="H964" t="inlineStr"/>
+      <c r="I964" t="inlineStr">
+        <is>
+          <t>5592992249046</t>
+        </is>
+      </c>
+      <c r="J964" t="inlineStr"/>
+      <c r="K964" t="n">
+        <v>80</v>
+      </c>
+      <c r="L964" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E965" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F965" t="inlineStr">
+        <is>
+          <t>Terapeuta Em Manaus</t>
+        </is>
+      </c>
+      <c r="G965" t="inlineStr">
+        <is>
+          <t>https://marciadamasceno.com</t>
+        </is>
+      </c>
+      <c r="H965" t="inlineStr"/>
+      <c r="I965" t="inlineStr">
+        <is>
+          <t>559299767074</t>
+        </is>
+      </c>
+      <c r="J965" t="inlineStr"/>
+      <c r="K965" t="n">
+        <v>89</v>
+      </c>
+      <c r="L965" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D966" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E966" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F966" t="inlineStr">
+        <is>
+          <t>Advogados Manaus</t>
+        </is>
+      </c>
+      <c r="G966" t="inlineStr">
+        <is>
+          <t>https://www.manausadvogados.com.br</t>
+        </is>
+      </c>
+      <c r="H966" t="inlineStr"/>
+      <c r="I966" t="inlineStr">
+        <is>
+          <t>5592981818182</t>
+        </is>
+      </c>
+      <c r="J966" t="inlineStr"/>
+      <c r="K966" t="n">
+        <v>45</v>
+      </c>
+      <c r="L966" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D967" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E967" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F967" t="inlineStr">
+        <is>
+          <t>Advogados em Manaus</t>
+        </is>
+      </c>
+      <c r="G967" t="inlineStr">
+        <is>
+          <t>https://fariasribeiroadvogados.com.br</t>
+        </is>
+      </c>
+      <c r="H967" t="inlineStr"/>
+      <c r="I967" t="inlineStr">
+        <is>
+          <t>5592995026464</t>
+        </is>
+      </c>
+      <c r="J967" t="inlineStr"/>
+      <c r="K967" t="n">
+        <v>64</v>
+      </c>
+      <c r="L967" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D968" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E968" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F968" t="inlineStr">
+        <is>
+          <t>Os Melhores Advogados de Manaus</t>
+        </is>
+      </c>
+      <c r="G968" t="inlineStr">
+        <is>
+          <t>https://advocaciasmanaus.com</t>
+        </is>
+      </c>
+      <c r="H968" t="inlineStr"/>
+      <c r="I968" t="inlineStr">
+        <is>
+          <t>5592991479179</t>
+        </is>
+      </c>
+      <c r="J968" t="inlineStr"/>
+      <c r="K968" t="n">
+        <v>55</v>
+      </c>
+      <c r="L968" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D969" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E969" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F969" t="inlineStr">
+        <is>
+          <t>Advogados e Escritórios de Advocacia em Manaus</t>
+        </is>
+      </c>
+      <c r="G969" t="inlineStr">
+        <is>
+          <t>https://www.encontramanausam.com.br</t>
+        </is>
+      </c>
+      <c r="H969" t="inlineStr"/>
+      <c r="I969" t="inlineStr"/>
+      <c r="J969" t="inlineStr"/>
+      <c r="K969" t="n">
+        <v>55</v>
+      </c>
+      <c r="L969" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D970" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="E970" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F970" t="inlineStr">
+        <is>
+          <t>Advogados Manaus</t>
+        </is>
+      </c>
+      <c r="G970" t="inlineStr">
+        <is>
+          <t>https://lehmann.adv.br</t>
+        </is>
+      </c>
+      <c r="H970" t="inlineStr"/>
+      <c r="I970" t="inlineStr"/>
+      <c r="J970" t="inlineStr"/>
+      <c r="K970" t="n">
+        <v>91</v>
+      </c>
+      <c r="L970" t="inlineStr">
+        <is>
+          <t>Baixo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Nordeste, 2026-08-25)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L970"/>
+  <dimension ref="A1:L981"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47113,10 +47113,8 @@
         </is>
       </c>
       <c r="H958" t="inlineStr"/>
-      <c r="I958" t="inlineStr">
-        <is>
-          <t>5568999787806</t>
-        </is>
+      <c r="I958" t="n">
+        <v>5568999787806</v>
       </c>
       <c r="J958" t="inlineStr"/>
       <c r="K958" t="n">
@@ -47261,10 +47259,8 @@
         </is>
       </c>
       <c r="H961" t="inlineStr"/>
-      <c r="I961" t="inlineStr">
-        <is>
-          <t>5596999050219</t>
-        </is>
+      <c r="I961" t="n">
+        <v>5596999050219</v>
       </c>
       <c r="J961" t="inlineStr"/>
       <c r="K961" t="n">
@@ -47409,10 +47405,8 @@
         </is>
       </c>
       <c r="H964" t="inlineStr"/>
-      <c r="I964" t="inlineStr">
-        <is>
-          <t>5592992249046</t>
-        </is>
+      <c r="I964" t="n">
+        <v>5592992249046</v>
       </c>
       <c r="J964" t="inlineStr"/>
       <c r="K964" t="n">
@@ -47461,10 +47455,8 @@
         </is>
       </c>
       <c r="H965" t="inlineStr"/>
-      <c r="I965" t="inlineStr">
-        <is>
-          <t>559299767074</t>
-        </is>
+      <c r="I965" t="n">
+        <v>559299767074</v>
       </c>
       <c r="J965" t="inlineStr"/>
       <c r="K965" t="n">
@@ -47513,10 +47505,8 @@
         </is>
       </c>
       <c r="H966" t="inlineStr"/>
-      <c r="I966" t="inlineStr">
-        <is>
-          <t>5592981818182</t>
-        </is>
+      <c r="I966" t="n">
+        <v>5592981818182</v>
       </c>
       <c r="J966" t="inlineStr"/>
       <c r="K966" t="n">
@@ -47565,10 +47555,8 @@
         </is>
       </c>
       <c r="H967" t="inlineStr"/>
-      <c r="I967" t="inlineStr">
-        <is>
-          <t>5592995026464</t>
-        </is>
+      <c r="I967" t="n">
+        <v>5592995026464</v>
       </c>
       <c r="J967" t="inlineStr"/>
       <c r="K967" t="n">
@@ -47617,10 +47605,8 @@
         </is>
       </c>
       <c r="H968" t="inlineStr"/>
-      <c r="I968" t="inlineStr">
-        <is>
-          <t>5592991479179</t>
-        </is>
+      <c r="I968" t="n">
+        <v>5592991479179</v>
       </c>
       <c r="J968" t="inlineStr"/>
       <c r="K968" t="n">
@@ -47728,6 +47714,538 @@
         </is>
       </c>
     </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D971" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E971" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F971" t="inlineStr">
+        <is>
+          <t>Maceió Saúde</t>
+        </is>
+      </c>
+      <c r="G971" t="inlineStr">
+        <is>
+          <t>https://maceiosaude.com</t>
+        </is>
+      </c>
+      <c r="H971" t="inlineStr"/>
+      <c r="I971" t="inlineStr"/>
+      <c r="J971" t="inlineStr"/>
+      <c r="K971" t="n">
+        <v>69</v>
+      </c>
+      <c r="L971" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D972" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E972" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F972" t="inlineStr">
+        <is>
+          <t>Clínica Médica em Salvador</t>
+        </is>
+      </c>
+      <c r="G972" t="inlineStr">
+        <is>
+          <t>https://clivalemais.com.br</t>
+        </is>
+      </c>
+      <c r="H972" t="inlineStr"/>
+      <c r="I972" t="inlineStr">
+        <is>
+          <t>557121027777</t>
+        </is>
+      </c>
+      <c r="J972" t="inlineStr"/>
+      <c r="K972" t="n">
+        <v>69</v>
+      </c>
+      <c r="L972" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D973" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E973" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F973" t="inlineStr">
+        <is>
+          <t>CMA Clínica e Day Hospital</t>
+        </is>
+      </c>
+      <c r="G973" t="inlineStr">
+        <is>
+          <t>https://clinicamedicacma.com.br</t>
+        </is>
+      </c>
+      <c r="H973" t="inlineStr"/>
+      <c r="I973" t="inlineStr"/>
+      <c r="J973" t="inlineStr"/>
+      <c r="K973" t="n">
+        <v>56</v>
+      </c>
+      <c r="L973" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D974" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E974" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F974" t="inlineStr">
+        <is>
+          <t>Lista de Médicos e Clínicas em Salvador - BA</t>
+        </is>
+      </c>
+      <c r="G974" t="inlineStr">
+        <is>
+          <t>https://inteligue.com.br</t>
+        </is>
+      </c>
+      <c r="H974" t="inlineStr"/>
+      <c r="I974" t="inlineStr"/>
+      <c r="J974" t="inlineStr"/>
+      <c r="K974" t="n">
+        <v>33</v>
+      </c>
+      <c r="L974" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D975" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E975" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F975" t="inlineStr">
+        <is>
+          <t>Dra Ana Carolina Odontologia, Dentista em Salvador, BA</t>
+        </is>
+      </c>
+      <c r="G975" t="inlineStr">
+        <is>
+          <t>https://dentistasalvadorbahia.com.br</t>
+        </is>
+      </c>
+      <c r="H975" t="inlineStr"/>
+      <c r="I975" t="inlineStr"/>
+      <c r="J975" t="inlineStr"/>
+      <c r="K975" t="n">
+        <v>67</v>
+      </c>
+      <c r="L975" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D976" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E976" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F976" t="inlineStr">
+        <is>
+          <t>OAB : Ordem dos Advogados do Brasil</t>
+        </is>
+      </c>
+      <c r="G976" t="inlineStr">
+        <is>
+          <t>https://www.oab-ba.org.br</t>
+        </is>
+      </c>
+      <c r="H976" t="inlineStr"/>
+      <c r="I976" t="inlineStr"/>
+      <c r="J976" t="inlineStr"/>
+      <c r="K976" t="n">
+        <v>73</v>
+      </c>
+      <c r="L976" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D977" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E977" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F977" t="inlineStr">
+        <is>
+          <t>CEFE</t>
+        </is>
+      </c>
+      <c r="G977" t="inlineStr">
+        <is>
+          <t>http://www.cefe.ufba.br</t>
+        </is>
+      </c>
+      <c r="H977" t="inlineStr"/>
+      <c r="I977" t="inlineStr"/>
+      <c r="J977" t="inlineStr"/>
+      <c r="K977" t="n">
+        <v>33</v>
+      </c>
+      <c r="L977" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D978" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E978" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F978" t="inlineStr">
+        <is>
+          <t>EDUCAÇÃO FÍSICA</t>
+        </is>
+      </c>
+      <c r="G978" t="inlineStr">
+        <is>
+          <t>https://inscricao.ucsal.br</t>
+        </is>
+      </c>
+      <c r="H978" t="inlineStr"/>
+      <c r="I978" t="inlineStr"/>
+      <c r="J978" t="inlineStr"/>
+      <c r="K978" t="n">
+        <v>33</v>
+      </c>
+      <c r="L978" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D979" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E979" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F979" t="inlineStr">
+        <is>
+          <t>Educação Física</t>
+        </is>
+      </c>
+      <c r="G979" t="inlineStr">
+        <is>
+          <t>https://faced.ufba.br</t>
+        </is>
+      </c>
+      <c r="H979" t="inlineStr"/>
+      <c r="I979" t="inlineStr"/>
+      <c r="J979" t="inlineStr"/>
+      <c r="K979" t="n">
+        <v>69</v>
+      </c>
+      <c r="L979" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D980" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E980" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F980" t="inlineStr">
+        <is>
+          <t>Academia Salvador</t>
+        </is>
+      </c>
+      <c r="G980" t="inlineStr">
+        <is>
+          <t>https://www.salvadordabahia.com</t>
+        </is>
+      </c>
+      <c r="H980" t="inlineStr"/>
+      <c r="I980" t="inlineStr"/>
+      <c r="J980" t="inlineStr"/>
+      <c r="K980" t="n">
+        <v>100</v>
+      </c>
+      <c r="L980" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D981" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E981" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F981" t="inlineStr">
+        <is>
+          <t>Prime Academia</t>
+        </is>
+      </c>
+      <c r="G981" t="inlineStr">
+        <is>
+          <t>https://www.wellprime.com.br</t>
+        </is>
+      </c>
+      <c r="H981" t="inlineStr"/>
+      <c r="I981" t="inlineStr"/>
+      <c r="J981" t="inlineStr"/>
+      <c r="K981" t="n">
+        <v>70</v>
+      </c>
+      <c r="L981" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Sudeste, +20 novos)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L998"/>
+  <dimension ref="A1:L1018"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48281,10 +48281,8 @@
         </is>
       </c>
       <c r="H982" t="inlineStr"/>
-      <c r="I982" t="inlineStr">
-        <is>
-          <t>5561999355005</t>
-        </is>
+      <c r="I982" t="n">
+        <v>5561999355005</v>
       </c>
       <c r="J982" t="inlineStr"/>
       <c r="K982" t="n">
@@ -48333,10 +48331,8 @@
         </is>
       </c>
       <c r="H983" t="inlineStr"/>
-      <c r="I983" t="inlineStr">
-        <is>
-          <t>556196138793</t>
-        </is>
+      <c r="I983" t="n">
+        <v>556196138793</v>
       </c>
       <c r="J983" t="inlineStr"/>
       <c r="K983" t="n">
@@ -48433,10 +48429,8 @@
         </is>
       </c>
       <c r="H985" t="inlineStr"/>
-      <c r="I985" t="inlineStr">
-        <is>
-          <t>5561992112177</t>
-        </is>
+      <c r="I985" t="n">
+        <v>5561992112177</v>
       </c>
       <c r="J985" t="inlineStr"/>
       <c r="K985" t="n">
@@ -48485,10 +48479,8 @@
         </is>
       </c>
       <c r="H986" t="inlineStr"/>
-      <c r="I986" t="inlineStr">
-        <is>
-          <t>5515981224202</t>
-        </is>
+      <c r="I986" t="n">
+        <v>5515981224202</v>
       </c>
       <c r="J986" t="inlineStr"/>
       <c r="K986" t="n">
@@ -48777,10 +48769,8 @@
         </is>
       </c>
       <c r="H992" t="inlineStr"/>
-      <c r="I992" t="inlineStr">
-        <is>
-          <t>5561999963898</t>
-        </is>
+      <c r="I992" t="n">
+        <v>5561999963898</v>
       </c>
       <c r="J992" t="inlineStr"/>
       <c r="K992" t="n">
@@ -48829,10 +48819,8 @@
         </is>
       </c>
       <c r="H993" t="inlineStr"/>
-      <c r="I993" t="inlineStr">
-        <is>
-          <t>5562998228647</t>
-        </is>
+      <c r="I993" t="n">
+        <v>5562998228647</v>
       </c>
       <c r="J993" t="inlineStr"/>
       <c r="K993" t="n">
@@ -49025,10 +49013,8 @@
         </is>
       </c>
       <c r="H997" t="inlineStr"/>
-      <c r="I997" t="inlineStr">
-        <is>
-          <t>5562996768223</t>
-        </is>
+      <c r="I997" t="n">
+        <v>5562996768223</v>
       </c>
       <c r="J997" t="inlineStr"/>
       <c r="K997" t="n">
@@ -49088,6 +49074,1010 @@
         </is>
       </c>
     </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E999" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F999" t="inlineStr">
+        <is>
+          <t>Victoria Medicina: Victória Medicina e Diagnóstico</t>
+        </is>
+      </c>
+      <c r="G999" t="inlineStr">
+        <is>
+          <t>https://victoriamedicina.com.br</t>
+        </is>
+      </c>
+      <c r="H999" t="inlineStr"/>
+      <c r="I999" t="inlineStr">
+        <is>
+          <t>552730270100</t>
+        </is>
+      </c>
+      <c r="J999" t="inlineStr"/>
+      <c r="K999" t="n">
+        <v>82</v>
+      </c>
+      <c r="L999" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1000" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F1000" t="inlineStr">
+        <is>
+          <t>MedLive Centro Médico em Vitória-ES</t>
+        </is>
+      </c>
+      <c r="G1000" t="inlineStr">
+        <is>
+          <t>https://medlive-es.com.br</t>
+        </is>
+      </c>
+      <c r="H1000" t="inlineStr"/>
+      <c r="I1000" t="inlineStr">
+        <is>
+          <t>5527998004211</t>
+        </is>
+      </c>
+      <c r="J1000" t="inlineStr"/>
+      <c r="K1000" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1000" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1001" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1001" t="inlineStr">
+        <is>
+          <t>Padilha Odontologia</t>
+        </is>
+      </c>
+      <c r="G1001" t="inlineStr">
+        <is>
+          <t>https://institutopadilha.com.br</t>
+        </is>
+      </c>
+      <c r="H1001" t="inlineStr"/>
+      <c r="I1001" t="inlineStr"/>
+      <c r="J1001" t="inlineStr"/>
+      <c r="K1001" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1001" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1002" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1002" t="inlineStr">
+        <is>
+          <t>Maxxi Dental</t>
+        </is>
+      </c>
+      <c r="G1002" t="inlineStr">
+        <is>
+          <t>https://maxxidental.com.br</t>
+        </is>
+      </c>
+      <c r="H1002" t="inlineStr"/>
+      <c r="I1002" t="inlineStr">
+        <is>
+          <t>552733253038</t>
+        </is>
+      </c>
+      <c r="J1002" t="inlineStr"/>
+      <c r="K1002" t="n">
+        <v>75</v>
+      </c>
+      <c r="L1002" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1003" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1003" t="inlineStr">
+        <is>
+          <t>Clínica Kamilla Scalzer: Dentista em Vitória ES</t>
+        </is>
+      </c>
+      <c r="G1003" t="inlineStr">
+        <is>
+          <t>https://clinicakamillascalzer.com.br</t>
+        </is>
+      </c>
+      <c r="H1003" t="inlineStr"/>
+      <c r="I1003" t="inlineStr"/>
+      <c r="J1003" t="inlineStr"/>
+      <c r="K1003" t="n">
+        <v>81</v>
+      </c>
+      <c r="L1003" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1004" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F1004" t="inlineStr">
+        <is>
+          <t>Um Estudo na Academia Popular de Santo Antônio em Vitória-ES</t>
+        </is>
+      </c>
+      <c r="G1004" t="inlineStr">
+        <is>
+          <t>https://periodicos.ufmg.br</t>
+        </is>
+      </c>
+      <c r="H1004" t="inlineStr"/>
+      <c r="I1004" t="inlineStr"/>
+      <c r="J1004" t="inlineStr"/>
+      <c r="K1004" t="n">
+        <v>56</v>
+      </c>
+      <c r="L1004" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="E1005" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F1005" t="inlineStr">
+        <is>
+          <t>Kit Para Montar Academia in Vitória, ES</t>
+        </is>
+      </c>
+      <c r="G1005" t="inlineStr">
+        <is>
+          <t>https://powerrun.com.br</t>
+        </is>
+      </c>
+      <c r="H1005" t="inlineStr"/>
+      <c r="I1005" t="inlineStr">
+        <is>
+          <t>5514982191126</t>
+        </is>
+      </c>
+      <c r="J1005" t="inlineStr"/>
+      <c r="K1005" t="n">
+        <v>81</v>
+      </c>
+      <c r="L1005" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1006" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1006" t="inlineStr">
+        <is>
+          <t>Policlínica Salud</t>
+        </is>
+      </c>
+      <c r="G1006" t="inlineStr">
+        <is>
+          <t>https://www.policlinicasalud.com.br</t>
+        </is>
+      </c>
+      <c r="H1006" t="inlineStr"/>
+      <c r="I1006" t="inlineStr"/>
+      <c r="J1006" t="inlineStr"/>
+      <c r="K1006" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1006" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1007" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F1007" t="inlineStr">
+        <is>
+          <t>Centro Médico MaterMed - 50 Anos cuidando de você!</t>
+        </is>
+      </c>
+      <c r="G1007" t="inlineStr">
+        <is>
+          <t>https://www.matermed.com.br</t>
+        </is>
+      </c>
+      <c r="H1007" t="inlineStr"/>
+      <c r="I1007" t="inlineStr">
+        <is>
+          <t>5531998784777</t>
+        </is>
+      </c>
+      <c r="J1007" t="inlineStr"/>
+      <c r="K1007" t="n">
+        <v>62</v>
+      </c>
+      <c r="L1007" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1008" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F1008" t="inlineStr">
+        <is>
+          <t>consulta com médico clínico geral valor r$100,00</t>
+        </is>
+      </c>
+      <c r="G1008" t="inlineStr">
+        <is>
+          <t>https://www.bhcentrodiagnostico.com</t>
+        </is>
+      </c>
+      <c r="H1008" t="inlineStr"/>
+      <c r="I1008" t="inlineStr">
+        <is>
+          <t>5531996022782</t>
+        </is>
+      </c>
+      <c r="J1008" t="inlineStr"/>
+      <c r="K1008" t="n">
+        <v>62</v>
+      </c>
+      <c r="L1008" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1009" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F1009" t="inlineStr">
+        <is>
+          <t>Hospital Evangélico de Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="G1009" t="inlineStr">
+        <is>
+          <t>https://he.org.br</t>
+        </is>
+      </c>
+      <c r="H1009" t="inlineStr"/>
+      <c r="I1009" t="inlineStr">
+        <is>
+          <t>553121388355</t>
+        </is>
+      </c>
+      <c r="J1009" t="inlineStr"/>
+      <c r="K1009" t="n">
+        <v>75</v>
+      </c>
+      <c r="L1009" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1010" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1010" t="inlineStr">
+        <is>
+          <t>Dentista</t>
+        </is>
+      </c>
+      <c r="G1010" t="inlineStr">
+        <is>
+          <t>https://www.odontosaudevida.com.br</t>
+        </is>
+      </c>
+      <c r="H1010" t="inlineStr"/>
+      <c r="I1010" t="inlineStr"/>
+      <c r="J1010" t="inlineStr"/>
+      <c r="K1010" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1010" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1011" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1011" t="inlineStr">
+        <is>
+          <t>Marcos Santos</t>
+        </is>
+      </c>
+      <c r="G1011" t="inlineStr">
+        <is>
+          <t>https://msantosodonto.com</t>
+        </is>
+      </c>
+      <c r="H1011" t="inlineStr"/>
+      <c r="I1011" t="inlineStr">
+        <is>
+          <t>5531993519143</t>
+        </is>
+      </c>
+      <c r="J1011" t="inlineStr"/>
+      <c r="K1011" t="n">
+        <v>62</v>
+      </c>
+      <c r="L1011" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1012" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F1012" t="inlineStr">
+        <is>
+          <t>Contextualmente</t>
+        </is>
+      </c>
+      <c r="G1012" t="inlineStr">
+        <is>
+          <t>https://www.contextualmente.com</t>
+        </is>
+      </c>
+      <c r="H1012" t="inlineStr"/>
+      <c r="I1012" t="inlineStr"/>
+      <c r="J1012" t="inlineStr"/>
+      <c r="K1012" t="n">
+        <v>33</v>
+      </c>
+      <c r="L1012" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1013" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F1013" t="inlineStr">
+        <is>
+          <t>Terapia Clínica</t>
+        </is>
+      </c>
+      <c r="G1013" t="inlineStr">
+        <is>
+          <t>https://terapiaclinica.com.br</t>
+        </is>
+      </c>
+      <c r="H1013" t="inlineStr"/>
+      <c r="I1013" t="inlineStr"/>
+      <c r="J1013" t="inlineStr"/>
+      <c r="K1013" t="n">
+        <v>87</v>
+      </c>
+      <c r="L1013" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1014" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F1014" t="inlineStr">
+        <is>
+          <t>Dr. Sérgio Antonio</t>
+        </is>
+      </c>
+      <c r="G1014" t="inlineStr">
+        <is>
+          <t>https://www.sergioantonioadvocacia.com.br</t>
+        </is>
+      </c>
+      <c r="H1014" t="inlineStr"/>
+      <c r="I1014" t="inlineStr"/>
+      <c r="J1014" t="inlineStr"/>
+      <c r="K1014" t="n">
+        <v>55</v>
+      </c>
+      <c r="L1014" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1015" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F1015" t="inlineStr">
+        <is>
+          <t>Advogado Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="G1015" t="inlineStr">
+        <is>
+          <t>https://cleidesobreira.com.br</t>
+        </is>
+      </c>
+      <c r="H1015" t="inlineStr"/>
+      <c r="I1015" t="inlineStr">
+        <is>
+          <t>5511988078120</t>
+        </is>
+      </c>
+      <c r="J1015" t="inlineStr"/>
+      <c r="K1015" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1015" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E1016" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F1016" t="inlineStr">
+        <is>
+          <t>Fisioterapeuta em Belo Horizonte - MG</t>
+        </is>
+      </c>
+      <c r="G1016" t="inlineStr">
+        <is>
+          <t>https://www.paularezendefisio.com.br</t>
+        </is>
+      </c>
+      <c r="H1016" t="inlineStr"/>
+      <c r="I1016" t="inlineStr">
+        <is>
+          <t>5531999731985</t>
+        </is>
+      </c>
+      <c r="J1016" t="inlineStr"/>
+      <c r="K1016" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1016" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1017" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1017" t="inlineStr">
+        <is>
+          <t>Consulta Carioca</t>
+        </is>
+      </c>
+      <c r="G1017" t="inlineStr">
+        <is>
+          <t>https://www.consultacarioca.com.br</t>
+        </is>
+      </c>
+      <c r="H1017" t="inlineStr"/>
+      <c r="I1017" t="inlineStr">
+        <is>
+          <t>5521969162030</t>
+        </is>
+      </c>
+      <c r="J1017" t="inlineStr"/>
+      <c r="K1017" t="n">
+        <v>76</v>
+      </c>
+      <c r="L1017" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>Sudeste</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E1018" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1018" t="inlineStr">
+        <is>
+          <t>Clínicas Prosaúde</t>
+        </is>
+      </c>
+      <c r="G1018" t="inlineStr">
+        <is>
+          <t>https://prosaude.com.br</t>
+        </is>
+      </c>
+      <c r="H1018" t="inlineStr"/>
+      <c r="I1018" t="inlineStr"/>
+      <c r="J1018" t="inlineStr"/>
+      <c r="K1018" t="n">
+        <v>56</v>
+      </c>
+      <c r="L1018" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Nordeste, +12 novos)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1060"/>
+  <dimension ref="A1:L1072"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51265,10 +51265,8 @@
         </is>
       </c>
       <c r="H1043" t="inlineStr"/>
-      <c r="I1043" t="inlineStr">
-        <is>
-          <t>556899355105</t>
-        </is>
+      <c r="I1043" t="n">
+        <v>556899355105</v>
       </c>
       <c r="J1043" t="inlineStr"/>
       <c r="K1043" t="n">
@@ -51317,10 +51315,8 @@
         </is>
       </c>
       <c r="H1044" t="inlineStr"/>
-      <c r="I1044" t="inlineStr">
-        <is>
-          <t>5508002242808</t>
-        </is>
+      <c r="I1044" t="n">
+        <v>5508002242808</v>
       </c>
       <c r="J1044" t="inlineStr"/>
       <c r="K1044" t="n">
@@ -51417,10 +51413,8 @@
         </is>
       </c>
       <c r="H1046" t="inlineStr"/>
-      <c r="I1046" t="inlineStr">
-        <is>
-          <t>5568999670789</t>
-        </is>
+      <c r="I1046" t="n">
+        <v>5568999670789</v>
       </c>
       <c r="J1046" t="inlineStr"/>
       <c r="K1046" t="n">
@@ -52093,16 +52087,618 @@
         </is>
       </c>
       <c r="H1060" t="inlineStr"/>
-      <c r="I1060" t="inlineStr">
-        <is>
-          <t>5592992863958</t>
-        </is>
+      <c r="I1060" t="n">
+        <v>5592992863958</v>
       </c>
       <c r="J1060" t="inlineStr"/>
       <c r="K1060" t="n">
         <v>73</v>
       </c>
       <c r="L1060" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D1061" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E1061" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F1061" t="inlineStr">
+        <is>
+          <t>Comac Material Médico</t>
+        </is>
+      </c>
+      <c r="G1061" t="inlineStr">
+        <is>
+          <t>https://www.comacmaterialmedico.com.br</t>
+        </is>
+      </c>
+      <c r="H1061" t="inlineStr"/>
+      <c r="I1061" t="inlineStr">
+        <is>
+          <t>558299981468</t>
+        </is>
+      </c>
+      <c r="J1061" t="inlineStr"/>
+      <c r="K1061" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1061" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D1062" t="inlineStr">
+        <is>
+          <t>Maceió</t>
+        </is>
+      </c>
+      <c r="E1062" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F1062" t="inlineStr">
+        <is>
+          <t>PERFIL DA MORTALIDADE POR ASFIXIAS NO INSTITUTO ...</t>
+        </is>
+      </c>
+      <c r="G1062" t="inlineStr">
+        <is>
+          <t>https://www.perspectivas.med.br</t>
+        </is>
+      </c>
+      <c r="H1062" t="inlineStr"/>
+      <c r="I1062" t="inlineStr"/>
+      <c r="J1062" t="inlineStr"/>
+      <c r="K1062" t="n">
+        <v>65</v>
+      </c>
+      <c r="L1062" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D1063" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E1063" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1063" t="inlineStr">
+        <is>
+          <t>Clínica ADS</t>
+        </is>
+      </c>
+      <c r="G1063" t="inlineStr">
+        <is>
+          <t>https://clinicaads.com.br</t>
+        </is>
+      </c>
+      <c r="H1063" t="inlineStr"/>
+      <c r="I1063" t="inlineStr">
+        <is>
+          <t>557199237237</t>
+        </is>
+      </c>
+      <c r="J1063" t="inlineStr"/>
+      <c r="K1063" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1063" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D1064" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E1064" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1064" t="inlineStr">
+        <is>
+          <t>Clínica da Família: HOME</t>
+        </is>
+      </c>
+      <c r="G1064" t="inlineStr">
+        <is>
+          <t>https://www.clinicamedicadafamilia.com.br</t>
+        </is>
+      </c>
+      <c r="H1064" t="inlineStr"/>
+      <c r="I1064" t="inlineStr">
+        <is>
+          <t>5571994180003</t>
+        </is>
+      </c>
+      <c r="J1064" t="inlineStr"/>
+      <c r="K1064" t="n">
+        <v>80</v>
+      </c>
+      <c r="L1064" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D1065" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E1065" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1065" t="inlineStr">
+        <is>
+          <t>Clínica Odontológica Vilasboas</t>
+        </is>
+      </c>
+      <c r="G1065" t="inlineStr">
+        <is>
+          <t>https://www.clinicavilasboas.com.br</t>
+        </is>
+      </c>
+      <c r="H1065" t="inlineStr"/>
+      <c r="I1065" t="inlineStr"/>
+      <c r="J1065" t="inlineStr"/>
+      <c r="K1065" t="n">
+        <v>80</v>
+      </c>
+      <c r="L1065" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D1066" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E1066" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1066" t="inlineStr">
+        <is>
+          <t>Dental Mac Salvador</t>
+        </is>
+      </c>
+      <c r="G1066" t="inlineStr">
+        <is>
+          <t>https://dentalmacssa.com.br</t>
+        </is>
+      </c>
+      <c r="H1066" t="inlineStr"/>
+      <c r="I1066" t="inlineStr">
+        <is>
+          <t>557133599096</t>
+        </is>
+      </c>
+      <c r="J1066" t="inlineStr"/>
+      <c r="K1066" t="n">
+        <v>81</v>
+      </c>
+      <c r="L1066" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D1067" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E1067" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1067" t="inlineStr">
+        <is>
+          <t>Oral Clean Odontologia Digital</t>
+        </is>
+      </c>
+      <c r="G1067" t="inlineStr">
+        <is>
+          <t>https://www.adoromeusorriso.com.br</t>
+        </is>
+      </c>
+      <c r="H1067" t="inlineStr"/>
+      <c r="I1067" t="inlineStr">
+        <is>
+          <t>5571999668851</t>
+        </is>
+      </c>
+      <c r="J1067" t="inlineStr"/>
+      <c r="K1067" t="n">
+        <v>62</v>
+      </c>
+      <c r="L1067" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D1068" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E1068" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1068" t="inlineStr">
+        <is>
+          <t>Climil Odontologia Moderna</t>
+        </is>
+      </c>
+      <c r="G1068" t="inlineStr">
+        <is>
+          <t>https://climilodontologiamoderna.com.br</t>
+        </is>
+      </c>
+      <c r="H1068" t="inlineStr"/>
+      <c r="I1068" t="inlineStr"/>
+      <c r="J1068" t="inlineStr"/>
+      <c r="K1068" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1068" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E1069" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1069" t="inlineStr">
+        <is>
+          <t>Encontre um especialista</t>
+        </is>
+      </c>
+      <c r="G1069" t="inlineStr">
+        <is>
+          <t>https://croba.org.br</t>
+        </is>
+      </c>
+      <c r="H1069" t="inlineStr"/>
+      <c r="I1069" t="inlineStr">
+        <is>
+          <t>5507131142525</t>
+        </is>
+      </c>
+      <c r="J1069" t="inlineStr"/>
+      <c r="K1069" t="n">
+        <v>88</v>
+      </c>
+      <c r="L1069" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D1070" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E1070" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F1070" t="inlineStr">
+        <is>
+          <t>Louise Diná</t>
+        </is>
+      </c>
+      <c r="G1070" t="inlineStr">
+        <is>
+          <t>https://www.psicologalouise.com.br</t>
+        </is>
+      </c>
+      <c r="H1070" t="inlineStr"/>
+      <c r="I1070" t="inlineStr">
+        <is>
+          <t>5571983631000</t>
+        </is>
+      </c>
+      <c r="J1070" t="inlineStr"/>
+      <c r="K1070" t="n">
+        <v>93</v>
+      </c>
+      <c r="L1070" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D1071" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E1071" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F1071" t="inlineStr">
+        <is>
+          <t>Psicólogo em Salvador BA: como encontrar o profissional certo</t>
+        </is>
+      </c>
+      <c r="G1071" t="inlineStr">
+        <is>
+          <t>https://lumusterapia.com.br</t>
+        </is>
+      </c>
+      <c r="H1071" t="inlineStr"/>
+      <c r="I1071" t="inlineStr"/>
+      <c r="J1071" t="inlineStr"/>
+      <c r="K1071" t="n">
+        <v>80</v>
+      </c>
+      <c r="L1071" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D1072" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="E1072" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F1072" t="inlineStr">
+        <is>
+          <t>Terapeutas para Ansiedade</t>
+        </is>
+      </c>
+      <c r="G1072" t="inlineStr">
+        <is>
+          <t>https://vitrine.terapiaacolher.com.br</t>
+        </is>
+      </c>
+      <c r="H1072" t="inlineStr"/>
+      <c r="I1072" t="inlineStr"/>
+      <c r="J1072" t="inlineStr"/>
+      <c r="K1072" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1072" t="inlineStr">
         <is>
           <t>Crítico</t>
         </is>

</xml_diff>

<commit_message>
Atualiza planilha diária de leads e conformidade (Centro-Oeste, +22 novos)
Co-authored-by: Leandro Oliveira <leandroeriksonoliveira@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads_automation/data/leads_conformidade_brasil.xlsx
+++ b/leads_automation/data/leads_conformidade_brasil.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1145"/>
+  <dimension ref="A1:L1167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55855,10 +55855,8 @@
         </is>
       </c>
       <c r="H1137" t="inlineStr"/>
-      <c r="I1137" t="inlineStr">
-        <is>
-          <t>5582993230900</t>
-        </is>
+      <c r="I1137" t="n">
+        <v>5582993230900</v>
       </c>
       <c r="J1137" t="inlineStr"/>
       <c r="K1137" t="n">
@@ -55907,10 +55905,8 @@
         </is>
       </c>
       <c r="H1138" t="inlineStr"/>
-      <c r="I1138" t="inlineStr">
-        <is>
-          <t>5582998260123</t>
-        </is>
+      <c r="I1138" t="n">
+        <v>5582998260123</v>
       </c>
       <c r="J1138" t="inlineStr"/>
       <c r="K1138" t="n">
@@ -55959,10 +55955,8 @@
         </is>
       </c>
       <c r="H1139" t="inlineStr"/>
-      <c r="I1139" t="inlineStr">
-        <is>
-          <t>5582991442003</t>
-        </is>
+      <c r="I1139" t="n">
+        <v>5582991442003</v>
       </c>
       <c r="J1139" t="inlineStr"/>
       <c r="K1139" t="n">
@@ -56203,10 +56197,8 @@
         </is>
       </c>
       <c r="H1144" t="inlineStr"/>
-      <c r="I1144" t="inlineStr">
-        <is>
-          <t>5571987803521</t>
-        </is>
+      <c r="I1144" t="n">
+        <v>5571987803521</v>
       </c>
       <c r="J1144" t="inlineStr"/>
       <c r="K1144" t="n">
@@ -56266,6 +56258,1102 @@
         </is>
       </c>
     </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1146" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1146" t="inlineStr">
+        <is>
+          <t>Sigmavita</t>
+        </is>
+      </c>
+      <c r="G1146" t="inlineStr">
+        <is>
+          <t>https://www.sigmavita.com.br</t>
+        </is>
+      </c>
+      <c r="H1146" t="inlineStr"/>
+      <c r="I1146" t="inlineStr"/>
+      <c r="J1146" t="inlineStr"/>
+      <c r="K1146" t="n">
+        <v>56</v>
+      </c>
+      <c r="L1146" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1147" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1147" t="inlineStr">
+        <is>
+          <t>Kypy Saúde - Clínica Médica em Brasília</t>
+        </is>
+      </c>
+      <c r="G1147" t="inlineStr">
+        <is>
+          <t>https://kypysaude.com.br</t>
+        </is>
+      </c>
+      <c r="H1147" t="inlineStr"/>
+      <c r="I1147" t="inlineStr">
+        <is>
+          <t>556193656589</t>
+        </is>
+      </c>
+      <c r="J1147" t="inlineStr"/>
+      <c r="K1147" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1147" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1148" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>Clínica Médica no Guará</t>
+        </is>
+      </c>
+      <c r="G1148" t="inlineStr">
+        <is>
+          <t>https://centroclinicoportoclaro.com.br</t>
+        </is>
+      </c>
+      <c r="H1148" t="inlineStr"/>
+      <c r="I1148" t="inlineStr">
+        <is>
+          <t>5561993041166</t>
+        </is>
+      </c>
+      <c r="J1148" t="inlineStr"/>
+      <c r="K1148" t="n">
+        <v>87</v>
+      </c>
+      <c r="L1148" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1149" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1149" t="inlineStr">
+        <is>
+          <t>Início - Clínica Odontológica em Brasília</t>
+        </is>
+      </c>
+      <c r="G1149" t="inlineStr">
+        <is>
+          <t>https://cobodontologiabrasilia.com.br</t>
+        </is>
+      </c>
+      <c r="H1149" t="inlineStr"/>
+      <c r="I1149" t="inlineStr"/>
+      <c r="J1149" t="inlineStr"/>
+      <c r="K1149" t="n">
+        <v>22</v>
+      </c>
+      <c r="L1149" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1150" t="inlineStr">
+        <is>
+          <t>dentista</t>
+        </is>
+      </c>
+      <c r="F1150" t="inlineStr">
+        <is>
+          <t>Clínica Oral Concept</t>
+        </is>
+      </c>
+      <c r="G1150" t="inlineStr">
+        <is>
+          <t>https://clinicaoralconcept.com.br</t>
+        </is>
+      </c>
+      <c r="H1150" t="inlineStr"/>
+      <c r="I1150" t="inlineStr"/>
+      <c r="J1150" t="inlineStr"/>
+      <c r="K1150" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1150" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1151" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1151" t="inlineStr">
+        <is>
+          <t>Lucas Bezerra: Psicólogo em Brasília e Online</t>
+        </is>
+      </c>
+      <c r="G1151" t="inlineStr">
+        <is>
+          <t>https://psicologobrasilia.com.br</t>
+        </is>
+      </c>
+      <c r="H1151" t="inlineStr"/>
+      <c r="I1151" t="inlineStr">
+        <is>
+          <t>5561984048581</t>
+        </is>
+      </c>
+      <c r="J1151" t="inlineStr"/>
+      <c r="K1151" t="n">
+        <v>64</v>
+      </c>
+      <c r="L1151" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1152" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1152" t="inlineStr">
+        <is>
+          <t>Fabíola Freitas</t>
+        </is>
+      </c>
+      <c r="G1152" t="inlineStr">
+        <is>
+          <t>https://www.conexasaude.com.br</t>
+        </is>
+      </c>
+      <c r="H1152" t="inlineStr"/>
+      <c r="I1152" t="inlineStr">
+        <is>
+          <t>5511976396153</t>
+        </is>
+      </c>
+      <c r="J1152" t="inlineStr"/>
+      <c r="K1152" t="n">
+        <v>80</v>
+      </c>
+      <c r="L1152" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1153" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1153" t="inlineStr">
+        <is>
+          <t>CRP DF: Conselho Regional de Psicologia do DF</t>
+        </is>
+      </c>
+      <c r="G1153" t="inlineStr">
+        <is>
+          <t>https://www.crp-01.org.br</t>
+        </is>
+      </c>
+      <c r="H1153" t="inlineStr"/>
+      <c r="I1153" t="inlineStr"/>
+      <c r="J1153" t="inlineStr"/>
+      <c r="K1153" t="n">
+        <v>75</v>
+      </c>
+      <c r="L1153" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1154" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1154" t="inlineStr">
+        <is>
+          <t>Terappia</t>
+        </is>
+      </c>
+      <c r="G1154" t="inlineStr">
+        <is>
+          <t>https://www.terappia.com.br</t>
+        </is>
+      </c>
+      <c r="H1154" t="inlineStr"/>
+      <c r="I1154" t="inlineStr">
+        <is>
+          <t>5521999850091</t>
+        </is>
+      </c>
+      <c r="J1154" t="inlineStr"/>
+      <c r="K1154" t="n">
+        <v>88</v>
+      </c>
+      <c r="L1154" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1155" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1155" t="inlineStr">
+        <is>
+          <t>CLÍNICA HOLLOS</t>
+        </is>
+      </c>
+      <c r="G1155" t="inlineStr">
+        <is>
+          <t>https://www.clinicahollos.com.br</t>
+        </is>
+      </c>
+      <c r="H1155" t="inlineStr"/>
+      <c r="I1155" t="inlineStr">
+        <is>
+          <t>5561992926161</t>
+        </is>
+      </c>
+      <c r="J1155" t="inlineStr"/>
+      <c r="K1155" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1155" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1156" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F1156" t="inlineStr">
+        <is>
+          <t>Psicóloga em Brasília: Terapia Cognitiva Online</t>
+        </is>
+      </c>
+      <c r="G1156" t="inlineStr">
+        <is>
+          <t>https://mariacarolinacolombo.com.br</t>
+        </is>
+      </c>
+      <c r="H1156" t="inlineStr"/>
+      <c r="I1156" t="inlineStr">
+        <is>
+          <t>556196811386</t>
+        </is>
+      </c>
+      <c r="J1156" t="inlineStr"/>
+      <c r="K1156" t="n">
+        <v>60</v>
+      </c>
+      <c r="L1156" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1157" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F1157" t="inlineStr">
+        <is>
+          <t>Elias Daher Psicanalista</t>
+        </is>
+      </c>
+      <c r="G1157" t="inlineStr">
+        <is>
+          <t>https://eliasdaherpsicanalista.com.br</t>
+        </is>
+      </c>
+      <c r="H1157" t="inlineStr"/>
+      <c r="I1157" t="inlineStr">
+        <is>
+          <t>5561992541042</t>
+        </is>
+      </c>
+      <c r="J1157" t="inlineStr"/>
+      <c r="K1157" t="n">
+        <v>81</v>
+      </c>
+      <c r="L1157" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1158" t="inlineStr">
+        <is>
+          <t>academia</t>
+        </is>
+      </c>
+      <c r="F1158" t="inlineStr">
+        <is>
+          <t>Melhores Academias em Brasilia</t>
+        </is>
+      </c>
+      <c r="G1158" t="inlineStr">
+        <is>
+          <t>https://academiasbr.com.br</t>
+        </is>
+      </c>
+      <c r="H1158" t="inlineStr"/>
+      <c r="I1158" t="inlineStr"/>
+      <c r="J1158" t="inlineStr"/>
+      <c r="K1158" t="n">
+        <v>80</v>
+      </c>
+      <c r="L1158" t="inlineStr">
+        <is>
+          <t>Baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="E1159" t="inlineStr">
+        <is>
+          <t>fisioterapeuta</t>
+        </is>
+      </c>
+      <c r="F1159" t="inlineStr">
+        <is>
+          <t>Fisioterapeuta no DF</t>
+        </is>
+      </c>
+      <c r="G1159" t="inlineStr">
+        <is>
+          <t>https://fisioterapeutaingrid.com</t>
+        </is>
+      </c>
+      <c r="H1159" t="inlineStr"/>
+      <c r="I1159" t="inlineStr"/>
+      <c r="J1159" t="inlineStr"/>
+      <c r="K1159" t="n">
+        <v>60</v>
+      </c>
+      <c r="L1159" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1160" t="inlineStr">
+        <is>
+          <t>clínica médica</t>
+        </is>
+      </c>
+      <c r="F1160" t="inlineStr">
+        <is>
+          <t>Clínica Médica de Alto Padrão em Goiânia</t>
+        </is>
+      </c>
+      <c r="G1160" t="inlineStr">
+        <is>
+          <t>https://clinicasaudeagora.com.br</t>
+        </is>
+      </c>
+      <c r="H1160" t="inlineStr"/>
+      <c r="I1160" t="inlineStr">
+        <is>
+          <t>5562981942470</t>
+        </is>
+      </c>
+      <c r="J1160" t="inlineStr"/>
+      <c r="K1160" t="n">
+        <v>80</v>
+      </c>
+      <c r="L1160" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1161" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F1161" t="inlineStr">
+        <is>
+          <t>Einstein Hospital Israelita em Goiânia</t>
+        </is>
+      </c>
+      <c r="G1161" t="inlineStr">
+        <is>
+          <t>https://www.einstein.br</t>
+        </is>
+      </c>
+      <c r="H1161" t="inlineStr"/>
+      <c r="I1161" t="inlineStr"/>
+      <c r="J1161" t="inlineStr"/>
+      <c r="K1161" t="n">
+        <v>33</v>
+      </c>
+      <c r="L1161" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1162" t="inlineStr">
+        <is>
+          <t>médico</t>
+        </is>
+      </c>
+      <c r="F1162" t="inlineStr">
+        <is>
+          <t>Santa Casa de Misericórdia de Goiânia</t>
+        </is>
+      </c>
+      <c r="G1162" t="inlineStr">
+        <is>
+          <t>https://www.santacasago.org.br</t>
+        </is>
+      </c>
+      <c r="H1162" t="inlineStr"/>
+      <c r="I1162" t="inlineStr"/>
+      <c r="J1162" t="inlineStr"/>
+      <c r="K1162" t="n">
+        <v>44</v>
+      </c>
+      <c r="L1162" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1163" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1163" t="inlineStr">
+        <is>
+          <t>psicólogo</t>
+        </is>
+      </c>
+      <c r="F1163" t="inlineStr">
+        <is>
+          <t>Thiago Valadares</t>
+        </is>
+      </c>
+      <c r="G1163" t="inlineStr">
+        <is>
+          <t>https://thiagovaladarespsi.com.br</t>
+        </is>
+      </c>
+      <c r="H1163" t="inlineStr"/>
+      <c r="I1163" t="inlineStr">
+        <is>
+          <t>5562982254507</t>
+        </is>
+      </c>
+      <c r="J1163" t="inlineStr"/>
+      <c r="K1163" t="n">
+        <v>73</v>
+      </c>
+      <c r="L1163" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1164" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1164" t="inlineStr">
+        <is>
+          <t>terapeuta</t>
+        </is>
+      </c>
+      <c r="F1164" t="inlineStr">
+        <is>
+          <t>A VIVÊNCIA DO AQUI-E-AGORA NA RELAÇÃO TERAPÊUTICA NA ...</t>
+        </is>
+      </c>
+      <c r="G1164" t="inlineStr">
+        <is>
+          <t>https://seer.pucgoias.edu.br</t>
+        </is>
+      </c>
+      <c r="H1164" t="inlineStr"/>
+      <c r="I1164" t="inlineStr"/>
+      <c r="J1164" t="inlineStr"/>
+      <c r="K1164" t="n">
+        <v>33</v>
+      </c>
+      <c r="L1164" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1165" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1165" t="inlineStr">
+        <is>
+          <t>advogado</t>
+        </is>
+      </c>
+      <c r="F1165" t="inlineStr">
+        <is>
+          <t>Advogado Goiânia</t>
+        </is>
+      </c>
+      <c r="G1165" t="inlineStr">
+        <is>
+          <t>https://goianiaadvogado.com.br</t>
+        </is>
+      </c>
+      <c r="H1165" t="inlineStr"/>
+      <c r="I1165" t="inlineStr"/>
+      <c r="J1165" t="inlineStr"/>
+      <c r="K1165" t="n">
+        <v>64</v>
+      </c>
+      <c r="L1165" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1166" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1166" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F1166" t="inlineStr">
+        <is>
+          <t>Educação Física</t>
+        </is>
+      </c>
+      <c r="G1166" t="inlineStr">
+        <is>
+          <t>https://www.institutodesaudeassistida.com.br</t>
+        </is>
+      </c>
+      <c r="H1166" t="inlineStr"/>
+      <c r="I1166" t="inlineStr"/>
+      <c r="J1166" t="inlineStr"/>
+      <c r="K1166" t="n">
+        <v>69</v>
+      </c>
+      <c r="L1166" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="D1167" t="inlineStr">
+        <is>
+          <t>Goiânia</t>
+        </is>
+      </c>
+      <c r="E1167" t="inlineStr">
+        <is>
+          <t>educação física</t>
+        </is>
+      </c>
+      <c r="F1167" t="inlineStr">
+        <is>
+          <t>Daniel Alves Personal</t>
+        </is>
+      </c>
+      <c r="G1167" t="inlineStr">
+        <is>
+          <t>https://www.clikofertas.com</t>
+        </is>
+      </c>
+      <c r="H1167" t="inlineStr"/>
+      <c r="I1167" t="inlineStr"/>
+      <c r="J1167" t="inlineStr"/>
+      <c r="K1167" t="n">
+        <v>0</v>
+      </c>
+      <c r="L1167" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>